<commit_message>
Refactor cliff mechanics and update project documentation for new segment types
- Revised the `Cliff` implementation to consolidate vertical wall types into a single `vertical_wall`, enhancing asset management and reducing redundancy.
- Updated the `Cliff` script to support runtime adjacency handling, ensuring visual consistency with neighboring segments.
- Adjusted `DECISIONS.md` to reflect the new cliff segment structure and its properties, clarifying design decisions.
- Modified `PROJECT_MAP.md` to accurately describe the updated cliff assets and their configurations.
- Integrated new cliff instances into the desert level, enriching gameplay with diverse destructible elements.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A52602A4-37A3-46AD-8E61-8ECB213E4663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B19413-A677-48A6-9367-3AF4A75E7350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
     <sheet name="glyphs" sheetId="2" r:id="rId2"/>
-    <sheet name="attunements" sheetId="3" r:id="rId3"/>
-    <sheet name="motion" sheetId="4" r:id="rId4"/>
-    <sheet name="objects_OLD" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet name="input" sheetId="6" r:id="rId6"/>
-    <sheet name="schema" sheetId="7" r:id="rId7"/>
+    <sheet name="attribute" sheetId="8" r:id="rId3"/>
+    <sheet name="attunements" sheetId="3" r:id="rId4"/>
+    <sheet name="motion" sheetId="4" r:id="rId5"/>
+    <sheet name="objects_OLD" sheetId="5" state="hidden" r:id="rId6"/>
+    <sheet name="input" sheetId="6" r:id="rId7"/>
+    <sheet name="schema" sheetId="7" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">objects_OLD!$A$1:$U$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">objects_OLD!$A$1:$U$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">orbs!$A$1:$W$44</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="301">
   <si>
     <t>id</t>
   </si>
@@ -910,6 +911,42 @@
   </si>
   <si>
     <t>experience</t>
+  </si>
+  <si>
+    <t>How fast the orb travels</t>
+  </si>
+  <si>
+    <t>Portion of hit damage also dealt to nearby enemies</t>
+  </si>
+  <si>
+    <t>Chance for a hit to critically strike</t>
+  </si>
+  <si>
+    <t>Extra damage multiplier on critical hits</t>
+  </si>
+  <si>
+    <t>Chance enemies and objects drop a glyph</t>
+  </si>
+  <si>
+    <t>Knockback strength. Enemies slammed into each other take this as damage; breakables take more damage</t>
+  </si>
+  <si>
+    <t>Stacks on hit. On death, the enemy explodes for more damage in a wider area the more stacks it had</t>
+  </si>
+  <si>
+    <t>Stacks on hit. Each stack slows move and attack speed by 5% (up to 90%)</t>
+  </si>
+  <si>
+    <t>Stacks on hit. At 10 stacks: deals 50 damage, stuns for 2 seconds, then clears</t>
+  </si>
+  <si>
+    <t>Stacks on hit. Deals 1 damage per stack every second until the enemy dies</t>
+  </si>
+  <si>
+    <t>Damage dealt to enemies on hit</t>
+  </si>
+  <si>
+    <t>Damage dealt to you on contact</t>
   </si>
 </sst>
 </file>
@@ -955,7 +992,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -998,6 +1035,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1021,7 +1064,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1040,6 +1083,8 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1528,14 +1573,14 @@
         <v>22</v>
       </c>
       <c r="B2" t="str">
-        <f>PROPER(A2)</f>
+        <f t="shared" ref="B2:B12" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Blank</v>
       </c>
       <c r="C2" t="s">
         <v>23</v>
       </c>
       <c r="H2" t="str">
-        <f t="shared" ref="H2:H33" si="0">IF(ISBLANK(F2),"",IF(COUNTIF($G$2:$G$101,G2)=1,"Yes","No"))</f>
+        <f t="shared" ref="H2:H33" si="1">IF(ISBLANK(F2),"",IF(COUNTIF($G$2:$G$101,G2)=1,"Yes","No"))</f>
         <v/>
       </c>
       <c r="I2" t="s">
@@ -1590,7 +1635,7 @@
         <v>25</v>
       </c>
       <c r="B3" t="str">
-        <f t="shared" ref="B3:B12" si="1">PROPER(A3)</f>
+        <f t="shared" si="0"/>
         <v>Conduit</v>
       </c>
       <c r="C3" t="s">
@@ -1610,7 +1655,7 @@
         <v>Air|Air|Fire</v>
       </c>
       <c r="H3" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="I3" t="s">
@@ -1665,7 +1710,7 @@
         <v>29</v>
       </c>
       <c r="B4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Contagion</v>
       </c>
       <c r="C4" t="s">
@@ -1685,7 +1730,7 @@
         <v>Earth|Earth|Air</v>
       </c>
       <c r="H4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="I4" t="s">
@@ -1740,7 +1785,7 @@
         <v>32</v>
       </c>
       <c r="B5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Ghost</v>
       </c>
       <c r="C5" t="s">
@@ -1760,7 +1805,7 @@
         <v>Air|Air|Earth</v>
       </c>
       <c r="H5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="I5" t="s">
@@ -1815,7 +1860,7 @@
         <v>34</v>
       </c>
       <c r="B6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Inferno</v>
       </c>
       <c r="C6" t="s">
@@ -1835,7 +1880,7 @@
         <v>Fire|Fire|Fire</v>
       </c>
       <c r="H6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="I6" t="s">
@@ -1890,7 +1935,7 @@
         <v>36</v>
       </c>
       <c r="B7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Shard</v>
       </c>
       <c r="C7" t="s">
@@ -1910,7 +1955,7 @@
         <v>Water|Water|Air</v>
       </c>
       <c r="H7" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="V7" t="str">
@@ -1926,7 +1971,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Runic</v>
       </c>
       <c r="C8" t="s">
@@ -1946,7 +1991,7 @@
         <v>Water|Water|Water</v>
       </c>
       <c r="H8" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="V8" t="str">
@@ -1962,7 +2007,7 @@
         <v>41</v>
       </c>
       <c r="B9" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Guardian</v>
       </c>
       <c r="C9" t="s">
@@ -1982,7 +2027,7 @@
         <v>Water|Water|Earth</v>
       </c>
       <c r="H9" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="V9" t="str">
@@ -1998,7 +2043,7 @@
         <v>43</v>
       </c>
       <c r="B10" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Mend</v>
       </c>
       <c r="C10" t="s">
@@ -2018,7 +2063,7 @@
         <v>Earth|Earth|Water</v>
       </c>
       <c r="H10" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="I10" t="s">
@@ -2037,7 +2082,7 @@
         <v>45</v>
       </c>
       <c r="B11" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Destroyer</v>
       </c>
       <c r="C11" t="s">
@@ -2057,7 +2102,7 @@
         <v>Fire|Air|Earth</v>
       </c>
       <c r="H11" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="I11" t="s">
@@ -2082,7 +2127,7 @@
         <v>272</v>
       </c>
       <c r="B12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>Vulcano</v>
       </c>
       <c r="C12" t="s">
@@ -2102,7 +2147,7 @@
         <v>Fire|Earth|Earth</v>
       </c>
       <c r="H12" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="I12" t="s">
@@ -2118,7 +2163,7 @@
         <v>274</v>
       </c>
       <c r="B13" t="str">
-        <f t="shared" ref="B12:B44" si="4">PROPER(SUBSTITUTE(A13,"_"," "))</f>
+        <f t="shared" ref="B13:B44" si="4">PROPER(SUBSTITUTE(A13,"_"," "))</f>
         <v>Lure</v>
       </c>
       <c r="C13" t="s">
@@ -2138,7 +2183,7 @@
         <v>Water|Air|Earth</v>
       </c>
       <c r="H13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="V13" t="str">
@@ -2168,7 +2213,7 @@
         <v>Water|Water|Fire</v>
       </c>
       <c r="H14" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
     </row>
@@ -2197,7 +2242,7 @@
         <v>Earth|Fire|Fire</v>
       </c>
       <c r="H15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
     </row>
@@ -2226,7 +2271,7 @@
         <v>Air|Air|Water</v>
       </c>
       <c r="H16" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="I16" t="s">
@@ -2258,7 +2303,7 @@
         <v>Fire|Earth|Air</v>
       </c>
       <c r="H17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
     </row>
@@ -2272,7 +2317,7 @@
         <v/>
       </c>
       <c r="H18" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2286,7 +2331,7 @@
         <v/>
       </c>
       <c r="H19" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2300,7 +2345,7 @@
         <v/>
       </c>
       <c r="H20" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2314,7 +2359,7 @@
         <v/>
       </c>
       <c r="H21" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2328,7 +2373,7 @@
         <v/>
       </c>
       <c r="H22" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2342,7 +2387,7 @@
         <v/>
       </c>
       <c r="H23" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2356,7 +2401,7 @@
         <v/>
       </c>
       <c r="H24" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2370,7 +2415,7 @@
         <v/>
       </c>
       <c r="H25" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2384,7 +2429,7 @@
         <v/>
       </c>
       <c r="H26" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2398,7 +2443,7 @@
         <v/>
       </c>
       <c r="H27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2412,7 +2457,7 @@
         <v/>
       </c>
       <c r="H28" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2426,7 +2471,7 @@
         <v/>
       </c>
       <c r="H29" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2440,7 +2485,7 @@
         <v/>
       </c>
       <c r="H30" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2454,7 +2499,7 @@
         <v/>
       </c>
       <c r="H31" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2468,7 +2513,7 @@
         <v/>
       </c>
       <c r="H32" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -2482,7 +2527,7 @@
         <v/>
       </c>
       <c r="H33" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3641,6 +3686,179 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C578474-C635-4D82-BABA-35BE76111A87}">
+  <sheetPr>
+    <tabColor theme="6" tint="0.59999389629810485"/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="110.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="str">
+        <f t="shared" ref="B2:B29" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
+        <v>Damage</v>
+      </c>
+      <c r="C2" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" si="0"/>
+        <v>Splash</v>
+      </c>
+      <c r="C3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>Burn</v>
+      </c>
+      <c r="C4" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Self Damage</v>
+      </c>
+      <c r="C5" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>Glyph Drop</v>
+      </c>
+      <c r="C6" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>Chill</v>
+      </c>
+      <c r="C7" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>Crit Chance</v>
+      </c>
+      <c r="C8" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>Speed</v>
+      </c>
+      <c r="C9" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>Shock</v>
+      </c>
+      <c r="C10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>Weight</v>
+      </c>
+      <c r="C11" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>Crit Damage</v>
+      </c>
+      <c r="C12" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>Poison</v>
+      </c>
+      <c r="C13" t="s">
+        <v>298</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="5" tint="0.59999389629810485"/>
@@ -4776,7 +4994,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor theme="4" tint="0.59999389629810485"/>
@@ -5009,7 +5227,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor theme="8" tint="0.59999389629810485"/>
@@ -6693,7 +6911,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
@@ -6729,12 +6947,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="14.7109375" customWidth="1"/>
@@ -7082,35 +7300,35 @@
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="15" t="s">
-        <v>271</v>
-      </c>
-      <c r="B32" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="C32" s="15" t="s">
+      <c r="A32" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C32" s="17" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="15" t="s">
-        <v>271</v>
-      </c>
-      <c r="B33" s="15" t="s">
+      <c r="A33" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B33" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="C33" s="17" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="15" t="s">
-        <v>271</v>
-      </c>
-      <c r="B34" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="C34" s="15" t="s">
+      <c r="A34" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C34" s="17" t="s">
         <v>266</v>
       </c>
     </row>
@@ -7119,7 +7337,7 @@
         <v>271</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="C35" s="15" t="s">
         <v>266</v>
@@ -7130,7 +7348,7 @@
         <v>271</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C36" s="15" t="s">
         <v>266</v>
@@ -7141,64 +7359,97 @@
         <v>271</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>4</v>
+        <v>78</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
         <v>271</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="C38" s="15" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
         <v>271</v>
       </c>
       <c r="B39" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="15" t="s">
+        <v>271</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="15" t="s">
+        <v>271</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="15" t="s">
+        <v>271</v>
+      </c>
+      <c r="B42" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C39" s="15" t="s">
+      <c r="C42" s="15" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="14" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B40" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="C40" s="14" t="s">
+      <c r="B43" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C43" s="14" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B41" s="14" t="s">
+      <c r="B44" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C41" s="14" t="s">
+      <c r="C44" s="14" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B45" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C42" s="14" t="s">
+      <c r="C45" s="14" t="s">
         <v>266</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove legacy documentation files and update project configurations for gameplay clarity
- Deleted outdated design documents (`A Final Spell.docx` and `A Final Spell.txt`) to streamline project resources.
- Updated project name in `project.godot` from "A Final Spell" to "Too Many Orbs" to better reflect the game's focus.
- Enhanced player control scripts to improve glyph throwing mechanics, allowing for more intuitive gameplay interactions.
- Revised `game_data.json` to include additional attributes and refine existing ones, ensuring accurate gameplay representation.
- Adjusted `orb_recipes.gd` to omit inactive recipes, improving the clarity of available options during gameplay.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B19413-A677-48A6-9367-3AF4A75E7350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{557E8C13-5900-460C-8AE7-C6521D70516F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="310">
   <si>
     <t>id</t>
   </si>
@@ -136,39 +136,24 @@
     <t>contagion</t>
   </si>
   <si>
-    <t>20% chance of adding Disease status to enemies. On death half their poison spreads to other nearby enemies</t>
-  </si>
-  <si>
     <t>Earth</t>
   </si>
   <si>
     <t>ghost</t>
   </si>
   <si>
-    <t>Enters and haunts enemies and deal its impact damage per second to them. Once dead, exits in a random direction.</t>
-  </si>
-  <si>
     <t>inferno</t>
   </si>
   <si>
-    <t>Leaves a trail of fire after the orb for 2 seconds, inflicting 1 Burn on enemies</t>
-  </si>
-  <si>
     <t>shard</t>
   </si>
   <si>
-    <t>Shoots ice chards around every 3 seconds, doing 30 damage and inflicting 2 Frost</t>
-  </si>
-  <si>
     <t>Water</t>
   </si>
   <si>
     <t>runic</t>
   </si>
   <si>
-    <t>Picks up glyphs instead of damaging them. Gets 5% damage increase for each deposited.</t>
-  </si>
-  <si>
     <t>guardian</t>
   </si>
   <si>
@@ -184,9 +169,6 @@
     <t>destroyer</t>
   </si>
   <si>
-    <t>High damage. Inflicts Burn, Frost and Poison. Chases the nearest player</t>
-  </si>
-  <si>
     <t>spite</t>
   </si>
   <si>
@@ -367,18 +349,12 @@
     <t>All poison stacks spread on death</t>
   </si>
   <si>
-    <t>improve</t>
-  </si>
-  <si>
     <t>Any picked up glyph goes up in rarity</t>
   </si>
   <si>
     <t>hoarder</t>
   </si>
   <si>
-    <t>Gets 5% damage increase for each deposited glyph</t>
-  </si>
-  <si>
     <t>affinity</t>
   </si>
   <si>
@@ -865,9 +841,6 @@
     <t>vulcano</t>
   </si>
   <si>
-    <t>Spews magma around it. Magma inflicts Burn on passing enemies</t>
-  </si>
-  <si>
     <t>lure</t>
   </si>
   <si>
@@ -880,9 +853,6 @@
     <t>hunger</t>
   </si>
   <si>
-    <t>Destroys objects in 1 hit. Every destroyed object increases damage and self damage by 10%</t>
-  </si>
-  <si>
     <t>vengance</t>
   </si>
   <si>
@@ -947,6 +917,63 @@
   </si>
   <si>
     <t>Damage dealt to you on contact</t>
+  </si>
+  <si>
+    <t>Very high base stats. Chases the nearest player</t>
+  </si>
+  <si>
+    <t>enchant</t>
+  </si>
+  <si>
+    <t>secure</t>
+  </si>
+  <si>
+    <t>Droped glyphs gets a shield protecting against one damage instance</t>
+  </si>
+  <si>
+    <t>Gets 5% damage increase for each dropped glyph</t>
+  </si>
+  <si>
+    <t>Enters and haunts enemies and deal its damage per second to them. Once dead, exits in a random direction.</t>
+  </si>
+  <si>
+    <t>Seeks glyphs out and picks them up instead of damaging them. Seeks out the summoning circle and drops them near</t>
+  </si>
+  <si>
+    <t>gravity</t>
+  </si>
+  <si>
+    <t>Slow nearby enemies by 30%</t>
+  </si>
+  <si>
+    <t>Every destroyed object increases weight by 1</t>
+  </si>
+  <si>
+    <t>smolder</t>
+  </si>
+  <si>
+    <t>Leaves a trail of fire after the orb for 2 seconds, inflicting 1 Smolder on enemies</t>
+  </si>
+  <si>
+    <t>nova</t>
+  </si>
+  <si>
+    <t>Makes a frost nova around the orb every 3 seconds inflicting 5 Chill</t>
+  </si>
+  <si>
+    <t>charge</t>
+  </si>
+  <si>
+    <t>rot</t>
+  </si>
+  <si>
+    <t>20% chance of adding Disease status to enemies. On death half their Rot spreads to other nearby enemies</t>
+  </si>
+  <si>
+    <t>Shoots ice chards around every 3 seconds, doing 30 damage and inflicting 2 Chill</t>
+  </si>
+  <si>
+    <t>Spews magma around it. Magma inflicts Smolder on passing enemies</t>
   </si>
 </sst>
 </file>
@@ -1064,7 +1091,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1084,7 +1111,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1493,7 +1519,7 @@
     <col min="14" max="14" width="8.5703125" customWidth="1"/>
     <col min="16" max="16" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14.5703125" customWidth="1"/>
-    <col min="18" max="18" width="8.85546875" customWidth="1"/>
+    <col min="18" max="18" width="11" customWidth="1"/>
     <col min="19" max="19" width="8.42578125" customWidth="1"/>
     <col min="20" max="20" width="8.5703125" customWidth="1"/>
     <col min="21" max="21" width="8.7109375" customWidth="1"/>
@@ -1550,16 +1576,16 @@
         <v>15</v>
       </c>
       <c r="R1" s="9" t="s">
-        <v>16</v>
+        <v>301</v>
       </c>
       <c r="S1" s="9" t="s">
         <v>17</v>
       </c>
       <c r="T1" s="9" t="s">
-        <v>18</v>
+        <v>305</v>
       </c>
       <c r="U1" s="9" t="s">
-        <v>19</v>
+        <v>306</v>
       </c>
       <c r="V1" s="13" t="s">
         <v>20</v>
@@ -1608,7 +1634,7 @@
         <v>0</v>
       </c>
       <c r="Q2" s="8">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="R2">
         <v>0</v>
@@ -1683,7 +1709,7 @@
         <v>0</v>
       </c>
       <c r="Q3" s="8">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="R3">
         <v>0</v>
@@ -1714,13 +1740,13 @@
         <v>Contagion</v>
       </c>
       <c r="C4" t="s">
+        <v>307</v>
+      </c>
+      <c r="D4" t="s">
         <v>30</v>
       </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F4" t="s">
         <v>27</v>
@@ -1758,7 +1784,7 @@
         <v>0.01</v>
       </c>
       <c r="Q4" s="8">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -1782,14 +1808,14 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Ghost</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>296</v>
       </c>
       <c r="D5" t="s">
         <v>27</v>
@@ -1798,7 +1824,7 @@
         <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G5" t="str">
         <f t="shared" si="2"/>
@@ -1833,7 +1859,7 @@
         <v>0</v>
       </c>
       <c r="Q5" s="8">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="R5">
         <v>0</v>
@@ -1857,14 +1883,14 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Inferno</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>302</v>
       </c>
       <c r="D6" t="s">
         <v>28</v>
@@ -1908,18 +1934,18 @@
         <v>0.05</v>
       </c>
       <c r="Q6" s="8">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="R6">
         <v>3</v>
       </c>
-      <c r="S6" s="8">
-        <v>0</v>
-      </c>
-      <c r="T6" s="8">
-        <v>0</v>
-      </c>
-      <c r="U6" s="8">
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6">
         <v>0</v>
       </c>
       <c r="V6" t="str">
@@ -1932,31 +1958,67 @@
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Shard</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>308</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E7" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G7" t="str">
         <f t="shared" si="2"/>
-        <v>Water|Water|Air</v>
+        <v>Water|Water|Fire</v>
       </c>
       <c r="H7" t="str">
         <f t="shared" si="1"/>
         <v>Yes</v>
+      </c>
+      <c r="J7">
+        <v>10</v>
+      </c>
+      <c r="K7">
+        <v>15</v>
+      </c>
+      <c r="L7" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="M7" s="8">
+        <v>2</v>
+      </c>
+      <c r="N7">
+        <v>90</v>
+      </c>
+      <c r="O7">
+        <v>3</v>
+      </c>
+      <c r="P7" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="Q7" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="R7">
+        <v>3</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="U7">
+        <v>0</v>
       </c>
       <c r="V7" t="str">
         <f>"res://entities/orbs/blank/"&amp;A7&amp;"_orb.tscn"</f>
@@ -1968,23 +2030,23 @@
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Runic</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>297</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F8" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G8" t="str">
         <f t="shared" si="2"/>
@@ -1994,6 +2056,42 @@
         <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
+      <c r="J8">
+        <v>10</v>
+      </c>
+      <c r="K8">
+        <v>15</v>
+      </c>
+      <c r="L8" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="M8" s="8">
+        <v>2</v>
+      </c>
+      <c r="N8">
+        <v>90</v>
+      </c>
+      <c r="O8">
+        <v>3</v>
+      </c>
+      <c r="P8" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="Q8" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="R8">
+        <v>3</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
       <c r="V8" t="str">
         <f t="shared" si="3"/>
         <v>res://entities/orbs/blank/runic_orb.tscn</v>
@@ -2004,23 +2102,23 @@
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Guardian</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G9" t="str">
         <f t="shared" si="2"/>
@@ -2040,23 +2138,23 @@
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>Mend</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F10" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G10" t="str">
         <f t="shared" si="2"/>
@@ -2067,7 +2165,7 @@
         <v>Yes</v>
       </c>
       <c r="I10" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="V10" t="str">
         <f t="shared" si="3"/>
@@ -2079,14 +2177,14 @@
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Destroyer</v>
       </c>
       <c r="C11" t="s">
-        <v>46</v>
+        <v>291</v>
       </c>
       <c r="D11" t="s">
         <v>28</v>
@@ -2095,7 +2193,7 @@
         <v>27</v>
       </c>
       <c r="F11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G11" t="str">
         <f t="shared" si="2"/>
@@ -2106,13 +2204,43 @@
         <v>Yes</v>
       </c>
       <c r="I11" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="J11">
         <v>50</v>
       </c>
       <c r="K11">
         <v>50</v>
+      </c>
+      <c r="L11" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="M11" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="N11">
+        <v>110</v>
+      </c>
+      <c r="O11">
+        <v>15</v>
+      </c>
+      <c r="P11" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="Q11" s="8">
+        <v>0.15</v>
+      </c>
+      <c r="R11">
+        <v>3</v>
+      </c>
+      <c r="S11">
+        <v>3</v>
+      </c>
+      <c r="T11">
+        <v>3</v>
+      </c>
+      <c r="U11">
+        <v>3</v>
       </c>
       <c r="V11" t="str">
         <f>"res://entities/orbs/blank/"&amp;A11&amp;"_orb.tscn"</f>
@@ -2124,23 +2252,23 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Vulcano</v>
       </c>
       <c r="C12" t="s">
-        <v>273</v>
+        <v>309</v>
       </c>
       <c r="D12" t="s">
         <v>28</v>
       </c>
       <c r="E12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G12" t="str">
         <f t="shared" si="2"/>
@@ -2151,7 +2279,7 @@
         <v>Yes</v>
       </c>
       <c r="I12" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="V12" t="str">
         <f>"res://entities/orbs/blank/"&amp;A12&amp;"_orb.tscn"</f>
@@ -2160,23 +2288,23 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" ref="B13:B44" si="4">PROPER(SUBSTITUTE(A13,"_"," "))</f>
         <v>Lure</v>
       </c>
       <c r="C13" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="D13" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E13" t="s">
         <v>27</v>
       </c>
       <c r="F13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G13" t="str">
         <f t="shared" si="2"/>
@@ -2197,20 +2325,20 @@
         <v/>
       </c>
       <c r="C14" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="D14" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E14" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="F14" t="s">
         <v>28</v>
       </c>
       <c r="G14" t="str">
         <f t="shared" si="2"/>
-        <v>Water|Water|Fire</v>
+        <v>Water|Air|Fire</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="1"/>
@@ -2219,17 +2347,17 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="4"/>
         <v>Hunger</v>
       </c>
       <c r="C15" t="s">
-        <v>278</v>
+        <v>300</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E15" t="s">
         <v>28</v>
@@ -2248,14 +2376,14 @@
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="4"/>
         <v>Vengance</v>
       </c>
       <c r="C16" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="D16" t="s">
         <v>27</v>
@@ -2264,7 +2392,7 @@
         <v>27</v>
       </c>
       <c r="F16" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G16" t="str">
         <f t="shared" si="2"/>
@@ -2275,25 +2403,25 @@
         <v>Yes</v>
       </c>
       <c r="I16" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="4"/>
         <v>Hunter</v>
       </c>
       <c r="C17" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="D17" t="s">
         <v>28</v>
       </c>
       <c r="E17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F17" t="s">
         <v>27</v>
@@ -2308,17 +2436,32 @@
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>303</v>
+      </c>
       <c r="B18" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Nova</v>
+      </c>
+      <c r="C18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D18" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" t="s">
+        <v>27</v>
       </c>
       <c r="G18" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Water|Water|Air</v>
       </c>
       <c r="H18" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Yes</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -3287,22 +3430,22 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>20</v>
@@ -3310,14 +3453,14 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B13" si="0">PROPER(A2)</f>
         <v>Coal</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D2" t="s">
         <v>28</v>
@@ -3341,14 +3484,14 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Fury</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
         <v>28</v>
@@ -3372,14 +3515,14 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Blast</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D4" t="s">
         <v>28</v>
@@ -3403,17 +3546,17 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Rime</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
         <v>17</v>
@@ -3434,17 +3577,17 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Sooth</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E6" t="s">
         <v>9</v>
@@ -3465,17 +3608,17 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Bounty</v>
       </c>
       <c r="C7" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E7" t="s">
         <v>15</v>
@@ -3496,14 +3639,14 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Static</v>
       </c>
       <c r="C8" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
         <v>27</v>
@@ -3527,14 +3670,14 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Shear</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D9" t="s">
         <v>27</v>
@@ -3558,14 +3701,14 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>Drag</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="D10" t="s">
         <v>27</v>
@@ -3589,17 +3732,17 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Blight</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E11" t="s">
         <v>19</v>
@@ -3620,17 +3763,17 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Dense</v>
       </c>
       <c r="C12" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E12" t="s">
         <v>13</v>
@@ -3651,17 +3794,17 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Crush</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E13" t="s">
         <v>11</v>
@@ -3706,7 +3849,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -3714,11 +3857,11 @@
         <v>8</v>
       </c>
       <c r="B2" t="str">
-        <f t="shared" ref="B2:B29" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
+        <f t="shared" ref="B2:B13" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Damage</v>
       </c>
       <c r="C2" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3730,7 +3873,7 @@
         <v>Splash</v>
       </c>
       <c r="C3" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3742,7 +3885,7 @@
         <v>Burn</v>
       </c>
       <c r="C4" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3754,7 +3897,7 @@
         <v>Self Damage</v>
       </c>
       <c r="C5" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3766,7 +3909,7 @@
         <v>Glyph Drop</v>
       </c>
       <c r="C6" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3778,7 +3921,7 @@
         <v>Chill</v>
       </c>
       <c r="C7" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3790,7 +3933,7 @@
         <v>Crit Chance</v>
       </c>
       <c r="C8" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3802,7 +3945,7 @@
         <v>Speed</v>
       </c>
       <c r="C9" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3814,7 +3957,7 @@
         <v>Shock</v>
       </c>
       <c r="C10" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3826,7 +3969,7 @@
         <v>Weight</v>
       </c>
       <c r="C11" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3838,7 +3981,7 @@
         <v>Crit Damage</v>
       </c>
       <c r="C12" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3850,7 +3993,7 @@
         <v>Poison</v>
       </c>
       <c r="C13" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -3863,13 +4006,13 @@
   <sheetPr>
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:I106"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="94.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="110.42578125" customWidth="1"/>
     <col min="5" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13" hidden="1" customWidth="1"/>
   </cols>
@@ -3882,10 +4025,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>3</v>
@@ -3902,17 +4045,17 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B2" t="str">
-        <f t="shared" ref="B2:B24" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
+        <f t="shared" ref="B2:B26" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Haunt</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E2" t="s">
         <v>27</v>
@@ -3921,10 +4064,10 @@
         <v>27</v>
       </c>
       <c r="G2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="H2" t="str">
-        <f t="shared" ref="H2:H33" si="1">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E2:G2))</f>
+        <f t="shared" ref="H2:H34" si="1">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E2:G2))</f>
         <v>Air|Air|Water</v>
       </c>
       <c r="I2" t="b">
@@ -3933,17 +4076,17 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Possesion</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E3" t="s">
         <v>28</v>
@@ -3964,17 +4107,17 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Trail</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E4" t="s">
         <v>28</v>
@@ -3983,7 +4126,7 @@
         <v>28</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H4" t="str">
         <f t="shared" si="1"/>
@@ -3995,17 +4138,17 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Kindling</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E5" t="s">
         <v>27</v>
@@ -4026,17 +4169,17 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Spark</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E6" t="s">
         <v>28</v>
@@ -4057,7 +4200,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
@@ -4067,10 +4210,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E7" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
         <v>27</v>
@@ -4082,10 +4225,13 @@
         <f t="shared" si="1"/>
         <v>Water|Air|Fire</v>
       </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
@@ -4095,25 +4241,28 @@
         <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E8" t="s">
         <v>27</v>
       </c>
       <c r="F8" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="H8" t="str">
         <f t="shared" si="1"/>
         <v>Air|Water|Water</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
@@ -4123,82 +4272,94 @@
         <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E9" t="s">
         <v>27</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H9" t="str">
         <f t="shared" si="1"/>
         <v>Air|Earth|Earth</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>Splinter</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="1"/>
         <v/>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Lethal</v>
       </c>
       <c r="C11" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="H11" t="str">
         <f t="shared" si="1"/>
         <v/>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Shatter</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D12" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="1"/>
         <v/>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
@@ -4208,16 +4369,19 @@
         <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="H13" t="str">
         <f t="shared" si="1"/>
         <v/>
+      </c>
+      <c r="I13" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
@@ -4227,16 +4391,19 @@
         <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="1"/>
         <v/>
+      </c>
+      <c r="I14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
@@ -4246,54 +4413,60 @@
         <v>29</v>
       </c>
       <c r="D15" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="H15" t="str">
         <f t="shared" si="1"/>
         <v/>
+      </c>
+      <c r="I15" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>107</v>
+        <v>292</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
-        <v>Improve</v>
+        <v>Enchant</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="E16" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F16" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G16" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="H16" t="str">
         <f t="shared" si="1"/>
-        <v>Water|Water|Earth</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+        <v>Water|Water|Air</v>
+      </c>
+      <c r="I16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>Hoarder</v>
       </c>
       <c r="C17" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>110</v>
+        <v>295</v>
       </c>
       <c r="E17" t="s">
         <v>28</v>
@@ -4308,210 +4481,268 @@
         <f t="shared" si="1"/>
         <v>Fire|Fire|Fire</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>111</v>
+        <v>293</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
+        <v>Secure</v>
+      </c>
+      <c r="C18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" t="s">
+        <v>294</v>
+      </c>
+      <c r="E18" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" t="s">
+        <v>30</v>
+      </c>
+      <c r="G18" t="s">
+        <v>30</v>
+      </c>
+      <c r="I18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
         <v>Affinity</v>
       </c>
-      <c r="C18" t="s">
-        <v>39</v>
-      </c>
-      <c r="D18" t="s">
-        <v>112</v>
-      </c>
-      <c r="E18" t="s">
-        <v>31</v>
-      </c>
-      <c r="F18" t="s">
-        <v>31</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="C19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" t="s">
+        <v>104</v>
+      </c>
+      <c r="E19" t="s">
+        <v>30</v>
+      </c>
+      <c r="F19" t="s">
+        <v>30</v>
+      </c>
+      <c r="G19" t="s">
         <v>28</v>
       </c>
-      <c r="H18" t="str">
+      <c r="H19" t="str">
         <f t="shared" si="1"/>
         <v>Earth|Earth|Fire</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>113</v>
-      </c>
-      <c r="B19" t="str">
+      <c r="I19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" t="str">
         <f t="shared" si="0"/>
         <v>Retribution</v>
       </c>
-      <c r="C19" t="s">
-        <v>41</v>
-      </c>
-      <c r="D19" t="s">
-        <v>114</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="C20" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" t="s">
+        <v>106</v>
+      </c>
+      <c r="E20" t="s">
         <v>28</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F20" t="s">
         <v>28</v>
       </c>
-      <c r="G19" t="s">
-        <v>31</v>
-      </c>
-      <c r="H19" t="str">
+      <c r="G20" t="s">
+        <v>30</v>
+      </c>
+      <c r="H20" t="str">
         <f t="shared" si="1"/>
         <v>Fire|Fire|Earth</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>115</v>
-      </c>
-      <c r="B20" t="str">
+      <c r="I20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>107</v>
+      </c>
+      <c r="B21" t="str">
         <f t="shared" si="0"/>
         <v>Flexible</v>
       </c>
-      <c r="C20" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" t="s">
-        <v>116</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="C21" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" t="s">
+        <v>108</v>
+      </c>
+      <c r="E21" t="s">
         <v>27</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F21" t="s">
         <v>27</v>
       </c>
-      <c r="G20" t="s">
-        <v>38</v>
-      </c>
-      <c r="H20" t="str">
+      <c r="G21" t="s">
+        <v>34</v>
+      </c>
+      <c r="H21" t="str">
         <f t="shared" si="1"/>
         <v>Air|Air|Water</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>117</v>
-      </c>
-      <c r="B21" t="str">
+      <c r="I21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v>Shield</v>
       </c>
-      <c r="C21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D21" t="s">
-        <v>118</v>
-      </c>
-      <c r="H21" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>288</v>
-      </c>
-      <c r="B22" t="str">
+      <c r="C22" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" t="s">
+        <v>110</v>
+      </c>
+      <c r="H22" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="I22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>278</v>
+      </c>
+      <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>Experience</v>
       </c>
-      <c r="C22" t="s">
-        <v>281</v>
-      </c>
-      <c r="D22" t="s">
-        <v>283</v>
-      </c>
-      <c r="H22" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>286</v>
-      </c>
-      <c r="B23" t="str">
+      <c r="C23" t="s">
+        <v>271</v>
+      </c>
+      <c r="D23" t="s">
+        <v>273</v>
+      </c>
+      <c r="H23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="I23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>276</v>
+      </c>
+      <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v>Stalk</v>
       </c>
-      <c r="C23" t="s">
-        <v>281</v>
-      </c>
-      <c r="D23" t="s">
-        <v>284</v>
-      </c>
-      <c r="H23" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>287</v>
-      </c>
-      <c r="B24" t="str">
+      <c r="C24" t="s">
+        <v>271</v>
+      </c>
+      <c r="D24" t="s">
+        <v>274</v>
+      </c>
+      <c r="H24" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="I24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>277</v>
+      </c>
+      <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>Fright</v>
       </c>
-      <c r="C24" t="s">
-        <v>281</v>
-      </c>
-      <c r="D24" t="s">
-        <v>285</v>
-      </c>
-      <c r="H24" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>271</v>
+      </c>
+      <c r="D25" t="s">
+        <v>275</v>
+      </c>
       <c r="H25" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>298</v>
+      </c>
+      <c r="B26" t="str">
+        <f t="shared" si="0"/>
+        <v>Gravity</v>
+      </c>
+      <c r="C26" t="s">
+        <v>268</v>
+      </c>
+      <c r="D26" t="s">
+        <v>299</v>
+      </c>
       <c r="H26" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H28" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H29" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H30" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H31" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H32" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4525,13 +4756,13 @@
     </row>
     <row r="34" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H34" t="str">
-        <f t="shared" ref="H34:H65" si="2">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E34:G34))</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="35" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H35" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="H35:H66" si="2">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E35:G35))</f>
         <v/>
       </c>
     </row>
@@ -4717,13 +4948,13 @@
     </row>
     <row r="66" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H66" t="str">
-        <f t="shared" ref="H66:H97" si="3">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E66:G66))</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="67" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H67" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="H67:H98" si="3">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E67:G67))</f>
         <v/>
       </c>
     </row>
@@ -4909,13 +5140,13 @@
     </row>
     <row r="98" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H98" t="str">
-        <f t="shared" ref="H98:H106" si="4">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E98:G98))</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="99" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H99" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="H99:H107" si="4">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E99:G99))</f>
         <v/>
       </c>
     </row>
@@ -4961,8 +5192,14 @@
         <v/>
       </c>
     </row>
+    <row r="107" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H107" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E1:G89">
+  <conditionalFormatting sqref="E1:G90">
     <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <formula>"Earth"</formula>
     </cfRule>
@@ -4977,20 +5214,32 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="41" operator="equal">
       <formula>"Earth"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="42" operator="equal">
       <formula>"Water"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="43" operator="equal">
       <formula>"Fire"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="44" operator="equal">
       <formula>"Air"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B625C9F3-AC3A-45E4-BF5F-4CA9BB4B1AFE}">
+          <x14:formula1>
+            <xm:f>input!$C$2:$F$2</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:G52</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -5015,7 +5264,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -5027,199 +5276,199 @@
         <v>Wayward</v>
       </c>
       <c r="C2" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Attracted</v>
       </c>
       <c r="C3" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Spite</v>
       </c>
       <c r="C4" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Rooted</v>
       </c>
       <c r="C5" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Patrol</v>
       </c>
       <c r="C6" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Familiar</v>
       </c>
       <c r="C7" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Rail</v>
       </c>
       <c r="C8" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Tide</v>
       </c>
       <c r="C9" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>Blink</v>
       </c>
       <c r="C10" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Loyal</v>
       </c>
       <c r="C11" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Hexed</v>
       </c>
       <c r="C12" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Stalker</v>
       </c>
       <c r="C13" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>Herd</v>
       </c>
       <c r="C14" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
         <v>Greedy</v>
       </c>
       <c r="C15" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
         <v>Oathbound</v>
       </c>
       <c r="C16" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>Echo</v>
       </c>
       <c r="C17" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>Phasing</v>
       </c>
       <c r="C18" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -5259,58 +5508,58 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="N1" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="P1" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="Q1" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="R1" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="T1" s="4" t="s">
         <v>158</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>166</v>
       </c>
       <c r="U1" s="3" t="s">
         <v>21</v>
@@ -5318,17 +5567,17 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B33" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Reception Desk</v>
       </c>
       <c r="C2" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D2" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="F2" s="2">
         <v>0</v>
@@ -5349,13 +5598,13 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="O2">
         <v>2</v>
       </c>
       <c r="T2" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="U2" t="b">
         <v>1</v>
@@ -5363,17 +5612,17 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Straw Pallet</v>
       </c>
       <c r="C3" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="D3" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="F3" s="2">
         <v>1</v>
@@ -5394,10 +5643,10 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M3" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O3">
         <v>2</v>
@@ -5411,17 +5660,17 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Wood Frame Bed</v>
       </c>
       <c r="C4" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="D4" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="F4" s="2">
         <v>0</v>
@@ -5442,10 +5691,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M4" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O4">
         <v>2</v>
@@ -5454,10 +5703,10 @@
         <v>0</v>
       </c>
       <c r="S4" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="T4" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="U4" t="b">
         <v>1</v>
@@ -5465,17 +5714,17 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Bunk Bed</v>
       </c>
       <c r="C5" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="D5" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="F5" s="2">
         <v>0</v>
@@ -5496,10 +5745,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M5" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O5">
         <v>2</v>
@@ -5508,10 +5757,10 @@
         <v>1</v>
       </c>
       <c r="S5" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="T5" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="U5" t="b">
         <v>1</v>
@@ -5519,17 +5768,17 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Canopy Bed</v>
       </c>
       <c r="C6" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="D6" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="F6" s="2">
         <v>0</v>
@@ -5550,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M6" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O6">
         <v>2</v>
@@ -5567,17 +5816,17 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Budget Wardrobe</v>
       </c>
       <c r="C7" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D7" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="F7" s="2">
         <v>0</v>
@@ -5598,10 +5847,10 @@
         <v>2</v>
       </c>
       <c r="L7" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M7" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O7">
         <v>3</v>
@@ -5610,10 +5859,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="T7" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="U7" t="b">
         <v>1</v>
@@ -5621,17 +5870,17 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Fine Wardrobe</v>
       </c>
       <c r="C8" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="D8" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="F8" s="2">
         <v>0</v>
@@ -5652,10 +5901,10 @@
         <v>4</v>
       </c>
       <c r="L8" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M8" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O8">
         <v>3</v>
@@ -5664,10 +5913,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="T8" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="U8" t="b">
         <v>1</v>
@@ -5675,17 +5924,17 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Ornate Wardrobe</v>
       </c>
       <c r="D9" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="E9" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="F9" s="2">
         <v>0</v>
@@ -5706,10 +5955,10 @@
         <v>7</v>
       </c>
       <c r="L9" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M9" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O9">
         <v>3</v>
@@ -5718,10 +5967,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="T9" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="U9" t="b">
         <v>1</v>
@@ -5729,7 +5978,7 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -5754,10 +6003,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M10" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O10">
         <v>1</v>
@@ -5771,14 +6020,14 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Wash Basin</v>
       </c>
       <c r="E11" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="F11" s="2">
         <v>0</v>
@@ -5799,10 +6048,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M11" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O11">
         <v>1</v>
@@ -5816,14 +6065,14 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Artisan Rug</v>
       </c>
       <c r="E12" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="F12" s="2">
         <v>0</v>
@@ -5844,7 +6093,7 @@
         <v>4</v>
       </c>
       <c r="L12" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="O12">
         <v>2</v>
@@ -5858,14 +6107,14 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Mirror</v>
       </c>
       <c r="E13" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="F13" s="2">
         <v>0</v>
@@ -5886,10 +6135,10 @@
         <v>3</v>
       </c>
       <c r="L13" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M13" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O13">
         <v>1</v>
@@ -5903,14 +6152,14 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>Trunk</v>
       </c>
       <c r="C14" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="F14" s="2">
         <v>0</v>
@@ -5931,10 +6180,10 @@
         <v>1</v>
       </c>
       <c r="L14" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M14" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O14">
         <v>2</v>
@@ -5948,7 +6197,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
@@ -5973,7 +6222,7 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="O15">
         <v>3</v>
@@ -5987,7 +6236,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
@@ -6012,10 +6261,10 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M16" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="O16">
         <v>1</v>
@@ -6029,14 +6278,14 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>Small Houseplant</v>
       </c>
       <c r="D17" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="F17" s="2">
         <v>0</v>
@@ -6057,7 +6306,7 @@
         <v>4</v>
       </c>
       <c r="L17" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="O17">
         <v>1</v>
@@ -6066,10 +6315,10 @@
         <v>0</v>
       </c>
       <c r="S17" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="T17" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="U17" t="b">
         <v>1</v>
@@ -6077,14 +6326,14 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>Big Houseplant</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="F18" s="2">
         <v>0</v>
@@ -6105,7 +6354,7 @@
         <v>6</v>
       </c>
       <c r="L18" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="O18">
         <v>2</v>
@@ -6119,14 +6368,14 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
         <v>Chamber Pot</v>
       </c>
       <c r="C19" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="F19" s="2">
         <v>0</v>
@@ -6147,10 +6396,10 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M19" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="O19">
         <v>1</v>
@@ -6164,17 +6413,17 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
         <v>Cooking Order Desk</v>
       </c>
       <c r="C20" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="D20" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="F20" s="2">
         <v>0</v>
@@ -6195,10 +6444,10 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M20" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="O20">
         <v>2</v>
@@ -6207,10 +6456,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="T20" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="U20" t="b">
         <v>1</v>
@@ -6218,17 +6467,17 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
         <v>Cooking Couldron</v>
       </c>
       <c r="C21" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="D21" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="F21" s="2">
         <v>0</v>
@@ -6249,10 +6498,10 @@
         <v>0</v>
       </c>
       <c r="L21" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M21" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="O21">
         <v>2</v>
@@ -6261,10 +6510,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="T21" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="U21" t="b">
         <v>1</v>
@@ -6272,14 +6521,14 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v>Small Seating Table</v>
       </c>
       <c r="D22" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="F22" s="2">
         <v>0</v>
@@ -6300,10 +6549,10 @@
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M22" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="O22">
         <v>2</v>
@@ -6312,10 +6561,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="T22" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="U22" t="b">
         <v>1</v>
@@ -6323,17 +6572,17 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>Pass Table</v>
       </c>
       <c r="C23" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="D23" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="F23" s="2">
         <v>0</v>
@@ -6354,10 +6603,10 @@
         <v>1</v>
       </c>
       <c r="L23" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M23" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="O23">
         <v>2</v>
@@ -6366,10 +6615,10 @@
         <v>0</v>
       </c>
       <c r="S23" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="T23" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="U23" t="b">
         <v>1</v>
@@ -6377,17 +6626,17 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v>Crate</v>
       </c>
       <c r="C24" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="D24" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="F24" s="2">
         <v>0</v>
@@ -6408,7 +6657,7 @@
         <v>0</v>
       </c>
       <c r="L24" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="O24">
         <v>2</v>
@@ -6417,10 +6666,10 @@
         <v>0</v>
       </c>
       <c r="S24" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="T24" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="U24" t="b">
         <v>1</v>
@@ -6428,17 +6677,17 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>Barrel</v>
       </c>
       <c r="C25" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="D25" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="F25" s="2">
         <v>0</v>
@@ -6459,7 +6708,7 @@
         <v>0</v>
       </c>
       <c r="L25" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="O25">
         <v>2</v>
@@ -6468,10 +6717,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="T25" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="U25" t="b">
         <v>1</v>
@@ -6479,17 +6728,17 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
         <v>Wall Torch</v>
       </c>
       <c r="C26" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="D26" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="F26" s="2">
         <v>0</v>
@@ -6510,7 +6759,7 @@
         <v>0</v>
       </c>
       <c r="L26" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="O26">
         <v>0</v>
@@ -6522,10 +6771,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="T26" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="U26" t="b">
         <v>1</v>
@@ -6533,17 +6782,17 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
         <v>Condiment Shelf</v>
       </c>
       <c r="C27" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="D27" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="F27" s="2">
         <v>0</v>
@@ -6564,10 +6813,10 @@
         <v>2</v>
       </c>
       <c r="L27" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="M27" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="O27">
         <v>1</v>
@@ -6579,10 +6828,10 @@
         <v>0</v>
       </c>
       <c r="S27" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="T27" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="U27" t="b">
         <v>1</v>
@@ -6590,17 +6839,17 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>Condiment Shelf Small</v>
       </c>
       <c r="C28" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="D28" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="F28" s="2">
         <v>0</v>
@@ -6621,10 +6870,10 @@
         <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="M28" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="O28">
         <v>1</v>
@@ -6636,10 +6885,10 @@
         <v>0</v>
       </c>
       <c r="S28" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="T28" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="U28" t="b">
         <v>1</v>
@@ -6647,17 +6896,17 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>Hanging Frying Pans</v>
       </c>
       <c r="C29" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="D29" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="F29" s="2">
         <v>0</v>
@@ -6678,10 +6927,10 @@
         <v>0</v>
       </c>
       <c r="L29" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="M29" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="O29">
         <v>0</v>
@@ -6692,14 +6941,14 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="0"/>
         <v>Butcher Table</v>
       </c>
       <c r="D30" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="F30" s="2">
         <v>0</v>
@@ -6720,10 +6969,10 @@
         <v>3</v>
       </c>
       <c r="L30" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M30" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="O30">
         <v>2</v>
@@ -6734,14 +6983,14 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>Hanging Meat</v>
       </c>
       <c r="D31" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -6924,22 +7173,22 @@
   <sheetData>
     <row r="2" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="C2" t="s">
         <v>28</v>
       </c>
       <c r="D2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E2" t="s">
         <v>27</v>
       </c>
       <c r="F2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -6960,464 +7209,464 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="B1" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="C1" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>16</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>19</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>20</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>0</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>20</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="C32" s="17" t="s">
-        <v>266</v>
+        <v>44</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="B33" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B33" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C33" s="17" t="s">
-        <v>266</v>
+      <c r="C33" s="16" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="B34" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="C34" s="17" t="s">
-        <v>266</v>
+        <v>44</v>
+      </c>
+      <c r="B34" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="B35" s="15" t="s">
         <v>0</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>1</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="B39" s="15" t="s">
         <v>3</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>4</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="15" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="B41" s="15" t="s">
         <v>5</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>21</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -7428,7 +7677,7 @@
         <v>0</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -7439,7 +7688,7 @@
         <v>1</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -7447,10 +7696,10 @@
         <v>7</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update project documentation and game data to reflect title change and gameplay mechanics
- Changed project title from "A Final Spell" to "Too Many Orbs" across multiple documentation files, including `GAME_BRIEF.md`, `DECISIONS.md`, and `PROJECT_MAP.md`, to align with the new game focus.
- Updated source-of-truth design document references to "Too Many Orbs.txt" in relevant files.
- Revised `game_data.json` to replace the "Blight" status effect with "Spore" and adjusted descriptions for clarity.
- Deleted outdated glyph image `blight_glyph.png` to streamline asset management.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{557E8C13-5900-460C-8AE7-C6521D70516F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C233A95-2789-4316-A9A8-C74FB0B66E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="308">
   <si>
     <t>id</t>
   </si>
@@ -247,9 +247,6 @@
     <t>blight</t>
   </si>
   <si>
-    <t>Poison on enemy hit</t>
-  </si>
-  <si>
     <t>dense</t>
   </si>
   <si>
@@ -328,27 +325,15 @@
     <t>shatter</t>
   </si>
   <si>
-    <t>If orb hits an enemy with 10 or more chill, kill it instantly</t>
-  </si>
-  <si>
     <t>carrion</t>
   </si>
   <si>
-    <t>On enemy death, a putrid cloud is left inflicting 1 poison on passing enemies</t>
-  </si>
-  <si>
     <t>outbreak</t>
   </si>
   <si>
-    <t>Nearby enemies also get Disease status along with the poison</t>
-  </si>
-  <si>
     <t>virulence</t>
   </si>
   <si>
-    <t>All poison stacks spread on death</t>
-  </si>
-  <si>
     <t>Any picked up glyph goes up in rarity</t>
   </si>
   <si>
@@ -871,9 +856,6 @@
     <t>Seeks out the marked enemy</t>
   </si>
   <si>
-    <t>The marked enemy gets 10 chill</t>
-  </si>
-  <si>
     <t>stalk</t>
   </si>
   <si>
@@ -901,9 +883,6 @@
     <t>Knockback strength. Enemies slammed into each other take this as damage; breakables take more damage</t>
   </si>
   <si>
-    <t>Stacks on hit. On death, the enemy explodes for more damage in a wider area the more stacks it had</t>
-  </si>
-  <si>
     <t>Stacks on hit. Each stack slows move and attack speed by 5% (up to 90%)</t>
   </si>
   <si>
@@ -949,31 +928,46 @@
     <t>Every destroyed object increases weight by 1</t>
   </si>
   <si>
-    <t>smolder</t>
-  </si>
-  <si>
-    <t>Leaves a trail of fire after the orb for 2 seconds, inflicting 1 Smolder on enemies</t>
-  </si>
-  <si>
     <t>nova</t>
   </si>
   <si>
     <t>Makes a frost nova around the orb every 3 seconds inflicting 5 Chill</t>
   </si>
   <si>
-    <t>charge</t>
-  </si>
-  <si>
-    <t>rot</t>
-  </si>
-  <si>
-    <t>20% chance of adding Disease status to enemies. On death half their Rot spreads to other nearby enemies</t>
-  </si>
-  <si>
     <t>Shoots ice chards around every 3 seconds, doing 30 damage and inflicting 2 Chill</t>
   </si>
   <si>
-    <t>Spews magma around it. Magma inflicts Smolder on passing enemies</t>
+    <t>Stacks on hit. Lowers damage dealt and increases damage received by 5% per stack.</t>
+  </si>
+  <si>
+    <t>Blight on enemy hit</t>
+  </si>
+  <si>
+    <t>spore</t>
+  </si>
+  <si>
+    <t>20% chance of adding Disease status to enemies. On death half their Blight spreads to other nearby enemies</t>
+  </si>
+  <si>
+    <t>Leaves a trail of fire after the orb for 2 seconds, inflicting 1 Burn on enemies</t>
+  </si>
+  <si>
+    <t>Spews magma around it. Magma inflicts Burn on passing enemies</t>
+  </si>
+  <si>
+    <t>The marked enemy gets 10 Chill</t>
+  </si>
+  <si>
+    <t>All Blight stacks spread on death</t>
+  </si>
+  <si>
+    <t>Nearby enemies also get Disease status along with the Blight</t>
+  </si>
+  <si>
+    <t>On enemy death, a putrid cloud is left inflicting 1 Blighton passing enemies</t>
+  </si>
+  <si>
+    <t>If orb hits an enemy with 10 or more Chill, kill it instantly</t>
   </si>
 </sst>
 </file>
@@ -1576,16 +1570,16 @@
         <v>15</v>
       </c>
       <c r="R1" s="9" t="s">
-        <v>301</v>
+        <v>16</v>
       </c>
       <c r="S1" s="9" t="s">
         <v>17</v>
       </c>
       <c r="T1" s="9" t="s">
-        <v>305</v>
+        <v>18</v>
       </c>
       <c r="U1" s="9" t="s">
-        <v>306</v>
+        <v>66</v>
       </c>
       <c r="V1" s="13" t="s">
         <v>20</v>
@@ -1740,7 +1734,7 @@
         <v>Contagion</v>
       </c>
       <c r="C4" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="D4" t="s">
         <v>30</v>
@@ -1815,7 +1809,7 @@
         <v>Ghost</v>
       </c>
       <c r="C5" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D5" t="s">
         <v>27</v>
@@ -1890,7 +1884,7 @@
         <v>Inferno</v>
       </c>
       <c r="C6" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D6" t="s">
         <v>28</v>
@@ -1965,7 +1959,7 @@
         <v>Shard</v>
       </c>
       <c r="C7" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="D7" t="s">
         <v>34</v>
@@ -2037,7 +2031,7 @@
         <v>Runic</v>
       </c>
       <c r="C8" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="D8" t="s">
         <v>34</v>
@@ -2165,7 +2159,7 @@
         <v>Yes</v>
       </c>
       <c r="I10" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="V10" t="str">
         <f t="shared" si="3"/>
@@ -2184,7 +2178,7 @@
         <v>Destroyer</v>
       </c>
       <c r="C11" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="D11" t="s">
         <v>28</v>
@@ -2252,14 +2246,14 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Vulcano</v>
       </c>
       <c r="C12" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="D12" t="s">
         <v>28</v>
@@ -2279,7 +2273,7 @@
         <v>Yes</v>
       </c>
       <c r="I12" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="V12" t="str">
         <f>"res://entities/orbs/blank/"&amp;A12&amp;"_orb.tscn"</f>
@@ -2288,14 +2282,14 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" ref="B13:B44" si="4">PROPER(SUBSTITUTE(A13,"_"," "))</f>
         <v>Lure</v>
       </c>
       <c r="C13" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="D13" t="s">
         <v>34</v>
@@ -2325,7 +2319,7 @@
         <v/>
       </c>
       <c r="C14" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="D14" t="s">
         <v>34</v>
@@ -2347,14 +2341,14 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="4"/>
         <v>Hunger</v>
       </c>
       <c r="C15" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="D15" t="s">
         <v>30</v>
@@ -2376,14 +2370,14 @@
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="4"/>
         <v>Vengance</v>
       </c>
       <c r="C16" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D16" t="s">
         <v>27</v>
@@ -2403,19 +2397,19 @@
         <v>Yes</v>
       </c>
       <c r="I16" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="4"/>
         <v>Hunter</v>
       </c>
       <c r="C17" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="D17" t="s">
         <v>28</v>
@@ -2437,14 +2431,14 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="4"/>
         <v>Nova</v>
       </c>
       <c r="C18" t="s">
-        <v>304</v>
+        <v>295</v>
       </c>
       <c r="D18" t="s">
         <v>34</v>
@@ -3732,20 +3726,20 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>299</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
-        <v>Blight</v>
+        <v>Spore</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>298</v>
       </c>
       <c r="D11" t="s">
         <v>30</v>
       </c>
       <c r="E11" t="s">
-        <v>19</v>
+        <v>66</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -3758,19 +3752,19 @@
       </c>
       <c r="I11" t="str">
         <f t="shared" si="1"/>
-        <v>res://items/glyphs/blight_glyph.png</v>
+        <v>res://items/glyphs/spore_glyph.png</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>Dense</v>
+      </c>
+      <c r="C12" t="s">
         <v>68</v>
-      </c>
-      <c r="B12" t="str">
-        <f t="shared" si="0"/>
-        <v>Dense</v>
-      </c>
-      <c r="C12" t="s">
-        <v>69</v>
       </c>
       <c r="D12" t="s">
         <v>30</v>
@@ -3794,14 +3788,14 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>Crush</v>
+      </c>
+      <c r="C13" t="s">
         <v>70</v>
-      </c>
-      <c r="B13" t="str">
-        <f t="shared" si="0"/>
-        <v>Crush</v>
-      </c>
-      <c r="C13" t="s">
-        <v>71</v>
       </c>
       <c r="D13" t="s">
         <v>30</v>
@@ -3861,7 +3855,7 @@
         <v>Damage</v>
       </c>
       <c r="C2" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3873,7 +3867,7 @@
         <v>Splash</v>
       </c>
       <c r="C3" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3885,7 +3879,7 @@
         <v>Burn</v>
       </c>
       <c r="C4" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3897,7 +3891,7 @@
         <v>Self Damage</v>
       </c>
       <c r="C5" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3909,7 +3903,7 @@
         <v>Glyph Drop</v>
       </c>
       <c r="C6" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3921,7 +3915,7 @@
         <v>Chill</v>
       </c>
       <c r="C7" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3933,7 +3927,7 @@
         <v>Crit Chance</v>
       </c>
       <c r="C8" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3945,7 +3939,7 @@
         <v>Speed</v>
       </c>
       <c r="C9" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3957,7 +3951,7 @@
         <v>Shock</v>
       </c>
       <c r="C10" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3969,7 +3963,7 @@
         <v>Weight</v>
       </c>
       <c r="C11" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3981,19 +3975,19 @@
         <v>Crit Damage</v>
       </c>
       <c r="C12" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>66</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
-        <v>Poison</v>
+        <v>Blight</v>
       </c>
       <c r="C13" t="s">
-        <v>288</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>
@@ -4025,7 +4019,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>42</v>
@@ -4045,7 +4039,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B26" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
@@ -4055,7 +4049,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E2" t="s">
         <v>27</v>
@@ -4076,7 +4070,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
@@ -4086,7 +4080,7 @@
         <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E3" t="s">
         <v>28</v>
@@ -4107,7 +4101,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
@@ -4117,7 +4111,7 @@
         <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E4" t="s">
         <v>28</v>
@@ -4138,7 +4132,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
@@ -4148,7 +4142,7 @@
         <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E5" t="s">
         <v>27</v>
@@ -4169,7 +4163,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
@@ -4179,7 +4173,7 @@
         <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E6" t="s">
         <v>28</v>
@@ -4200,7 +4194,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
@@ -4210,7 +4204,7 @@
         <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E7" t="s">
         <v>34</v>
@@ -4231,7 +4225,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
@@ -4241,7 +4235,7 @@
         <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E8" t="s">
         <v>27</v>
@@ -4262,7 +4256,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
@@ -4272,7 +4266,7 @@
         <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E9" t="s">
         <v>27</v>
@@ -4293,7 +4287,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -4303,7 +4297,7 @@
         <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="1"/>
@@ -4315,7 +4309,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
@@ -4325,7 +4319,7 @@
         <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H11" t="str">
         <f t="shared" si="1"/>
@@ -4337,7 +4331,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
@@ -4347,7 +4341,7 @@
         <v>33</v>
       </c>
       <c r="D12" t="s">
-        <v>94</v>
+        <v>307</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="1"/>
@@ -4359,7 +4353,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
@@ -4369,7 +4363,7 @@
         <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>306</v>
       </c>
       <c r="H13" t="str">
         <f t="shared" si="1"/>
@@ -4381,7 +4375,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
@@ -4391,7 +4385,7 @@
         <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>98</v>
+        <v>305</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="1"/>
@@ -4403,7 +4397,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
@@ -4413,7 +4407,7 @@
         <v>29</v>
       </c>
       <c r="D15" t="s">
-        <v>100</v>
+        <v>304</v>
       </c>
       <c r="H15" t="str">
         <f t="shared" si="1"/>
@@ -4425,7 +4419,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
@@ -4435,7 +4429,7 @@
         <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E16" t="s">
         <v>34</v>
@@ -4456,7 +4450,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
@@ -4466,7 +4460,7 @@
         <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="E17" t="s">
         <v>28</v>
@@ -4487,7 +4481,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
@@ -4497,7 +4491,7 @@
         <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="E18" t="s">
         <v>34</v>
@@ -4514,7 +4508,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
@@ -4524,7 +4518,7 @@
         <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E19" t="s">
         <v>30</v>
@@ -4545,7 +4539,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
@@ -4555,7 +4549,7 @@
         <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E20" t="s">
         <v>28</v>
@@ -4576,7 +4570,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
@@ -4586,7 +4580,7 @@
         <v>36</v>
       </c>
       <c r="D21" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E21" t="s">
         <v>27</v>
@@ -4607,7 +4601,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
@@ -4617,7 +4611,7 @@
         <v>36</v>
       </c>
       <c r="D22" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="H22" t="str">
         <f t="shared" si="1"/>
@@ -4629,17 +4623,17 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>Experience</v>
       </c>
       <c r="C23" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="D23" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="H23" t="str">
         <f t="shared" si="1"/>
@@ -4651,17 +4645,17 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v>Stalk</v>
       </c>
       <c r="C24" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="D24" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="H24" t="str">
         <f t="shared" si="1"/>
@@ -4673,17 +4667,17 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>Fright</v>
       </c>
       <c r="C25" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="D25" t="s">
-        <v>275</v>
+        <v>303</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="1"/>
@@ -4695,17 +4689,17 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
         <v>Gravity</v>
       </c>
       <c r="C26" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D26" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="H26" t="str">
         <f t="shared" si="1"/>
@@ -5276,19 +5270,19 @@
         <v>Wayward</v>
       </c>
       <c r="C2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Attracted</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -5300,175 +5294,175 @@
         <v>Spite</v>
       </c>
       <c r="C4" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Rooted</v>
       </c>
       <c r="C5" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Patrol</v>
       </c>
       <c r="C6" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Familiar</v>
       </c>
       <c r="C7" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Rail</v>
       </c>
       <c r="C8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Tide</v>
       </c>
       <c r="C9" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>Blink</v>
       </c>
       <c r="C10" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Loyal</v>
       </c>
       <c r="C11" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Hexed</v>
       </c>
       <c r="C12" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Stalker</v>
       </c>
       <c r="C13" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>Herd</v>
       </c>
       <c r="C14" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
         <v>Greedy</v>
       </c>
       <c r="C15" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
         <v>Oathbound</v>
       </c>
       <c r="C16" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>Echo</v>
       </c>
       <c r="C17" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>Phasing</v>
       </c>
       <c r="C18" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -5511,55 +5505,55 @@
         <v>42</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="P1" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="Q1" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="R1" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="T1" s="4" t="s">
         <v>153</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>158</v>
       </c>
       <c r="U1" s="3" t="s">
         <v>21</v>
@@ -5567,17 +5561,17 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B33" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Reception Desk</v>
       </c>
       <c r="C2" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D2" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="F2" s="2">
         <v>0</v>
@@ -5598,13 +5592,13 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="O2">
         <v>2</v>
       </c>
       <c r="T2" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="U2" t="b">
         <v>1</v>
@@ -5612,17 +5606,17 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Straw Pallet</v>
       </c>
       <c r="C3" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="D3" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="F3" s="2">
         <v>1</v>
@@ -5643,10 +5637,10 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
+        <v>157</v>
+      </c>
+      <c r="M3" t="s">
         <v>162</v>
-      </c>
-      <c r="M3" t="s">
-        <v>167</v>
       </c>
       <c r="O3">
         <v>2</v>
@@ -5660,17 +5654,17 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Wood Frame Bed</v>
       </c>
       <c r="C4" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="D4" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="F4" s="2">
         <v>0</v>
@@ -5691,10 +5685,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
+        <v>157</v>
+      </c>
+      <c r="M4" t="s">
         <v>162</v>
-      </c>
-      <c r="M4" t="s">
-        <v>167</v>
       </c>
       <c r="O4">
         <v>2</v>
@@ -5703,10 +5697,10 @@
         <v>0</v>
       </c>
       <c r="S4" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="T4" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="U4" t="b">
         <v>1</v>
@@ -5714,17 +5708,17 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Bunk Bed</v>
       </c>
       <c r="C5" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="D5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="F5" s="2">
         <v>0</v>
@@ -5745,10 +5739,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
+        <v>157</v>
+      </c>
+      <c r="M5" t="s">
         <v>162</v>
-      </c>
-      <c r="M5" t="s">
-        <v>167</v>
       </c>
       <c r="O5">
         <v>2</v>
@@ -5757,10 +5751,10 @@
         <v>1</v>
       </c>
       <c r="S5" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="T5" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="U5" t="b">
         <v>1</v>
@@ -5768,17 +5762,17 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Canopy Bed</v>
       </c>
       <c r="C6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="D6" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="F6" s="2">
         <v>0</v>
@@ -5799,10 +5793,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
+        <v>157</v>
+      </c>
+      <c r="M6" t="s">
         <v>162</v>
-      </c>
-      <c r="M6" t="s">
-        <v>167</v>
       </c>
       <c r="O6">
         <v>2</v>
@@ -5816,17 +5810,17 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Budget Wardrobe</v>
       </c>
       <c r="C7" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D7" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="F7" s="2">
         <v>0</v>
@@ -5847,10 +5841,10 @@
         <v>2</v>
       </c>
       <c r="L7" t="s">
+        <v>157</v>
+      </c>
+      <c r="M7" t="s">
         <v>162</v>
-      </c>
-      <c r="M7" t="s">
-        <v>167</v>
       </c>
       <c r="O7">
         <v>3</v>
@@ -5859,10 +5853,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="T7" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="U7" t="b">
         <v>1</v>
@@ -5870,17 +5864,17 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Fine Wardrobe</v>
       </c>
       <c r="C8" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="D8" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="F8" s="2">
         <v>0</v>
@@ -5901,10 +5895,10 @@
         <v>4</v>
       </c>
       <c r="L8" t="s">
+        <v>157</v>
+      </c>
+      <c r="M8" t="s">
         <v>162</v>
-      </c>
-      <c r="M8" t="s">
-        <v>167</v>
       </c>
       <c r="O8">
         <v>3</v>
@@ -5913,10 +5907,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="T8" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="U8" t="b">
         <v>1</v>
@@ -5924,17 +5918,17 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Ornate Wardrobe</v>
       </c>
       <c r="D9" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E9" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="F9" s="2">
         <v>0</v>
@@ -5955,10 +5949,10 @@
         <v>7</v>
       </c>
       <c r="L9" t="s">
+        <v>157</v>
+      </c>
+      <c r="M9" t="s">
         <v>162</v>
-      </c>
-      <c r="M9" t="s">
-        <v>167</v>
       </c>
       <c r="O9">
         <v>3</v>
@@ -5967,10 +5961,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="T9" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="U9" t="b">
         <v>1</v>
@@ -5978,7 +5972,7 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -6003,10 +5997,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
+        <v>157</v>
+      </c>
+      <c r="M10" t="s">
         <v>162</v>
-      </c>
-      <c r="M10" t="s">
-        <v>167</v>
       </c>
       <c r="O10">
         <v>1</v>
@@ -6020,14 +6014,14 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Wash Basin</v>
       </c>
       <c r="E11" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="F11" s="2">
         <v>0</v>
@@ -6048,10 +6042,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
+        <v>157</v>
+      </c>
+      <c r="M11" t="s">
         <v>162</v>
-      </c>
-      <c r="M11" t="s">
-        <v>167</v>
       </c>
       <c r="O11">
         <v>1</v>
@@ -6065,14 +6059,14 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Artisan Rug</v>
       </c>
       <c r="E12" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="F12" s="2">
         <v>0</v>
@@ -6093,7 +6087,7 @@
         <v>4</v>
       </c>
       <c r="L12" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="O12">
         <v>2</v>
@@ -6107,14 +6101,14 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Mirror</v>
       </c>
       <c r="E13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="F13" s="2">
         <v>0</v>
@@ -6135,10 +6129,10 @@
         <v>3</v>
       </c>
       <c r="L13" t="s">
+        <v>157</v>
+      </c>
+      <c r="M13" t="s">
         <v>162</v>
-      </c>
-      <c r="M13" t="s">
-        <v>167</v>
       </c>
       <c r="O13">
         <v>1</v>
@@ -6152,14 +6146,14 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>Trunk</v>
       </c>
       <c r="C14" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="F14" s="2">
         <v>0</v>
@@ -6180,10 +6174,10 @@
         <v>1</v>
       </c>
       <c r="L14" t="s">
+        <v>157</v>
+      </c>
+      <c r="M14" t="s">
         <v>162</v>
-      </c>
-      <c r="M14" t="s">
-        <v>167</v>
       </c>
       <c r="O14">
         <v>2</v>
@@ -6197,7 +6191,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
@@ -6222,7 +6216,7 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="O15">
         <v>3</v>
@@ -6236,7 +6230,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
@@ -6261,10 +6255,10 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
+        <v>157</v>
+      </c>
+      <c r="M16" t="s">
         <v>162</v>
-      </c>
-      <c r="M16" t="s">
-        <v>167</v>
       </c>
       <c r="O16">
         <v>1</v>
@@ -6278,14 +6272,14 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>Small Houseplant</v>
       </c>
       <c r="D17" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="F17" s="2">
         <v>0</v>
@@ -6306,7 +6300,7 @@
         <v>4</v>
       </c>
       <c r="L17" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="O17">
         <v>1</v>
@@ -6315,10 +6309,10 @@
         <v>0</v>
       </c>
       <c r="S17" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="T17" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="U17" t="b">
         <v>1</v>
@@ -6326,14 +6320,14 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>Big Houseplant</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="F18" s="2">
         <v>0</v>
@@ -6354,7 +6348,7 @@
         <v>6</v>
       </c>
       <c r="L18" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="O18">
         <v>2</v>
@@ -6368,14 +6362,14 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
         <v>Chamber Pot</v>
       </c>
       <c r="C19" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="F19" s="2">
         <v>0</v>
@@ -6396,10 +6390,10 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="M19" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="O19">
         <v>1</v>
@@ -6413,17 +6407,17 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
         <v>Cooking Order Desk</v>
       </c>
       <c r="C20" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="D20" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="F20" s="2">
         <v>0</v>
@@ -6444,10 +6438,10 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="M20" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="O20">
         <v>2</v>
@@ -6456,10 +6450,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="T20" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="U20" t="b">
         <v>1</v>
@@ -6467,17 +6461,17 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
         <v>Cooking Couldron</v>
       </c>
       <c r="C21" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="D21" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="F21" s="2">
         <v>0</v>
@@ -6498,10 +6492,10 @@
         <v>0</v>
       </c>
       <c r="L21" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="M21" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="O21">
         <v>2</v>
@@ -6510,10 +6504,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="T21" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="U21" t="b">
         <v>1</v>
@@ -6521,14 +6515,14 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v>Small Seating Table</v>
       </c>
       <c r="D22" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="F22" s="2">
         <v>0</v>
@@ -6549,10 +6543,10 @@
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="M22" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="O22">
         <v>2</v>
@@ -6561,10 +6555,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="T22" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="U22" t="b">
         <v>1</v>
@@ -6572,17 +6566,17 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>Pass Table</v>
       </c>
       <c r="C23" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="D23" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="F23" s="2">
         <v>0</v>
@@ -6603,10 +6597,10 @@
         <v>1</v>
       </c>
       <c r="L23" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="M23" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="O23">
         <v>2</v>
@@ -6615,10 +6609,10 @@
         <v>0</v>
       </c>
       <c r="S23" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="T23" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="U23" t="b">
         <v>1</v>
@@ -6626,17 +6620,17 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v>Crate</v>
       </c>
       <c r="C24" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="D24" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="F24" s="2">
         <v>0</v>
@@ -6657,7 +6651,7 @@
         <v>0</v>
       </c>
       <c r="L24" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="O24">
         <v>2</v>
@@ -6666,10 +6660,10 @@
         <v>0</v>
       </c>
       <c r="S24" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="T24" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="U24" t="b">
         <v>1</v>
@@ -6677,17 +6671,17 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>Barrel</v>
       </c>
       <c r="C25" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="D25" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="F25" s="2">
         <v>0</v>
@@ -6708,7 +6702,7 @@
         <v>0</v>
       </c>
       <c r="L25" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="O25">
         <v>2</v>
@@ -6717,10 +6711,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="T25" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="U25" t="b">
         <v>1</v>
@@ -6728,17 +6722,17 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
         <v>Wall Torch</v>
       </c>
       <c r="C26" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="D26" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="F26" s="2">
         <v>0</v>
@@ -6759,7 +6753,7 @@
         <v>0</v>
       </c>
       <c r="L26" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="O26">
         <v>0</v>
@@ -6771,10 +6765,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="T26" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="U26" t="b">
         <v>1</v>
@@ -6782,17 +6776,17 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
         <v>Condiment Shelf</v>
       </c>
       <c r="C27" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="D27" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="F27" s="2">
         <v>0</v>
@@ -6813,10 +6807,10 @@
         <v>2</v>
       </c>
       <c r="L27" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="M27" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="O27">
         <v>1</v>
@@ -6828,10 +6822,10 @@
         <v>0</v>
       </c>
       <c r="S27" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="T27" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="U27" t="b">
         <v>1</v>
@@ -6839,17 +6833,17 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>Condiment Shelf Small</v>
       </c>
       <c r="C28" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="D28" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="F28" s="2">
         <v>0</v>
@@ -6870,10 +6864,10 @@
         <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="M28" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="O28">
         <v>1</v>
@@ -6885,10 +6879,10 @@
         <v>0</v>
       </c>
       <c r="S28" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="T28" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="U28" t="b">
         <v>1</v>
@@ -6896,17 +6890,17 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>Hanging Frying Pans</v>
       </c>
       <c r="C29" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="D29" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="F29" s="2">
         <v>0</v>
@@ -6927,10 +6921,10 @@
         <v>0</v>
       </c>
       <c r="L29" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="M29" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="O29">
         <v>0</v>
@@ -6941,14 +6935,14 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="0"/>
         <v>Butcher Table</v>
       </c>
       <c r="D30" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="F30" s="2">
         <v>0</v>
@@ -6969,10 +6963,10 @@
         <v>3</v>
       </c>
       <c r="L30" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="M30" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="O30">
         <v>2</v>
@@ -6983,14 +6977,14 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>Hanging Meat</v>
       </c>
       <c r="D31" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -7173,10 +7167,10 @@
   <sheetData>
     <row r="2" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C2" t="s">
         <v>28</v>
@@ -7209,343 +7203,343 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="B1" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C1" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>16</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>19</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>20</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>0</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B26" s="12" t="s">
         <v>43</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B27" s="12" t="s">
         <v>44</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>45</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B29" s="12" t="s">
         <v>46</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B30" s="12" t="s">
         <v>47</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>20</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -7556,7 +7550,7 @@
         <v>0</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -7567,7 +7561,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -7578,95 +7572,95 @@
         <v>42</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B35" s="15" t="s">
         <v>0</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>1</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>42</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B39" s="15" t="s">
         <v>3</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>4</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="15" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B41" s="15" t="s">
         <v>5</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>21</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -7677,7 +7671,7 @@
         <v>0</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -7688,7 +7682,7 @@
         <v>1</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -7699,7 +7693,7 @@
         <v>42</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor summoning circle mechanics and update gameplay documentation for enhanced orb interactions
- Revised the summoning circle to support real-time orb capture and interactions without pausing the game, improving co-op gameplay fluidity.
- Updated `DECISIONS.md` to reflect changes in orb activation, upgrade, and ritual cancel mechanics, including proximity-based interactions.
- Adjusted `GAME_BRIEF.md` and `PROJECT_MAP.md` to incorporate new mechanics for orb purchasing and transformation during rituals.
- Enhanced player controls for clearer input handling related to summoning circle actions, ensuring a smoother gameplay experience.
- Improved orb behavior during capture and release, maintaining game flow and player engagement.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C233A95-2789-4316-A9A8-C74FB0B66E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4817CA53-7466-42A8-8067-5F92F7D508B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -952,9 +952,6 @@
     <t>Leaves a trail of fire after the orb for 2 seconds, inflicting 1 Burn on enemies</t>
   </si>
   <si>
-    <t>Spews magma around it. Magma inflicts Burn on passing enemies</t>
-  </si>
-  <si>
     <t>The marked enemy gets 10 Chill</t>
   </si>
   <si>
@@ -968,6 +965,9 @@
   </si>
   <si>
     <t>If orb hits an enemy with 10 or more Chill, kill it instantly</t>
+  </si>
+  <si>
+    <t>Spews lava puddles around it. Lava inflicts 1 Burn per second on passing enemies</t>
   </si>
 </sst>
 </file>
@@ -1500,7 +1500,7 @@
   <cols>
     <col min="1" max="1" width="19.42578125" customWidth="1"/>
     <col min="2" max="2" width="17.5703125" customWidth="1"/>
-    <col min="3" max="3" width="104.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="114.7109375" customWidth="1"/>
     <col min="4" max="4" width="16.7109375" customWidth="1"/>
     <col min="5" max="5" width="10.5703125" customWidth="1"/>
     <col min="6" max="6" width="13.42578125" customWidth="1"/>
@@ -2253,7 +2253,7 @@
         <v>Vulcano</v>
       </c>
       <c r="C12" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="D12" t="s">
         <v>28</v>
@@ -2275,9 +2275,48 @@
       <c r="I12" t="s">
         <v>110</v>
       </c>
+      <c r="J12">
+        <v>15</v>
+      </c>
+      <c r="K12">
+        <v>15</v>
+      </c>
+      <c r="L12" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="M12" s="8">
+        <v>2</v>
+      </c>
+      <c r="N12">
+        <v>100</v>
+      </c>
+      <c r="O12">
+        <v>6</v>
+      </c>
+      <c r="P12" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="R12">
+        <v>2</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
       <c r="V12" t="str">
         <f>"res://entities/orbs/blank/"&amp;A12&amp;"_orb.tscn"</f>
         <v>res://entities/orbs/blank/vulcano_orb.tscn</v>
+      </c>
+      <c r="W12" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
@@ -4341,7 +4380,7 @@
         <v>33</v>
       </c>
       <c r="D12" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="1"/>
@@ -4363,7 +4402,7 @@
         <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H13" t="str">
         <f t="shared" si="1"/>
@@ -4385,7 +4424,7 @@
         <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="1"/>
@@ -4407,7 +4446,7 @@
         <v>29</v>
       </c>
       <c r="D15" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H15" t="str">
         <f t="shared" si="1"/>
@@ -4677,7 +4716,7 @@
         <v>266</v>
       </c>
       <c r="D25" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
Enhance orb mechanics and update documentation for new Vulcano orb
- Introduced the Vulcano orb, which features a rooted motion mechanic that allows it to slide and park, creating lava puddles that apply burn damage to enemies.
- Updated `DECISIONS.md` to reflect the addition of the Vulcano orb and its unique mechanics, including its interaction with other orbs and gameplay strategies.
- Revised `GAME_BRIEF.md` and `PROJECT_MAP.md` to include details about the Vulcano orb's abilities and its integration into the game.
- Adjusted `game_data.json` to ensure accurate descriptions and functionality for the new Vulcano orb and its associated effects.
- Enhanced player experience by incorporating the Vulcano orb into the starting orb selection for gameplay variety.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4817CA53-7466-42A8-8067-5F92F7D508B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85D5B4BD-C992-46EE-A519-EC9B0CFA5A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2276,7 +2276,7 @@
         <v>110</v>
       </c>
       <c r="J12">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="K12">
         <v>15</v>
@@ -2288,7 +2288,7 @@
         <v>2</v>
       </c>
       <c r="N12">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="O12">
         <v>6</v>

</xml_diff>

<commit_message>
Refine Vulcano orb mechanics and enhance related documentation
- Updated the Vulcano orb's behavior to function as a turret while parked, with improved hitbox management and lava globe spewing mechanics.
- Revised `DECISIONS.md` to reflect the new turret functionality and its interaction with the game environment.
- Enhanced `GAME_BRIEF.md` and `PROJECT_MAP.md` to include detailed descriptions of the Vulcano orb's updated abilities and gameplay strategies.
- Adjusted `game_data.json` to ensure accurate descriptions of the Vulcano orb's effects and interactions.
- Improved the visual representation of lava globes and puddles, including new animations for the expiration phase.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85D5B4BD-C992-46EE-A519-EC9B0CFA5A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1444AE99-37BD-45D7-B4F3-31AF6E1E89DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -343,9 +343,6 @@
     <t>affinity</t>
   </si>
   <si>
-    <t>While holding a glyph, inflict 5 of that glyphs corresponding elemental status to any hit enemies (burn, chill, shock or poison)</t>
-  </si>
-  <si>
     <t>retribution</t>
   </si>
   <si>
@@ -907,18 +904,12 @@
     <t>secure</t>
   </si>
   <si>
-    <t>Droped glyphs gets a shield protecting against one damage instance</t>
-  </si>
-  <si>
     <t>Gets 5% damage increase for each dropped glyph</t>
   </si>
   <si>
     <t>Enters and haunts enemies and deal its damage per second to them. Once dead, exits in a random direction.</t>
   </si>
   <si>
-    <t>Seeks glyphs out and picks them up instead of damaging them. Seeks out the summoning circle and drops them near</t>
-  </si>
-  <si>
     <t>gravity</t>
   </si>
   <si>
@@ -968,6 +959,15 @@
   </si>
   <si>
     <t>Spews lava puddles around it. Lava inflicts 1 Burn per second on passing enemies</t>
+  </si>
+  <si>
+    <t>While holding a glyph, inflict 5 of that glyphs corresponding elemental status to any hit enemies (burn, chill, shock or blight)</t>
+  </si>
+  <si>
+    <t>Dropped glyphs gets a shield protecting against one damage instance</t>
+  </si>
+  <si>
+    <t>Seeks out and picks up glyphs and drops them near the summoning circle.</t>
   </si>
 </sst>
 </file>
@@ -1734,7 +1734,7 @@
         <v>Contagion</v>
       </c>
       <c r="C4" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="D4" t="s">
         <v>30</v>
@@ -1809,7 +1809,7 @@
         <v>Ghost</v>
       </c>
       <c r="C5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D5" t="s">
         <v>27</v>
@@ -1884,7 +1884,7 @@
         <v>Inferno</v>
       </c>
       <c r="C6" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="D6" t="s">
         <v>28</v>
@@ -1959,7 +1959,7 @@
         <v>Shard</v>
       </c>
       <c r="C7" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D7" t="s">
         <v>34</v>
@@ -2031,7 +2031,7 @@
         <v>Runic</v>
       </c>
       <c r="C8" t="s">
-        <v>290</v>
+        <v>307</v>
       </c>
       <c r="D8" t="s">
         <v>34</v>
@@ -2091,7 +2091,7 @@
         <v>res://entities/orbs/blank/runic_orb.tscn</v>
       </c>
       <c r="W8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
@@ -2159,7 +2159,7 @@
         <v>Yes</v>
       </c>
       <c r="I10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="V10" t="str">
         <f t="shared" si="3"/>
@@ -2178,7 +2178,7 @@
         <v>Destroyer</v>
       </c>
       <c r="C11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D11" t="s">
         <v>28</v>
@@ -2246,14 +2246,14 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Vulcano</v>
       </c>
       <c r="C12" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="D12" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>Yes</v>
       </c>
       <c r="I12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J12">
         <v>5</v>
@@ -2321,14 +2321,14 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" ref="B13:B44" si="4">PROPER(SUBSTITUTE(A13,"_"," "))</f>
         <v>Lure</v>
       </c>
       <c r="C13" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D13" t="s">
         <v>34</v>
@@ -2358,7 +2358,7 @@
         <v/>
       </c>
       <c r="C14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D14" t="s">
         <v>34</v>
@@ -2380,14 +2380,14 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="4"/>
         <v>Hunger</v>
       </c>
       <c r="C15" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D15" t="s">
         <v>30</v>
@@ -2409,14 +2409,14 @@
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="4"/>
         <v>Vengance</v>
       </c>
       <c r="C16" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D16" t="s">
         <v>27</v>
@@ -2436,19 +2436,19 @@
         <v>Yes</v>
       </c>
       <c r="I16" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="4"/>
         <v>Hunter</v>
       </c>
       <c r="C17" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D17" t="s">
         <v>28</v>
@@ -2470,14 +2470,14 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="4"/>
         <v>Nova</v>
       </c>
       <c r="C18" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D18" t="s">
         <v>34</v>
@@ -3765,14 +3765,14 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Spore</v>
       </c>
       <c r="C11" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D11" t="s">
         <v>30</v>
@@ -3894,7 +3894,7 @@
         <v>Damage</v>
       </c>
       <c r="C2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3906,7 +3906,7 @@
         <v>Splash</v>
       </c>
       <c r="C3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3918,7 +3918,7 @@
         <v>Burn</v>
       </c>
       <c r="C4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3930,7 +3930,7 @@
         <v>Self Damage</v>
       </c>
       <c r="C5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3942,7 +3942,7 @@
         <v>Glyph Drop</v>
       </c>
       <c r="C6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3954,7 +3954,7 @@
         <v>Chill</v>
       </c>
       <c r="C7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3966,7 +3966,7 @@
         <v>Crit Chance</v>
       </c>
       <c r="C8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3978,7 +3978,7 @@
         <v>Speed</v>
       </c>
       <c r="C9" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3990,7 +3990,7 @@
         <v>Shock</v>
       </c>
       <c r="C10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -4002,7 +4002,7 @@
         <v>Weight</v>
       </c>
       <c r="C11" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -4014,7 +4014,7 @@
         <v>Crit Damage</v>
       </c>
       <c r="C12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -4026,7 +4026,7 @@
         <v>Blight</v>
       </c>
       <c r="C13" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -4380,7 +4380,7 @@
         <v>33</v>
       </c>
       <c r="D12" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="1"/>
@@ -4402,7 +4402,7 @@
         <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="H13" t="str">
         <f t="shared" si="1"/>
@@ -4424,7 +4424,7 @@
         <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="1"/>
@@ -4446,7 +4446,7 @@
         <v>29</v>
       </c>
       <c r="D15" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="H15" t="str">
         <f t="shared" si="1"/>
@@ -4458,7 +4458,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
@@ -4499,7 +4499,7 @@
         <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E17" t="s">
         <v>28</v>
@@ -4520,7 +4520,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
@@ -4530,7 +4530,7 @@
         <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>287</v>
+        <v>306</v>
       </c>
       <c r="E18" t="s">
         <v>34</v>
@@ -4557,7 +4557,7 @@
         <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>99</v>
+        <v>305</v>
       </c>
       <c r="E19" t="s">
         <v>30</v>
@@ -4578,7 +4578,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
@@ -4588,7 +4588,7 @@
         <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E20" t="s">
         <v>28</v>
@@ -4609,7 +4609,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
@@ -4619,7 +4619,7 @@
         <v>36</v>
       </c>
       <c r="D21" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E21" t="s">
         <v>27</v>
@@ -4640,7 +4640,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
@@ -4650,7 +4650,7 @@
         <v>36</v>
       </c>
       <c r="D22" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H22" t="str">
         <f t="shared" si="1"/>
@@ -4662,17 +4662,17 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>Experience</v>
       </c>
       <c r="C23" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D23" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="H23" t="str">
         <f t="shared" si="1"/>
@@ -4684,17 +4684,17 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v>Stalk</v>
       </c>
       <c r="C24" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D24" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H24" t="str">
         <f t="shared" si="1"/>
@@ -4706,17 +4706,17 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>Fright</v>
       </c>
       <c r="C25" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D25" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="1"/>
@@ -4728,17 +4728,17 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
         <v>Gravity</v>
       </c>
       <c r="C26" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D26" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="H26" t="str">
         <f t="shared" si="1"/>
@@ -5309,19 +5309,19 @@
         <v>Wayward</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" si="0"/>
+        <v>Attracted</v>
+      </c>
+      <c r="C3" t="s">
         <v>107</v>
-      </c>
-      <c r="B3" t="str">
-        <f t="shared" si="0"/>
-        <v>Attracted</v>
-      </c>
-      <c r="C3" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -5333,175 +5333,175 @@
         <v>Spite</v>
       </c>
       <c r="C4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Rooted</v>
+      </c>
+      <c r="C5" t="s">
         <v>110</v>
-      </c>
-      <c r="B5" t="str">
-        <f t="shared" si="0"/>
-        <v>Rooted</v>
-      </c>
-      <c r="C5" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>Patrol</v>
+      </c>
+      <c r="C6" t="s">
         <v>112</v>
-      </c>
-      <c r="B6" t="str">
-        <f t="shared" si="0"/>
-        <v>Patrol</v>
-      </c>
-      <c r="C6" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>Familiar</v>
+      </c>
+      <c r="C7" t="s">
         <v>114</v>
-      </c>
-      <c r="B7" t="str">
-        <f t="shared" si="0"/>
-        <v>Familiar</v>
-      </c>
-      <c r="C7" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>Rail</v>
+      </c>
+      <c r="C8" t="s">
         <v>116</v>
-      </c>
-      <c r="B8" t="str">
-        <f t="shared" si="0"/>
-        <v>Rail</v>
-      </c>
-      <c r="C8" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>Tide</v>
+      </c>
+      <c r="C9" t="s">
         <v>118</v>
-      </c>
-      <c r="B9" t="str">
-        <f t="shared" si="0"/>
-        <v>Tide</v>
-      </c>
-      <c r="C9" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>Blink</v>
+      </c>
+      <c r="C10" t="s">
         <v>120</v>
-      </c>
-      <c r="B10" t="str">
-        <f t="shared" si="0"/>
-        <v>Blink</v>
-      </c>
-      <c r="C10" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>Loyal</v>
+      </c>
+      <c r="C11" t="s">
         <v>122</v>
-      </c>
-      <c r="B11" t="str">
-        <f t="shared" si="0"/>
-        <v>Loyal</v>
-      </c>
-      <c r="C11" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>Hexed</v>
+      </c>
+      <c r="C12" t="s">
         <v>124</v>
-      </c>
-      <c r="B12" t="str">
-        <f t="shared" si="0"/>
-        <v>Hexed</v>
-      </c>
-      <c r="C12" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>Stalker</v>
+      </c>
+      <c r="C13" t="s">
         <v>126</v>
-      </c>
-      <c r="B13" t="str">
-        <f t="shared" si="0"/>
-        <v>Stalker</v>
-      </c>
-      <c r="C13" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>127</v>
+      </c>
+      <c r="B14" t="str">
+        <f t="shared" si="0"/>
+        <v>Herd</v>
+      </c>
+      <c r="C14" t="s">
         <v>128</v>
-      </c>
-      <c r="B14" t="str">
-        <f t="shared" si="0"/>
-        <v>Herd</v>
-      </c>
-      <c r="C14" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>129</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>Greedy</v>
+      </c>
+      <c r="C15" t="s">
         <v>130</v>
-      </c>
-      <c r="B15" t="str">
-        <f t="shared" si="0"/>
-        <v>Greedy</v>
-      </c>
-      <c r="C15" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>131</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>Oathbound</v>
+      </c>
+      <c r="C16" t="s">
         <v>132</v>
-      </c>
-      <c r="B16" t="str">
-        <f t="shared" si="0"/>
-        <v>Oathbound</v>
-      </c>
-      <c r="C16" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>133</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>Echo</v>
+      </c>
+      <c r="C17" t="s">
         <v>134</v>
-      </c>
-      <c r="B17" t="str">
-        <f t="shared" si="0"/>
-        <v>Echo</v>
-      </c>
-      <c r="C17" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>135</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>Phasing</v>
+      </c>
+      <c r="C18" t="s">
         <v>136</v>
-      </c>
-      <c r="B18" t="str">
-        <f t="shared" si="0"/>
-        <v>Phasing</v>
-      </c>
-      <c r="C18" t="s">
-        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -5544,55 +5544,55 @@
         <v>42</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="T1" s="4" t="s">
         <v>152</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>153</v>
       </c>
       <c r="U1" s="3" t="s">
         <v>21</v>
@@ -5600,44 +5600,44 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B33" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Reception Desk</v>
       </c>
       <c r="C2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D2" t="s">
         <v>155</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" s="2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+      <c r="L2" t="s">
         <v>156</v>
-      </c>
-      <c r="F2" s="2">
-        <v>0</v>
-      </c>
-      <c r="G2" s="2">
-        <v>0</v>
-      </c>
-      <c r="H2" s="2">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2">
-        <v>0</v>
-      </c>
-      <c r="J2" s="2">
-        <v>0</v>
-      </c>
-      <c r="K2" s="2">
-        <v>0</v>
-      </c>
-      <c r="L2" t="s">
-        <v>157</v>
       </c>
       <c r="O2">
         <v>2</v>
       </c>
       <c r="T2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="U2" t="b">
         <v>1</v>
@@ -5645,17 +5645,17 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" si="0"/>
+        <v>Straw Pallet</v>
+      </c>
+      <c r="C3" t="s">
         <v>159</v>
       </c>
-      <c r="B3" t="str">
-        <f t="shared" si="0"/>
-        <v>Straw Pallet</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>160</v>
-      </c>
-      <c r="D3" t="s">
-        <v>161</v>
       </c>
       <c r="F3" s="2">
         <v>1</v>
@@ -5676,10 +5676,10 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O3">
         <v>2</v>
@@ -5693,17 +5693,17 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>Wood Frame Bed</v>
+      </c>
+      <c r="C4" t="s">
         <v>163</v>
       </c>
-      <c r="B4" t="str">
-        <f t="shared" si="0"/>
-        <v>Wood Frame Bed</v>
-      </c>
-      <c r="C4" t="s">
-        <v>164</v>
-      </c>
       <c r="D4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F4" s="2">
         <v>0</v>
@@ -5724,10 +5724,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O4">
         <v>2</v>
@@ -5736,10 +5736,10 @@
         <v>0</v>
       </c>
       <c r="S4" t="s">
+        <v>164</v>
+      </c>
+      <c r="T4" t="s">
         <v>165</v>
-      </c>
-      <c r="T4" t="s">
-        <v>166</v>
       </c>
       <c r="U4" t="b">
         <v>1</v>
@@ -5747,17 +5747,17 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>166</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Bunk Bed</v>
+      </c>
+      <c r="C5" t="s">
         <v>167</v>
       </c>
-      <c r="B5" t="str">
-        <f t="shared" si="0"/>
-        <v>Bunk Bed</v>
-      </c>
-      <c r="C5" t="s">
-        <v>168</v>
-      </c>
       <c r="D5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F5" s="2">
         <v>0</v>
@@ -5778,10 +5778,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O5">
         <v>2</v>
@@ -5790,10 +5790,10 @@
         <v>1</v>
       </c>
       <c r="S5" t="s">
+        <v>168</v>
+      </c>
+      <c r="T5" t="s">
         <v>169</v>
-      </c>
-      <c r="T5" t="s">
-        <v>170</v>
       </c>
       <c r="U5" t="b">
         <v>1</v>
@@ -5801,17 +5801,17 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>Canopy Bed</v>
+      </c>
+      <c r="C6" t="s">
         <v>171</v>
       </c>
-      <c r="B6" t="str">
-        <f t="shared" si="0"/>
-        <v>Canopy Bed</v>
-      </c>
-      <c r="C6" t="s">
-        <v>172</v>
-      </c>
       <c r="D6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F6" s="2">
         <v>0</v>
@@ -5832,10 +5832,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O6">
         <v>2</v>
@@ -5849,17 +5849,17 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>172</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>Budget Wardrobe</v>
+      </c>
+      <c r="C7" t="s">
         <v>173</v>
       </c>
-      <c r="B7" t="str">
-        <f t="shared" si="0"/>
-        <v>Budget Wardrobe</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>174</v>
-      </c>
-      <c r="D7" t="s">
-        <v>175</v>
       </c>
       <c r="F7" s="2">
         <v>0</v>
@@ -5880,10 +5880,10 @@
         <v>2</v>
       </c>
       <c r="L7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O7">
         <v>3</v>
@@ -5892,10 +5892,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="s">
+        <v>175</v>
+      </c>
+      <c r="T7" t="s">
         <v>176</v>
-      </c>
-      <c r="T7" t="s">
-        <v>177</v>
       </c>
       <c r="U7" t="b">
         <v>1</v>
@@ -5903,17 +5903,17 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>Fine Wardrobe</v>
+      </c>
+      <c r="C8" t="s">
         <v>178</v>
       </c>
-      <c r="B8" t="str">
-        <f t="shared" si="0"/>
-        <v>Fine Wardrobe</v>
-      </c>
-      <c r="C8" t="s">
-        <v>179</v>
-      </c>
       <c r="D8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F8" s="2">
         <v>0</v>
@@ -5934,10 +5934,10 @@
         <v>4</v>
       </c>
       <c r="L8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O8">
         <v>3</v>
@@ -5946,10 +5946,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="U8" t="b">
         <v>1</v>
@@ -5957,17 +5957,17 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>180</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>Ornate Wardrobe</v>
+      </c>
+      <c r="D9" t="s">
+        <v>174</v>
+      </c>
+      <c r="E9" t="s">
         <v>181</v>
-      </c>
-      <c r="B9" t="str">
-        <f t="shared" si="0"/>
-        <v>Ornate Wardrobe</v>
-      </c>
-      <c r="D9" t="s">
-        <v>175</v>
-      </c>
-      <c r="E9" t="s">
-        <v>182</v>
       </c>
       <c r="F9" s="2">
         <v>0</v>
@@ -5988,10 +5988,10 @@
         <v>7</v>
       </c>
       <c r="L9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O9">
         <v>3</v>
@@ -6000,10 +6000,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="U9" t="b">
         <v>1</v>
@@ -6011,7 +6011,7 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -6036,10 +6036,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O10">
         <v>1</v>
@@ -6053,14 +6053,14 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>Wash Basin</v>
+      </c>
+      <c r="E11" t="s">
         <v>185</v>
-      </c>
-      <c r="B11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wash Basin</v>
-      </c>
-      <c r="E11" t="s">
-        <v>186</v>
       </c>
       <c r="F11" s="2">
         <v>0</v>
@@ -6081,10 +6081,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O11">
         <v>1</v>
@@ -6098,14 +6098,14 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>Artisan Rug</v>
+      </c>
+      <c r="E12" t="s">
         <v>187</v>
-      </c>
-      <c r="B12" t="str">
-        <f t="shared" si="0"/>
-        <v>Artisan Rug</v>
-      </c>
-      <c r="E12" t="s">
-        <v>188</v>
       </c>
       <c r="F12" s="2">
         <v>0</v>
@@ -6126,7 +6126,7 @@
         <v>4</v>
       </c>
       <c r="L12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O12">
         <v>2</v>
@@ -6140,14 +6140,14 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>Mirror</v>
+      </c>
+      <c r="E13" t="s">
         <v>189</v>
-      </c>
-      <c r="B13" t="str">
-        <f t="shared" si="0"/>
-        <v>Mirror</v>
-      </c>
-      <c r="E13" t="s">
-        <v>190</v>
       </c>
       <c r="F13" s="2">
         <v>0</v>
@@ -6168,10 +6168,10 @@
         <v>3</v>
       </c>
       <c r="L13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O13">
         <v>1</v>
@@ -6185,14 +6185,14 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="B14" t="str">
+        <f t="shared" si="0"/>
+        <v>Trunk</v>
+      </c>
+      <c r="C14" t="s">
         <v>191</v>
-      </c>
-      <c r="B14" t="str">
-        <f t="shared" si="0"/>
-        <v>Trunk</v>
-      </c>
-      <c r="C14" t="s">
-        <v>192</v>
       </c>
       <c r="F14" s="2">
         <v>0</v>
@@ -6213,10 +6213,10 @@
         <v>1</v>
       </c>
       <c r="L14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O14">
         <v>2</v>
@@ -6230,7 +6230,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
@@ -6255,7 +6255,7 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O15">
         <v>3</v>
@@ -6269,7 +6269,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
@@ -6294,10 +6294,10 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M16" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O16">
         <v>1</v>
@@ -6311,14 +6311,14 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>194</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>Small Houseplant</v>
+      </c>
+      <c r="D17" t="s">
         <v>195</v>
-      </c>
-      <c r="B17" t="str">
-        <f t="shared" si="0"/>
-        <v>Small Houseplant</v>
-      </c>
-      <c r="D17" t="s">
-        <v>196</v>
       </c>
       <c r="F17" s="2">
         <v>0</v>
@@ -6339,7 +6339,7 @@
         <v>4</v>
       </c>
       <c r="L17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O17">
         <v>1</v>
@@ -6348,10 +6348,10 @@
         <v>0</v>
       </c>
       <c r="S17" t="s">
+        <v>196</v>
+      </c>
+      <c r="T17" t="s">
         <v>197</v>
-      </c>
-      <c r="T17" t="s">
-        <v>198</v>
       </c>
       <c r="U17" t="b">
         <v>1</v>
@@ -6359,14 +6359,14 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>Big Houseplant</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>199</v>
-      </c>
-      <c r="B18" t="str">
-        <f t="shared" si="0"/>
-        <v>Big Houseplant</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>200</v>
       </c>
       <c r="F18" s="2">
         <v>0</v>
@@ -6387,7 +6387,7 @@
         <v>6</v>
       </c>
       <c r="L18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O18">
         <v>2</v>
@@ -6401,14 +6401,14 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
+        <v>Chamber Pot</v>
+      </c>
+      <c r="C19" t="s">
         <v>201</v>
-      </c>
-      <c r="B19" t="str">
-        <f t="shared" si="0"/>
-        <v>Chamber Pot</v>
-      </c>
-      <c r="C19" t="s">
-        <v>202</v>
       </c>
       <c r="F19" s="2">
         <v>0</v>
@@ -6429,10 +6429,10 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M19" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O19">
         <v>1</v>
@@ -6446,41 +6446,41 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>202</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>Cooking Order Desk</v>
+      </c>
+      <c r="C20" t="s">
         <v>203</v>
       </c>
-      <c r="B20" t="str">
-        <f t="shared" si="0"/>
-        <v>Cooking Order Desk</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>204</v>
       </c>
-      <c r="D20" t="s">
+      <c r="F20" s="2">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0</v>
+      </c>
+      <c r="H20" s="2">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2">
+        <v>0</v>
+      </c>
+      <c r="J20" s="2">
+        <v>0</v>
+      </c>
+      <c r="K20" s="2">
+        <v>0</v>
+      </c>
+      <c r="L20" t="s">
+        <v>156</v>
+      </c>
+      <c r="M20" t="s">
         <v>205</v>
-      </c>
-      <c r="F20" s="2">
-        <v>0</v>
-      </c>
-      <c r="G20" s="2">
-        <v>0</v>
-      </c>
-      <c r="H20" s="2">
-        <v>0</v>
-      </c>
-      <c r="I20" s="2">
-        <v>0</v>
-      </c>
-      <c r="J20" s="2">
-        <v>0</v>
-      </c>
-      <c r="K20" s="2">
-        <v>0</v>
-      </c>
-      <c r="L20" t="s">
-        <v>157</v>
-      </c>
-      <c r="M20" t="s">
-        <v>206</v>
       </c>
       <c r="O20">
         <v>2</v>
@@ -6489,10 +6489,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="s">
+        <v>206</v>
+      </c>
+      <c r="T20" t="s">
         <v>207</v>
-      </c>
-      <c r="T20" t="s">
-        <v>208</v>
       </c>
       <c r="U20" t="b">
         <v>1</v>
@@ -6500,41 +6500,41 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>208</v>
+      </c>
+      <c r="B21" t="str">
+        <f t="shared" si="0"/>
+        <v>Cooking Couldron</v>
+      </c>
+      <c r="C21" t="s">
         <v>209</v>
       </c>
-      <c r="B21" t="str">
-        <f t="shared" si="0"/>
-        <v>Cooking Couldron</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>210</v>
       </c>
-      <c r="D21" t="s">
+      <c r="F21" s="2">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2">
+        <v>0</v>
+      </c>
+      <c r="H21" s="2">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2">
+        <v>0</v>
+      </c>
+      <c r="J21" s="2">
+        <v>0</v>
+      </c>
+      <c r="K21" s="2">
+        <v>0</v>
+      </c>
+      <c r="L21" t="s">
+        <v>156</v>
+      </c>
+      <c r="M21" t="s">
         <v>211</v>
-      </c>
-      <c r="F21" s="2">
-        <v>0</v>
-      </c>
-      <c r="G21" s="2">
-        <v>0</v>
-      </c>
-      <c r="H21" s="2">
-        <v>0</v>
-      </c>
-      <c r="I21" s="2">
-        <v>0</v>
-      </c>
-      <c r="J21" s="2">
-        <v>0</v>
-      </c>
-      <c r="K21" s="2">
-        <v>0</v>
-      </c>
-      <c r="L21" t="s">
-        <v>157</v>
-      </c>
-      <c r="M21" t="s">
-        <v>212</v>
       </c>
       <c r="O21">
         <v>2</v>
@@ -6543,10 +6543,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="s">
+        <v>212</v>
+      </c>
+      <c r="T21" t="s">
         <v>213</v>
-      </c>
-      <c r="T21" t="s">
-        <v>214</v>
       </c>
       <c r="U21" t="b">
         <v>1</v>
@@ -6554,14 +6554,14 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>214</v>
+      </c>
+      <c r="B22" t="str">
+        <f t="shared" si="0"/>
+        <v>Small Seating Table</v>
+      </c>
+      <c r="D22" t="s">
         <v>215</v>
-      </c>
-      <c r="B22" t="str">
-        <f t="shared" si="0"/>
-        <v>Small Seating Table</v>
-      </c>
-      <c r="D22" t="s">
-        <v>216</v>
       </c>
       <c r="F22" s="2">
         <v>0</v>
@@ -6582,10 +6582,10 @@
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M22" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="O22">
         <v>2</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="s">
+        <v>216</v>
+      </c>
+      <c r="T22" t="s">
         <v>217</v>
-      </c>
-      <c r="T22" t="s">
-        <v>218</v>
       </c>
       <c r="U22" t="b">
         <v>1</v>
@@ -6605,17 +6605,17 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>218</v>
+      </c>
+      <c r="B23" t="str">
+        <f t="shared" si="0"/>
+        <v>Pass Table</v>
+      </c>
+      <c r="C23" t="s">
         <v>219</v>
       </c>
-      <c r="B23" t="str">
-        <f t="shared" si="0"/>
-        <v>Pass Table</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>220</v>
-      </c>
-      <c r="D23" t="s">
-        <v>221</v>
       </c>
       <c r="F23" s="2">
         <v>0</v>
@@ -6636,10 +6636,10 @@
         <v>1</v>
       </c>
       <c r="L23" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M23" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="O23">
         <v>2</v>
@@ -6648,10 +6648,10 @@
         <v>0</v>
       </c>
       <c r="S23" t="s">
+        <v>221</v>
+      </c>
+      <c r="T23" t="s">
         <v>222</v>
-      </c>
-      <c r="T23" t="s">
-        <v>223</v>
       </c>
       <c r="U23" t="b">
         <v>1</v>
@@ -6659,18 +6659,18 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>223</v>
+      </c>
+      <c r="B24" t="str">
+        <f t="shared" si="0"/>
+        <v>Crate</v>
+      </c>
+      <c r="C24" t="s">
         <v>224</v>
       </c>
-      <c r="B24" t="str">
-        <f t="shared" si="0"/>
-        <v>Crate</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>225</v>
       </c>
-      <c r="D24" t="s">
-        <v>226</v>
-      </c>
       <c r="F24" s="2">
         <v>0</v>
       </c>
@@ -6690,7 +6690,7 @@
         <v>0</v>
       </c>
       <c r="L24" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O24">
         <v>2</v>
@@ -6699,10 +6699,10 @@
         <v>0</v>
       </c>
       <c r="S24" t="s">
+        <v>226</v>
+      </c>
+      <c r="T24" t="s">
         <v>227</v>
-      </c>
-      <c r="T24" t="s">
-        <v>228</v>
       </c>
       <c r="U24" t="b">
         <v>1</v>
@@ -6710,18 +6710,18 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>Barrel</v>
       </c>
       <c r="C25" t="s">
+        <v>224</v>
+      </c>
+      <c r="D25" t="s">
         <v>225</v>
       </c>
-      <c r="D25" t="s">
-        <v>226</v>
-      </c>
       <c r="F25" s="2">
         <v>0</v>
       </c>
@@ -6741,7 +6741,7 @@
         <v>0</v>
       </c>
       <c r="L25" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O25">
         <v>2</v>
@@ -6750,10 +6750,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="s">
+        <v>229</v>
+      </c>
+      <c r="T25" t="s">
         <v>230</v>
-      </c>
-      <c r="T25" t="s">
-        <v>231</v>
       </c>
       <c r="U25" t="b">
         <v>1</v>
@@ -6761,38 +6761,38 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>231</v>
+      </c>
+      <c r="B26" t="str">
+        <f t="shared" si="0"/>
+        <v>Wall Torch</v>
+      </c>
+      <c r="C26" t="s">
         <v>232</v>
       </c>
-      <c r="B26" t="str">
-        <f t="shared" si="0"/>
-        <v>Wall Torch</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>233</v>
       </c>
-      <c r="D26" t="s">
+      <c r="F26" s="2">
+        <v>0</v>
+      </c>
+      <c r="G26" s="2">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2">
+        <v>0</v>
+      </c>
+      <c r="I26" s="2">
+        <v>0</v>
+      </c>
+      <c r="J26" s="2">
+        <v>0</v>
+      </c>
+      <c r="K26" s="2">
+        <v>0</v>
+      </c>
+      <c r="L26" t="s">
         <v>234</v>
-      </c>
-      <c r="F26" s="2">
-        <v>0</v>
-      </c>
-      <c r="G26" s="2">
-        <v>0</v>
-      </c>
-      <c r="H26" s="2">
-        <v>0</v>
-      </c>
-      <c r="I26" s="2">
-        <v>0</v>
-      </c>
-      <c r="J26" s="2">
-        <v>0</v>
-      </c>
-      <c r="K26" s="2">
-        <v>0</v>
-      </c>
-      <c r="L26" t="s">
-        <v>235</v>
       </c>
       <c r="O26">
         <v>0</v>
@@ -6804,10 +6804,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="s">
+        <v>235</v>
+      </c>
+      <c r="T26" t="s">
         <v>236</v>
-      </c>
-      <c r="T26" t="s">
-        <v>237</v>
       </c>
       <c r="U26" t="b">
         <v>1</v>
@@ -6815,17 +6815,17 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>237</v>
+      </c>
+      <c r="B27" t="str">
+        <f t="shared" si="0"/>
+        <v>Condiment Shelf</v>
+      </c>
+      <c r="C27" t="s">
         <v>238</v>
       </c>
-      <c r="B27" t="str">
-        <f t="shared" si="0"/>
-        <v>Condiment Shelf</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>239</v>
-      </c>
-      <c r="D27" t="s">
-        <v>240</v>
       </c>
       <c r="F27" s="2">
         <v>0</v>
@@ -6846,10 +6846,10 @@
         <v>2</v>
       </c>
       <c r="L27" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M27" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="O27">
         <v>1</v>
@@ -6861,10 +6861,10 @@
         <v>0</v>
       </c>
       <c r="S27" t="s">
+        <v>240</v>
+      </c>
+      <c r="T27" t="s">
         <v>241</v>
-      </c>
-      <c r="T27" t="s">
-        <v>242</v>
       </c>
       <c r="U27" t="b">
         <v>1</v>
@@ -6872,17 +6872,17 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>Condiment Shelf Small</v>
       </c>
       <c r="C28" t="s">
+        <v>238</v>
+      </c>
+      <c r="D28" t="s">
         <v>239</v>
-      </c>
-      <c r="D28" t="s">
-        <v>240</v>
       </c>
       <c r="F28" s="2">
         <v>0</v>
@@ -6903,10 +6903,10 @@
         <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M28" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="O28">
         <v>1</v>
@@ -6918,10 +6918,10 @@
         <v>0</v>
       </c>
       <c r="S28" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="T28" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="U28" t="b">
         <v>1</v>
@@ -6929,18 +6929,18 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>Hanging Frying Pans</v>
       </c>
       <c r="C29" t="s">
+        <v>238</v>
+      </c>
+      <c r="D29" t="s">
         <v>239</v>
       </c>
-      <c r="D29" t="s">
-        <v>240</v>
-      </c>
       <c r="F29" s="2">
         <v>0</v>
       </c>
@@ -6960,10 +6960,10 @@
         <v>0</v>
       </c>
       <c r="L29" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="M29" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="O29">
         <v>0</v>
@@ -6974,14 +6974,14 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>245</v>
+      </c>
+      <c r="B30" t="str">
+        <f t="shared" si="0"/>
+        <v>Butcher Table</v>
+      </c>
+      <c r="D30" t="s">
         <v>246</v>
-      </c>
-      <c r="B30" t="str">
-        <f t="shared" si="0"/>
-        <v>Butcher Table</v>
-      </c>
-      <c r="D30" t="s">
-        <v>247</v>
       </c>
       <c r="F30" s="2">
         <v>0</v>
@@ -7002,10 +7002,10 @@
         <v>3</v>
       </c>
       <c r="L30" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M30" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="O30">
         <v>2</v>
@@ -7016,14 +7016,14 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>Hanging Meat</v>
       </c>
       <c r="D31" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -7206,10 +7206,10 @@
   <sheetData>
     <row r="2" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>249</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>250</v>
       </c>
       <c r="C2" t="s">
         <v>28</v>
@@ -7242,343 +7242,343 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B1" t="s">
         <v>251</v>
       </c>
-      <c r="B1" t="s">
-        <v>252</v>
-      </c>
       <c r="C1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>16</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>19</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>20</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>0</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B26" s="12" t="s">
         <v>43</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B27" s="12" t="s">
         <v>44</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>45</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B29" s="12" t="s">
         <v>46</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B30" s="12" t="s">
         <v>47</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>20</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -7589,7 +7589,7 @@
         <v>0</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -7600,7 +7600,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -7611,95 +7611,95 @@
         <v>42</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B35" s="15" t="s">
         <v>0</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>1</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B37" s="15" t="s">
         <v>71</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>42</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B39" s="15" t="s">
         <v>3</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>4</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="15" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B41" s="15" t="s">
         <v>5</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>21</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -7710,7 +7710,7 @@
         <v>0</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -7721,7 +7721,7 @@
         <v>1</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -7732,7 +7732,7 @@
         <v>42</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update orb mechanics and documentation for Runic orb integration
- Introduced the Runic orb, which features a homing mechanic to seek and collect floor glyphs, enhancing gameplay strategy.
- Updated `DECISIONS.md` to reflect the addition of the Runic orb and its unique mechanics, including its interaction with other orbs and gameplay strategies.
- Revised `GAME_BRIEF.md` and `PROJECT_MAP.md` to include details about the Runic orb's abilities and its integration into the game.
- Adjusted `game_data.json` to ensure accurate descriptions and functionality for the new Runic orb and its associated effects.
- Enhanced the starting orb selection to include the Runic orb, providing players with more variety at the beginning of gameplay.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1444AE99-37BD-45D7-B4F3-31AF6E1E89DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80951A2B-1C11-435D-9992-BB287CB52316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2063,7 +2063,7 @@
         <v>2</v>
       </c>
       <c r="N8">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="O8">
         <v>3</v>
@@ -2072,7 +2072,7 @@
         <v>0.05</v>
       </c>
       <c r="Q8" s="8">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="R8">
         <v>3</v>

</xml_diff>

<commit_message>
Refactor summoning circle mechanics and enhance input prompts for improved gameplay interaction
- Updated the summoning circle to support real-time orb capture and interactions without pausing the game, enhancing co-op gameplay fluidity.
- Introduced a new `InputPrompt` system for displaying contextual actions (buy, activate, cancel) based on player proximity and input device.
- Revised `DECISIONS.md` to document changes in orb activation, upgrade, and ritual cancel mechanics, including proximity-based interactions and input prompts.
- Enhanced `GAME_BRIEF.md` and `PROJECT_MAP.md` to reflect the new input handling and summoning circle mechanics.
- Improved player controls for clearer input handling related to summoning circle actions, ensuring a smoother gameplay experience.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80951A2B-1C11-435D-9992-BB287CB52316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D750112-C045-4D11-A68F-ABC6BCAA90AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="315">
   <si>
     <t>id</t>
   </si>
@@ -968,6 +968,27 @@
   </si>
   <si>
     <t>Seeks out and picks up glyphs and drops them near the summoning circle.</t>
+  </si>
+  <si>
+    <t>charge</t>
+  </si>
+  <si>
+    <t>Absorbs Shock from enemies. When hitting 20, the next impact creates a powerful thunder strike doing 60 AoE damage</t>
+  </si>
+  <si>
+    <t>recharge</t>
+  </si>
+  <si>
+    <t>The thunder strike applies 5 Shock</t>
+  </si>
+  <si>
+    <t>Gains 1 Shock every 2 seconds</t>
+  </si>
+  <si>
+    <t>Absorbs Shock from enemies without removing it</t>
+  </si>
+  <si>
+    <t>On redirect, lower the cooldown of the next frost nova by 0.2 seconds</t>
   </si>
 </sst>
 </file>
@@ -2498,17 +2519,32 @@
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>308</v>
+      </c>
       <c r="B19" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Charge</v>
+      </c>
+      <c r="C19" t="s">
+        <v>309</v>
+      </c>
+      <c r="D19" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" t="s">
+        <v>27</v>
       </c>
       <c r="G19" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Air|Air|Air</v>
       </c>
       <c r="H19" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Yes</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -4081,7 +4117,7 @@
         <v>72</v>
       </c>
       <c r="B2" t="str">
-        <f t="shared" ref="B2:B26" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
+        <f t="shared" ref="B2:B27" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Haunt</v>
       </c>
       <c r="C2" t="s">
@@ -4744,29 +4780,102 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
+      <c r="I26" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>310</v>
+      </c>
+      <c r="B27" t="str">
+        <f t="shared" si="0"/>
+        <v>Recharge</v>
+      </c>
+      <c r="C27" t="s">
+        <v>308</v>
+      </c>
+      <c r="D27" t="s">
+        <v>312</v>
+      </c>
+      <c r="E27" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27" t="s">
+        <v>27</v>
+      </c>
+      <c r="G27" t="s">
+        <v>27</v>
+      </c>
       <c r="H27" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Air|Air|Air</v>
+      </c>
+      <c r="I27" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>308</v>
+      </c>
+      <c r="D28" t="s">
+        <v>311</v>
+      </c>
+      <c r="E28" t="s">
+        <v>27</v>
+      </c>
+      <c r="F28" t="s">
+        <v>28</v>
+      </c>
+      <c r="G28" t="s">
+        <v>28</v>
+      </c>
       <c r="H28" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Air|Fire|Fire</v>
+      </c>
+      <c r="I28" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>308</v>
+      </c>
+      <c r="D29" t="s">
+        <v>313</v>
+      </c>
+      <c r="E29" t="s">
+        <v>27</v>
+      </c>
+      <c r="F29" t="s">
+        <v>34</v>
+      </c>
+      <c r="G29" t="s">
+        <v>34</v>
+      </c>
       <c r="H29" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Air|Water|Water</v>
+      </c>
+      <c r="I29" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>291</v>
+      </c>
+      <c r="D30" t="s">
+        <v>314</v>
+      </c>
       <c r="H30" t="str">
         <f t="shared" si="1"/>
         <v/>
+      </c>
+      <c r="I30" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update game data and summoning circle configuration for improved gameplay clarity
- Refactored `game_data.json` to enhance the organization of attributes and attunements, ensuring clearer descriptions and functionality.
- Updated the `summoning_circle.tscn` to streamline visibility settings for UI elements, improving player interaction and feedback during gameplay.
- Adjusted the `game_data.xlsx` to reflect changes in the JSON structure, ensuring consistency across data formats.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D750112-C045-4D11-A68F-ABC6BCAA90AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783630E1-3B5B-4666-84FC-658E2BF5C8FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="315">
   <si>
     <t>id</t>
   </si>
@@ -1999,6 +1999,9 @@
         <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
+      <c r="I7" t="s">
+        <v>24</v>
+      </c>
       <c r="J7">
         <v>10</v>
       </c>
@@ -2398,6 +2401,10 @@
         <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
+      <c r="V14" t="str">
+        <f t="shared" ref="V14:V18" si="5">"res://entities/orbs/blank/"&amp;A14&amp;"_orb.tscn"</f>
+        <v>res://entities/orbs/blank/_orb.tscn</v>
+      </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -2427,6 +2434,10 @@
         <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
+      <c r="V15" t="str">
+        <f t="shared" si="5"/>
+        <v>res://entities/orbs/blank/hunger_orb.tscn</v>
+      </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -2459,8 +2470,12 @@
       <c r="I16" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="V16" t="str">
+        <f t="shared" si="5"/>
+        <v>res://entities/orbs/blank/vengance_orb.tscn</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>265</v>
       </c>
@@ -2488,8 +2503,12 @@
         <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="V17" t="str">
+        <f t="shared" si="5"/>
+        <v>res://entities/orbs/blank/hunter_orb.tscn</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>291</v>
       </c>
@@ -2517,8 +2536,54 @@
         <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I18" t="s">
+        <v>24</v>
+      </c>
+      <c r="J18">
+        <v>10</v>
+      </c>
+      <c r="K18">
+        <v>12</v>
+      </c>
+      <c r="L18" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="M18" s="8">
+        <v>2</v>
+      </c>
+      <c r="N18">
+        <v>105</v>
+      </c>
+      <c r="O18">
+        <v>8</v>
+      </c>
+      <c r="P18" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="Q18" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <v>3</v>
+      </c>
+      <c r="T18">
+        <v>0</v>
+      </c>
+      <c r="U18">
+        <v>0</v>
+      </c>
+      <c r="V18" t="str">
+        <f t="shared" si="5"/>
+        <v>res://entities/orbs/blank/nova_orb.tscn</v>
+      </c>
+      <c r="W18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>308</v>
       </c>
@@ -2547,7 +2612,7 @@
         <v>Yes</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B20" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2561,7 +2626,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B21" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2575,7 +2640,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B22" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2589,7 +2654,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B23" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2603,7 +2668,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B24" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2617,7 +2682,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B25" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2631,7 +2696,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B26" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2645,7 +2710,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B27" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2659,7 +2724,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B28" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2673,7 +2738,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B29" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2687,7 +2752,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B30" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2701,7 +2766,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B31" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2715,7 +2780,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B32" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -2753,7 +2818,7 @@
         <v/>
       </c>
       <c r="H34" t="str">
-        <f t="shared" ref="H34:H65" si="5">IF(ISBLANK(F34),"",IF(COUNTIF($G$2:$G$101,G34)=1,"Yes","No"))</f>
+        <f t="shared" ref="H34:H65" si="6">IF(ISBLANK(F34),"",IF(COUNTIF($G$2:$G$101,G34)=1,"Yes","No"))</f>
         <v/>
       </c>
     </row>
@@ -2763,11 +2828,11 @@
         <v/>
       </c>
       <c r="G35" t="str">
-        <f t="shared" ref="G35:G66" si="6">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(D35:F35))</f>
+        <f t="shared" ref="G35:G66" si="7">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(D35:F35))</f>
         <v/>
       </c>
       <c r="H35" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
@@ -2777,11 +2842,11 @@
         <v/>
       </c>
       <c r="G36" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H36" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H36" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2791,11 +2856,11 @@
         <v/>
       </c>
       <c r="G37" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H37" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H37" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2805,11 +2870,11 @@
         <v/>
       </c>
       <c r="G38" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H38" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H38" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2819,11 +2884,11 @@
         <v/>
       </c>
       <c r="G39" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H39" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H39" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2833,11 +2898,11 @@
         <v/>
       </c>
       <c r="G40" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H40" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H40" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2847,11 +2912,11 @@
         <v/>
       </c>
       <c r="G41" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H41" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H41" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2861,11 +2926,11 @@
         <v/>
       </c>
       <c r="G42" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H42" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H42" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2875,11 +2940,11 @@
         <v/>
       </c>
       <c r="G43" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H43" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H43" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -2889,551 +2954,551 @@
         <v/>
       </c>
       <c r="G44" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H44" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H44" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G45" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H45" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H45" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G46" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H46" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H46" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G47" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H47" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H47" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="G48" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H48" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H48" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="49" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G49" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H49" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H49" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="50" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G50" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H50" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H50" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="51" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G51" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H51" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H51" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="52" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G52" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H52" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H52" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="53" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G53" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H53" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H53" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="54" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G54" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H54" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H54" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="55" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G55" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H55" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H55" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="56" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G56" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H56" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H56" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="57" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G57" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H57" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H57" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="58" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G58" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H58" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H58" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="59" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G59" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H59" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H59" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="60" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G60" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H60" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H60" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="61" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G61" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H61" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H61" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="62" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G62" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H62" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H62" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="63" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G63" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H63" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H63" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="64" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G64" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H64" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H64" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="65" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G65" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="H65" t="str">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H65" t="str">
-        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="66" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G66" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="H66" t="str">
-        <f t="shared" ref="H66:H97" si="7">IF(ISBLANK(F66),"",IF(COUNTIF($G$2:$G$101,G66)=1,"Yes","No"))</f>
+        <f t="shared" ref="H66:H97" si="8">IF(ISBLANK(F66),"",IF(COUNTIF($G$2:$G$101,G66)=1,"Yes","No"))</f>
         <v/>
       </c>
     </row>
     <row r="67" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G67" t="str">
-        <f t="shared" ref="G67:G98" si="8">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(D67:F67))</f>
+        <f t="shared" ref="G67:G98" si="9">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(D67:F67))</f>
         <v/>
       </c>
       <c r="H67" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="68" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G68" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H68" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H68" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="69" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G69" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H69" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H69" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="70" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G70" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H70" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H70" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="71" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G71" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H71" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H71" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="72" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G72" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H72" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H72" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="73" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G73" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H73" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H73" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="74" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G74" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H74" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H74" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="75" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G75" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H75" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H75" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="76" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G76" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H76" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H76" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="77" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G77" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H77" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H77" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="78" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G78" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H78" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H78" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="79" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G79" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H79" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H79" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="80" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G80" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H80" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H80" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="81" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G81" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H81" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H81" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="82" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G82" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H82" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H82" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="83" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G83" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H83" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H83" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="84" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G84" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H84" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H84" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="85" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G85" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H85" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H85" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="86" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G86" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H86" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H86" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="87" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G87" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H87" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H87" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="88" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G88" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H88" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H88" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="89" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G89" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H89" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H89" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="90" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G90" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H90" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H90" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="91" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G91" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H91" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H91" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="92" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G92" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H92" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H92" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="93" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G93" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H93" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H93" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="94" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G94" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H94" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H94" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="95" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G95" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H95" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H95" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="96" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G96" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H96" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H96" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="97" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G97" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="H97" t="str">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="H97" t="str">
-        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="98" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G98" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="H98" t="str">
-        <f t="shared" ref="H98" si="9">IF(ISBLANK(F98),"",IF(COUNTIF($G$2:$G$101,G98)=1,"Yes","No"))</f>
+        <f t="shared" ref="H98" si="10">IF(ISBLANK(F98),"",IF(COUNTIF($G$2:$G$101,G98)=1,"Yes","No"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement Nova orb mechanics and update related documentation
- Introduced the Nova orb, which pulses a frost nova every 3 seconds, applying Chill to nearby enemies while flying. This enhances gameplay strategy by providing area control without direct damage.
- Updated `DECISIONS.md` to document the Nova orb's mechanics, including its interaction with Chill stacks and visual effects.
- Revised `GAME_BRIEF.md` to include details about the Nova orb's abilities and its integration into the game.
- Enhanced `PROJECT_MAP.md` to reflect the addition of the Nova orb and its associated assets.
- Adjusted `game_data.json` to ensure accurate descriptions and functionality for the new Nova orb and its effects.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783630E1-3B5B-4666-84FC-658E2BF5C8FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5022CBD-B7B4-497E-99E9-12F798A51626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="38730" windowHeight="21210" tabRatio="696" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
     <sheet name="glyphs" sheetId="2" r:id="rId2"/>
     <sheet name="attribute" sheetId="8" r:id="rId3"/>
     <sheet name="attunements" sheetId="3" r:id="rId4"/>
-    <sheet name="motion" sheetId="4" r:id="rId5"/>
-    <sheet name="objects_OLD" sheetId="5" state="hidden" r:id="rId6"/>
-    <sheet name="input" sheetId="6" r:id="rId7"/>
-    <sheet name="schema" sheetId="7" r:id="rId8"/>
+    <sheet name="relics" sheetId="9" r:id="rId5"/>
+    <sheet name="motion" sheetId="4" r:id="rId6"/>
+    <sheet name="objects_OLD" sheetId="5" state="hidden" r:id="rId7"/>
+    <sheet name="input" sheetId="6" r:id="rId8"/>
+    <sheet name="schema" sheetId="7" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">objects_OLD!$A$1:$U$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">objects_OLD!$A$1:$U$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">orbs!$A$1:$W$44</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="341">
   <si>
     <t>id</t>
   </si>
@@ -989,6 +990,84 @@
   </si>
   <si>
     <t>On redirect, lower the cooldown of the next frost nova by 0.2 seconds</t>
+  </si>
+  <si>
+    <t>Each time 3 or more stacks of Frost is inflicted, inflict 1 burn</t>
+  </si>
+  <si>
+    <t>Once every 20 seconds when the orb would hit the player, redirect Orb instead</t>
+  </si>
+  <si>
+    <t>Activating the summoning circle costs 50% less</t>
+  </si>
+  <si>
+    <t>Crystals deposited while the circle is active refund 1 mana</t>
+  </si>
+  <si>
+    <t>Each time Shock triggers, trigger Poison</t>
+  </si>
+  <si>
+    <t>An image of you is left behind after dashing, attracting enemies. Image last for 3 seconds and have 1 hp</t>
+  </si>
+  <si>
+    <t>When two orb meet a explosion is created inflicting 10 Burn</t>
+  </si>
+  <si>
+    <t>Dashing through an enemy deals 10 damage</t>
+  </si>
+  <si>
+    <t>Thrown crystals stun 0.5 seconds on hit</t>
+  </si>
+  <si>
+    <t>Breakables have a +10% chance of dropping glyphs</t>
+  </si>
+  <si>
+    <t>While carrying a glyph, take 20% less damage</t>
+  </si>
+  <si>
+    <t>After redirecting, players becomes immune to all damage for 0.3 second</t>
+  </si>
+  <si>
+    <t>When 1 stack of a basic status afflicts an enemy, add 1 stack of another random one</t>
+  </si>
+  <si>
+    <t>Trigger enemies burn on impact</t>
+  </si>
+  <si>
+    <t>friction</t>
+  </si>
+  <si>
+    <t>prio</t>
+  </si>
+  <si>
+    <t>Circle activation also damages all nearby enemies</t>
+  </si>
+  <si>
+    <t>Tithe</t>
+  </si>
+  <si>
+    <t>tithe</t>
+  </si>
+  <si>
+    <t>Standing in the summoning circle slowly heals</t>
+  </si>
+  <si>
+    <t>groove</t>
+  </si>
+  <si>
+    <t>Bonus 10% bonus damage to chilled enemies</t>
+  </si>
+  <si>
+    <t>boil</t>
+  </si>
+  <si>
+    <t>Glyphs have double HP</t>
+  </si>
+  <si>
+    <t>sturdy</t>
+  </si>
+  <si>
+    <t>All AOE effects are 20% larger</t>
   </si>
 </sst>
 </file>
@@ -1106,7 +1185,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1126,6 +1205,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1239,6 +1319,11 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFB17ED8"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -5451,9 +5536,192 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F642FAC-7326-47E8-9F14-D9D50EC3456E}">
+  <sheetPr>
+    <tabColor theme="4" tint="0.59999389629810485"/>
+  </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="94.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="95.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>329</v>
+      </c>
+      <c r="C11" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>322</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>323</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>324</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>325</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>323</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>333</v>
+      </c>
+      <c r="B18" t="s">
+        <v>332</v>
+      </c>
+      <c r="C18" t="s">
+        <v>331</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>335</v>
+      </c>
+      <c r="C19" t="s">
+        <v>334</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>337</v>
+      </c>
+      <c r="C20" t="s">
+        <v>336</v>
+      </c>
+      <c r="F20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>339</v>
+      </c>
+      <c r="C21" t="s">
+        <v>338</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>340</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
-    <tabColor theme="4" tint="0.59999389629810485"/>
+    <tabColor rgb="FFB17ED8"/>
   </sheetPr>
   <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5683,7 +5951,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor theme="8" tint="0.59999389629810485"/>
@@ -7367,7 +7635,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
@@ -7403,7 +7671,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>

</xml_diff>

<commit_message>
Update desert scene and summoning circle mechanics
- Added a new PhysicsMaterial to the desert scene for enhanced interaction dynamics.
- Removed an obsolete PhysicsMaterial from the desert scene to streamline material management.
- Updated the summoning circle scene to include new rite textures and labels, enhancing visual feedback for players.
- Introduced a new RiteInfo node to display rite details, improving user interface clarity during gameplay.
- Adjusted visibility settings for various nodes to optimize UI presentation during rituals.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5022CBD-B7B4-497E-99E9-12F798A51626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B608D2-9E3C-48A3-B49F-FD85E40CB19F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-165" yWindow="-165" windowWidth="38730" windowHeight="21210" tabRatio="696" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
     <sheet name="glyphs" sheetId="2" r:id="rId2"/>
     <sheet name="attribute" sheetId="8" r:id="rId3"/>
     <sheet name="attunements" sheetId="3" r:id="rId4"/>
-    <sheet name="relics" sheetId="9" r:id="rId5"/>
+    <sheet name="rites" sheetId="9" r:id="rId5"/>
     <sheet name="motion" sheetId="4" r:id="rId6"/>
     <sheet name="objects_OLD" sheetId="5" state="hidden" r:id="rId7"/>
     <sheet name="input" sheetId="6" r:id="rId8"/>
@@ -26,6 +26,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">objects_OLD!$A$1:$U$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">orbs!$A$1:$W$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">rites!$A$1:$G$19</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="437">
   <si>
     <t>id</t>
   </si>
@@ -995,57 +996,30 @@
     <t>Each time 3 or more stacks of Frost is inflicted, inflict 1 burn</t>
   </si>
   <si>
-    <t>Once every 20 seconds when the orb would hit the player, redirect Orb instead</t>
-  </si>
-  <si>
     <t>Activating the summoning circle costs 50% less</t>
   </si>
   <si>
-    <t>Crystals deposited while the circle is active refund 1 mana</t>
-  </si>
-  <si>
-    <t>Each time Shock triggers, trigger Poison</t>
-  </si>
-  <si>
     <t>An image of you is left behind after dashing, attracting enemies. Image last for 3 seconds and have 1 hp</t>
   </si>
   <si>
-    <t>When two orb meet a explosion is created inflicting 10 Burn</t>
-  </si>
-  <si>
     <t>Dashing through an enemy deals 10 damage</t>
   </si>
   <si>
-    <t>Thrown crystals stun 0.5 seconds on hit</t>
-  </si>
-  <si>
     <t>Breakables have a +10% chance of dropping glyphs</t>
   </si>
   <si>
-    <t>While carrying a glyph, take 20% less damage</t>
-  </si>
-  <si>
     <t>After redirecting, players becomes immune to all damage for 0.3 second</t>
   </si>
   <si>
     <t>When 1 stack of a basic status afflicts an enemy, add 1 stack of another random one</t>
   </si>
   <si>
-    <t>Trigger enemies burn on impact</t>
-  </si>
-  <si>
-    <t>friction</t>
-  </si>
-  <si>
     <t>prio</t>
   </si>
   <si>
     <t>Circle activation also damages all nearby enemies</t>
   </si>
   <si>
-    <t>Tithe</t>
-  </si>
-  <si>
     <t>tithe</t>
   </si>
   <si>
@@ -1055,19 +1029,334 @@
     <t>groove</t>
   </si>
   <si>
-    <t>Bonus 10% bonus damage to chilled enemies</t>
-  </si>
-  <si>
     <t>boil</t>
   </si>
   <si>
     <t>Glyphs have double HP</t>
   </si>
   <si>
-    <t>sturdy</t>
-  </si>
-  <si>
     <t>All AOE effects are 20% larger</t>
+  </si>
+  <si>
+    <t>frostburn</t>
+  </si>
+  <si>
+    <t>Once every 20 seconds, block self-damage</t>
+  </si>
+  <si>
+    <t>efficiancy</t>
+  </si>
+  <si>
+    <t>accelerant</t>
+  </si>
+  <si>
+    <t>png_path</t>
+  </si>
+  <si>
+    <t>10% bonus damage to enemies with Chill</t>
+  </si>
+  <si>
+    <t>When two orbs meet an explosion is created inflicting 10 damage</t>
+  </si>
+  <si>
+    <t>While carrying a glyph, take 25% less damage</t>
+  </si>
+  <si>
+    <t>rites</t>
+  </si>
+  <si>
+    <t>ward</t>
+  </si>
+  <si>
+    <t>rebate</t>
+  </si>
+  <si>
+    <t>Glyphs deposited while the circle is active refund +1 mana</t>
+  </si>
+  <si>
+    <t>grace</t>
+  </si>
+  <si>
+    <t>flux</t>
+  </si>
+  <si>
+    <t>clash</t>
+  </si>
+  <si>
+    <t>skewer</t>
+  </si>
+  <si>
+    <t>concuss</t>
+  </si>
+  <si>
+    <t>salvage</t>
+  </si>
+  <si>
+    <t>ballast</t>
+  </si>
+  <si>
+    <t>swell</t>
+  </si>
+  <si>
+    <t>tempered</t>
+  </si>
+  <si>
+    <t>tag</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>ember</t>
+  </si>
+  <si>
+    <t>Enemies that die with 10 or more burn explode for 10 damage</t>
+  </si>
+  <si>
+    <t>smolder</t>
+  </si>
+  <si>
+    <t>Burn stacks never decay below 1</t>
+  </si>
+  <si>
+    <t>Redirects stop raising self-damage. Speed and enemy damage still rise.</t>
+  </si>
+  <si>
+    <t>mercy</t>
+  </si>
+  <si>
+    <t>Each redirect also adds 1 weight.</t>
+  </si>
+  <si>
+    <t>heft</t>
+  </si>
+  <si>
+    <t>The first orb hit after redirect deals +25% damage</t>
+  </si>
+  <si>
+    <t>followthrough</t>
+  </si>
+  <si>
+    <t>martyr</t>
+  </si>
+  <si>
+    <t>Orbs cannot drop you below 1 HP</t>
+  </si>
+  <si>
+    <t>penance</t>
+  </si>
+  <si>
+    <t>Self-damage taken is added to the mana pool, 1 mana per 3 HP</t>
+  </si>
+  <si>
+    <t>surrogate</t>
+  </si>
+  <si>
+    <t>While you carry a glyph, orb contact damages that glyph instead of you.</t>
+  </si>
+  <si>
+    <t>glass</t>
+  </si>
+  <si>
+    <t>Damage and self-damage is dealt is 30% higher for all orbs</t>
+  </si>
+  <si>
+    <t>payback</t>
+  </si>
+  <si>
+    <t>For 3s after an orb hits you, that orb deals +20% damage to enemies</t>
+  </si>
+  <si>
+    <t>reduce</t>
+  </si>
+  <si>
+    <t>All damage to you is reduced by 1</t>
+  </si>
+  <si>
+    <t>surplus</t>
+  </si>
+  <si>
+    <t>Mana left at level clear carries into the next level.</t>
+  </si>
+  <si>
+    <t>refund</t>
+  </si>
+  <si>
+    <t>Disarming a waiting circle refunds what you paid to arm it.</t>
+  </si>
+  <si>
+    <t>subsidy</t>
+  </si>
+  <si>
+    <t>Blank Orbs cost half the price</t>
+  </si>
+  <si>
+    <t>swarm</t>
+  </si>
+  <si>
+    <t>Increase orb cap to 6</t>
+  </si>
+  <si>
+    <t>An orb that destroys a glyph adds half that glyph's deposit value as mana.</t>
+  </si>
+  <si>
+    <t>premium</t>
+  </si>
+  <si>
+    <t>Unique glyphs deposit 30 mana.</t>
+  </si>
+  <si>
+    <t>While the circle is waiting for an orb, enemies inside its info radius move 20% slower.</t>
+  </si>
+  <si>
+    <t>vigil</t>
+  </si>
+  <si>
+    <t>keeper</t>
+  </si>
+  <si>
+    <t>Transforming gives you one new socketed at random.</t>
+  </si>
+  <si>
+    <t>circle &amp; mana</t>
+  </si>
+  <si>
+    <t>self damage</t>
+  </si>
+  <si>
+    <t>redirect</t>
+  </si>
+  <si>
+    <t>Carrying a glyph does not block dash.</t>
+  </si>
+  <si>
+    <t>unburden</t>
+  </si>
+  <si>
+    <t>courier</t>
+  </si>
+  <si>
+    <t>Thrown glyphs travel 100% farther.</t>
+  </si>
+  <si>
+    <t>The first glyph each level is at least Rare.</t>
+  </si>
+  <si>
+    <t>Glyphs have -50% HP. Deposit mana is +50%.</t>
+  </si>
+  <si>
+    <t>imbue</t>
+  </si>
+  <si>
+    <t>Depositing a Unique glyph also bakes its attribute onto a random live orb for the rest of the level.</t>
+  </si>
+  <si>
+    <t>brittle</t>
+  </si>
+  <si>
+    <t>auspice</t>
+  </si>
+  <si>
+    <t>sepsis</t>
+  </si>
+  <si>
+    <t>Blight also raises Burn tick damage</t>
+  </si>
+  <si>
+    <t>glacier</t>
+  </si>
+  <si>
+    <t>Chill stacks past 15 deal 1 each when applied</t>
+  </si>
+  <si>
+    <t>hairpin</t>
+  </si>
+  <si>
+    <t>Shock triggers at 8 stacks</t>
+  </si>
+  <si>
+    <t>leftover</t>
+  </si>
+  <si>
+    <t>A Shock trigger leaves 3 stacks instead of clearing it to 0</t>
+  </si>
+  <si>
+    <t>Shock stun lasts 3s</t>
+  </si>
+  <si>
+    <t>daze</t>
+  </si>
+  <si>
+    <t>Bowling can chain: an enemy slammed into a second enemy can slam that one into a third, once.</t>
+  </si>
+  <si>
+    <t>wide</t>
+  </si>
+  <si>
+    <t>sickly</t>
+  </si>
+  <si>
+    <t>Double crit chance on enemies afflicted with +5 Blight</t>
+  </si>
+  <si>
+    <t>One enemy in each wave starts with 5 Chill</t>
+  </si>
+  <si>
+    <t>enemy_wave, chill</t>
+  </si>
+  <si>
+    <t>knockback, weight</t>
+  </si>
+  <si>
+    <t>crit_chance, blight</t>
+  </si>
+  <si>
+    <t>blight, burn</t>
+  </si>
+  <si>
+    <t>glyph</t>
+  </si>
+  <si>
+    <t>Two nearby glyphs have a small chance of merging into one of a higher rarity</t>
+  </si>
+  <si>
+    <t>fuse</t>
+  </si>
+  <si>
+    <t>Destroying every breakable in the level deals 200 damage to all enemies</t>
+  </si>
+  <si>
+    <t>clearcut</t>
+  </si>
+  <si>
+    <t>aoe</t>
+  </si>
+  <si>
+    <t>burn, chill</t>
+  </si>
+  <si>
+    <t>self-damage</t>
+  </si>
+  <si>
+    <t>summoning_circle</t>
+  </si>
+  <si>
+    <t>Each time Shock triggers, trigger Burn twice</t>
+  </si>
+  <si>
+    <t>shock, burn</t>
+  </si>
+  <si>
+    <t>breakable</t>
+  </si>
+  <si>
+    <t>dash</t>
+  </si>
+  <si>
+    <t>clyph</t>
+  </si>
+  <si>
+    <t>Thrown glyphs stun 0.5 seconds on hit</t>
   </si>
 </sst>
 </file>
@@ -1113,7 +1402,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1162,6 +1451,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB17ED8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1205,7 +1500,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5035,6 +5330,9 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D32" t="s">
+        <v>317</v>
+      </c>
       <c r="H32" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -5540,15 +5838,18 @@
   <sheetPr>
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
     <col min="3" max="3" width="94.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="95.85546875" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="5" max="5" width="37.42578125" customWidth="1"/>
+    <col min="13" max="13" width="95.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -5558,162 +5859,972 @@
       <c r="C1" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="13" t="s">
-        <v>20</v>
+      <c r="D1" s="4" t="s">
+        <v>351</v>
       </c>
       <c r="E1" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="G1" s="3" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B2" t="str">
+        <f t="shared" ref="B2:B53" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
+        <v>Frostburn</v>
+      </c>
       <c r="C2" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>428</v>
+      </c>
+      <c r="E2" t="str">
+        <f>"res://ui/rites/"&amp;A2&amp;".png"</f>
+        <v>res://ui/rites/frostburn.png</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>339</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" si="0"/>
+        <v>Ward</v>
+      </c>
       <c r="C3" t="s">
+        <v>331</v>
+      </c>
+      <c r="D3" t="s">
+        <v>429</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E19" si="1">"res://ui/rites/"&amp;A3&amp;".png"</f>
+        <v>res://ui/rites/ward.png</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>332</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>Efficiancy</v>
+      </c>
+      <c r="C4" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C4" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/efficiancy.png</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>340</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Rebate</v>
+      </c>
       <c r="C5" t="s">
+        <v>341</v>
+      </c>
+      <c r="D5" t="s">
+        <v>422</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/rebate.png</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>342</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>Grace</v>
+      </c>
+      <c r="C6" t="s">
+        <v>320</v>
+      </c>
+      <c r="D6" t="s">
+        <v>392</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/grace.png</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>343</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>Flux</v>
+      </c>
+      <c r="C7" t="s">
+        <v>321</v>
+      </c>
+      <c r="D7" t="s">
+        <v>352</v>
+      </c>
+      <c r="E7" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/flux.png</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>333</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>Accelerant</v>
+      </c>
+      <c r="C8" t="s">
+        <v>431</v>
+      </c>
+      <c r="D8" t="s">
+        <v>432</v>
+      </c>
+      <c r="E8" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/accelerant.png</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>344</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>Clash</v>
+      </c>
+      <c r="C9" t="s">
+        <v>336</v>
+      </c>
+      <c r="D9" t="s">
+        <v>248</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/clash.png</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>345</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>Skewer</v>
+      </c>
+      <c r="C10" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C6" t="s">
+      <c r="D10" t="s">
+        <v>434</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/skewer.png</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>346</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>Concuss</v>
+      </c>
+      <c r="C11" t="s">
+        <v>436</v>
+      </c>
+      <c r="D11" t="s">
+        <v>435</v>
+      </c>
+      <c r="E11" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/concuss.png</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>347</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>Salvage</v>
+      </c>
+      <c r="C12" t="s">
+        <v>319</v>
+      </c>
+      <c r="D12" t="s">
+        <v>433</v>
+      </c>
+      <c r="E12" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/salvage.png</v>
+      </c>
+      <c r="G12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>348</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>Ballast</v>
+      </c>
+      <c r="C13" t="s">
+        <v>337</v>
+      </c>
+      <c r="D13" t="s">
+        <v>422</v>
+      </c>
+      <c r="E13" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/ballast.png</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>349</v>
+      </c>
+      <c r="B14" t="str">
+        <f t="shared" si="0"/>
+        <v>Swell</v>
+      </c>
+      <c r="C14" t="s">
+        <v>436</v>
+      </c>
+      <c r="D14" t="s">
+        <v>422</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/swell.png</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>324</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>Tithe</v>
+      </c>
+      <c r="C15" t="s">
+        <v>323</v>
+      </c>
+      <c r="D15" t="s">
+        <v>430</v>
+      </c>
+      <c r="E15" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/tithe.png</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C7" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C8" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C9" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C10" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>329</v>
-      </c>
-      <c r="C11" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C13" t="s">
-        <v>322</v>
-      </c>
-      <c r="F13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C14" t="s">
-        <v>323</v>
-      </c>
-      <c r="F14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C15" t="s">
-        <v>324</v>
-      </c>
-      <c r="F15">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>Groove</v>
+      </c>
       <c r="C16" t="s">
         <v>325</v>
       </c>
-      <c r="F16">
+      <c r="D16" t="s">
+        <v>430</v>
+      </c>
+      <c r="E16" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/groove.png</v>
+      </c>
+      <c r="G16">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>327</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>Boil</v>
+      </c>
       <c r="C17" t="s">
-        <v>323</v>
-      </c>
-      <c r="F17">
+        <v>335</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/boil.png</v>
+      </c>
+      <c r="G17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>350</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>Tempered</v>
+      </c>
+      <c r="C18" t="s">
+        <v>328</v>
+      </c>
+      <c r="D18" t="s">
+        <v>422</v>
+      </c>
+      <c r="E18" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/tempered.png</v>
+      </c>
+      <c r="F18" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>333</v>
-      </c>
-      <c r="B18" t="s">
-        <v>332</v>
-      </c>
-      <c r="C18" t="s">
-        <v>331</v>
-      </c>
-      <c r="F18">
+      <c r="G18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>349</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
+        <v>Swell</v>
+      </c>
+      <c r="C19" t="s">
+        <v>329</v>
+      </c>
+      <c r="D19" t="s">
+        <v>427</v>
+      </c>
+      <c r="E19" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/swell.png</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>353</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>Ember</v>
+      </c>
+      <c r="C20" t="s">
+        <v>354</v>
+      </c>
+      <c r="D20" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>335</v>
-      </c>
-      <c r="C19" t="s">
-        <v>334</v>
-      </c>
-      <c r="F19">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>355</v>
+      </c>
+      <c r="B21" t="str">
+        <f t="shared" si="0"/>
+        <v>Smolder</v>
+      </c>
+      <c r="C21" t="s">
+        <v>356</v>
+      </c>
+      <c r="D21" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>358</v>
+      </c>
+      <c r="B22" t="str">
+        <f t="shared" si="0"/>
+        <v>Mercy</v>
+      </c>
+      <c r="C22" t="s">
+        <v>357</v>
+      </c>
+      <c r="D22" t="s">
+        <v>392</v>
+      </c>
+      <c r="G22">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>337</v>
-      </c>
-      <c r="C20" t="s">
-        <v>336</v>
-      </c>
-      <c r="F20">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>360</v>
+      </c>
+      <c r="B23" t="str">
+        <f t="shared" si="0"/>
+        <v>Heft</v>
+      </c>
+      <c r="C23" t="s">
+        <v>359</v>
+      </c>
+      <c r="D23" t="s">
+        <v>392</v>
+      </c>
+      <c r="G23">
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>339</v>
-      </c>
-      <c r="C21" t="s">
-        <v>338</v>
-      </c>
-      <c r="F21">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>362</v>
+      </c>
+      <c r="B24" t="str">
+        <f t="shared" si="0"/>
+        <v>Followthrough</v>
+      </c>
+      <c r="C24" t="s">
+        <v>361</v>
+      </c>
+      <c r="D24" t="s">
+        <v>392</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>363</v>
+      </c>
+      <c r="B25" t="str">
+        <f t="shared" si="0"/>
+        <v>Martyr</v>
+      </c>
+      <c r="C25" t="s">
+        <v>364</v>
+      </c>
+      <c r="D25" t="s">
+        <v>391</v>
+      </c>
+      <c r="G25">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C22" t="s">
-        <v>340</v>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>365</v>
+      </c>
+      <c r="B26" t="str">
+        <f t="shared" si="0"/>
+        <v>Penance</v>
+      </c>
+      <c r="C26" t="s">
+        <v>366</v>
+      </c>
+      <c r="D26" t="s">
+        <v>391</v>
+      </c>
+      <c r="G26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>367</v>
+      </c>
+      <c r="B27" t="str">
+        <f t="shared" si="0"/>
+        <v>Surrogate</v>
+      </c>
+      <c r="C27" t="s">
+        <v>368</v>
+      </c>
+      <c r="D27" t="s">
+        <v>391</v>
+      </c>
+      <c r="G27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>369</v>
+      </c>
+      <c r="B28" t="str">
+        <f t="shared" si="0"/>
+        <v>Glass</v>
+      </c>
+      <c r="C28" t="s">
+        <v>370</v>
+      </c>
+      <c r="D28" t="s">
+        <v>391</v>
+      </c>
+      <c r="G28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>371</v>
+      </c>
+      <c r="B29" t="str">
+        <f t="shared" si="0"/>
+        <v>Payback</v>
+      </c>
+      <c r="C29" t="s">
+        <v>372</v>
+      </c>
+      <c r="D29" t="s">
+        <v>391</v>
+      </c>
+      <c r="G29">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>373</v>
+      </c>
+      <c r="B30" t="str">
+        <f t="shared" si="0"/>
+        <v>Reduce</v>
+      </c>
+      <c r="C30" t="s">
+        <v>374</v>
+      </c>
+      <c r="D30" t="s">
+        <v>391</v>
+      </c>
+      <c r="G30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>375</v>
+      </c>
+      <c r="B31" t="str">
+        <f t="shared" si="0"/>
+        <v>Surplus</v>
+      </c>
+      <c r="C31" t="s">
+        <v>376</v>
+      </c>
+      <c r="D31" t="s">
+        <v>390</v>
+      </c>
+      <c r="G31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>377</v>
+      </c>
+      <c r="B32" t="str">
+        <f t="shared" si="0"/>
+        <v>Refund</v>
+      </c>
+      <c r="C32" t="s">
+        <v>378</v>
+      </c>
+      <c r="D32" t="s">
+        <v>390</v>
+      </c>
+      <c r="G32">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>379</v>
+      </c>
+      <c r="B33" t="str">
+        <f t="shared" si="0"/>
+        <v>Subsidy</v>
+      </c>
+      <c r="C33" t="s">
+        <v>380</v>
+      </c>
+      <c r="D33" t="s">
+        <v>390</v>
+      </c>
+      <c r="G33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>381</v>
+      </c>
+      <c r="B34" t="str">
+        <f t="shared" si="0"/>
+        <v>Swarm</v>
+      </c>
+      <c r="C34" t="s">
+        <v>382</v>
+      </c>
+      <c r="D34" t="s">
+        <v>390</v>
+      </c>
+      <c r="G34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>347</v>
+      </c>
+      <c r="B35" t="str">
+        <f t="shared" si="0"/>
+        <v>Salvage</v>
+      </c>
+      <c r="C35" t="s">
+        <v>383</v>
+      </c>
+      <c r="D35" t="s">
+        <v>390</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>384</v>
+      </c>
+      <c r="B36" t="str">
+        <f t="shared" si="0"/>
+        <v>Premium</v>
+      </c>
+      <c r="C36" t="s">
+        <v>385</v>
+      </c>
+      <c r="D36" t="s">
+        <v>390</v>
+      </c>
+      <c r="G36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>387</v>
+      </c>
+      <c r="B37" t="str">
+        <f t="shared" si="0"/>
+        <v>Vigil</v>
+      </c>
+      <c r="C37" t="s">
+        <v>386</v>
+      </c>
+      <c r="D37" t="s">
+        <v>390</v>
+      </c>
+      <c r="G37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>388</v>
+      </c>
+      <c r="B38" t="str">
+        <f t="shared" si="0"/>
+        <v>Keeper</v>
+      </c>
+      <c r="C38" t="s">
+        <v>389</v>
+      </c>
+      <c r="D38" t="s">
+        <v>390</v>
+      </c>
+      <c r="G38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>394</v>
+      </c>
+      <c r="B39" t="str">
+        <f t="shared" si="0"/>
+        <v>Unburden</v>
+      </c>
+      <c r="C39" t="s">
+        <v>393</v>
+      </c>
+      <c r="D39" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>395</v>
+      </c>
+      <c r="B40" t="str">
+        <f t="shared" si="0"/>
+        <v>Courier</v>
+      </c>
+      <c r="C40" t="s">
+        <v>396</v>
+      </c>
+      <c r="D40" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>402</v>
+      </c>
+      <c r="B41" t="str">
+        <f t="shared" si="0"/>
+        <v>Auspice</v>
+      </c>
+      <c r="C41" t="s">
+        <v>397</v>
+      </c>
+      <c r="D41" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>401</v>
+      </c>
+      <c r="B42" t="str">
+        <f t="shared" si="0"/>
+        <v>Brittle</v>
+      </c>
+      <c r="C42" t="s">
+        <v>398</v>
+      </c>
+      <c r="D42" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>399</v>
+      </c>
+      <c r="B43" t="str">
+        <f t="shared" si="0"/>
+        <v>Imbue</v>
+      </c>
+      <c r="C43" t="s">
+        <v>400</v>
+      </c>
+      <c r="D43" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>403</v>
+      </c>
+      <c r="B44" t="str">
+        <f t="shared" si="0"/>
+        <v>Sepsis</v>
+      </c>
+      <c r="C44" t="s">
+        <v>404</v>
+      </c>
+      <c r="D44" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>405</v>
+      </c>
+      <c r="B45" t="str">
+        <f t="shared" si="0"/>
+        <v>Glacier</v>
+      </c>
+      <c r="C45" t="s">
+        <v>406</v>
+      </c>
+      <c r="D45" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>407</v>
+      </c>
+      <c r="B46" t="str">
+        <f t="shared" si="0"/>
+        <v>Hairpin</v>
+      </c>
+      <c r="C46" t="s">
+        <v>408</v>
+      </c>
+      <c r="D46" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>409</v>
+      </c>
+      <c r="B47" t="str">
+        <f t="shared" si="0"/>
+        <v>Leftover</v>
+      </c>
+      <c r="C47" t="s">
+        <v>410</v>
+      </c>
+      <c r="D47" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>412</v>
+      </c>
+      <c r="B48" t="str">
+        <f t="shared" si="0"/>
+        <v>Daze</v>
+      </c>
+      <c r="C48" t="s">
+        <v>411</v>
+      </c>
+      <c r="D48" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>415</v>
+      </c>
+      <c r="B49" t="str">
+        <f t="shared" si="0"/>
+        <v>Sickly</v>
+      </c>
+      <c r="C49" t="s">
+        <v>416</v>
+      </c>
+      <c r="D49" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>414</v>
+      </c>
+      <c r="B50" t="str">
+        <f t="shared" si="0"/>
+        <v>Wide</v>
+      </c>
+      <c r="C50" t="s">
+        <v>413</v>
+      </c>
+      <c r="D50" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>270</v>
+      </c>
+      <c r="B51" t="str">
+        <f t="shared" si="0"/>
+        <v>Fright</v>
+      </c>
+      <c r="C51" t="s">
+        <v>417</v>
+      </c>
+      <c r="D51" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>424</v>
+      </c>
+      <c r="B52" t="str">
+        <f t="shared" si="0"/>
+        <v>Fuse</v>
+      </c>
+      <c r="C52" t="s">
+        <v>423</v>
+      </c>
+      <c r="D52" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>426</v>
+      </c>
+      <c r="B53" t="str">
+        <f t="shared" si="0"/>
+        <v>Clearcut</v>
+      </c>
+      <c r="C53" t="s">
+        <v>425</v>
+      </c>
+      <c r="D53" t="s">
+        <v>433</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G19" xr:uid="{9F642FAC-7326-47E8-9F14-D9D50EC3456E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -7676,7 +8787,7 @@
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="14.7109375" customWidth="1"/>
@@ -8146,7 +9257,7 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>7</v>
+        <v>338</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>0</v>
@@ -8157,7 +9268,7 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>7</v>
+        <v>338</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>1</v>
@@ -8168,12 +9279,67 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>7</v>
+        <v>338</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>42</v>
       </c>
       <c r="C45" s="14" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="14" t="s">
+        <v>338</v>
+      </c>
+      <c r="B46" s="14" t="s">
+        <v>334</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="14" t="s">
+        <v>338</v>
+      </c>
+      <c r="B47" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C47" s="14" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B48" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C48" s="17" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" s="17" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B50" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C50" s="17" t="s">
         <v>252</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement Rite slot inspection and update summoning circle mechanics
- Added functionality for inspecting filled RiteSlots within proximity, displaying associated RiteInfo (name and description) when no orb is captured.
- Introduced a dashed focus overlay for inspected RiteSlots to enhance visual feedback.
- Updated the summoning circle scene to include new RiteSlots and associated UI elements for improved user experience during rituals.
- Revised `GAME_BRIEF.md` to document the new Rite inspection mechanics and their impact on gameplay.
- Enhanced `PROJECT_MAP.md` to reflect changes related to the RiteSlots and their integration into the game.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B608D2-9E3C-48A3-B49F-FD85E40CB19F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51F0D366-EA39-4FAF-8190-4D30EFB1E1FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -9307,7 +9307,7 @@
         <v>21</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update summoning circle scene with new rite textures and slots
- Added new textures for frostburn, tempered, and clash rites to enhance visual feedback.
- Adjusted positions of glyph sockets for better alignment within the summoning circle.
- Updated rite slots to include visibility settings and associated textures for improved user experience during rituals.
- Made minor adjustments to node properties for better organization and clarity in the scene structure.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51F0D366-EA39-4FAF-8190-4D30EFB1E1FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BCE543D-063E-4B49-BA66-906644CD52E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">objects_OLD!$A$1:$U$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">orbs!$A$1:$W$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">rites!$A$1:$G$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">rites!$A$1:$G$18</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="437">
   <si>
     <t>id</t>
   </si>
@@ -1353,10 +1353,10 @@
     <t>dash</t>
   </si>
   <si>
-    <t>clyph</t>
-  </si>
-  <si>
     <t>Thrown glyphs stun 0.5 seconds on hit</t>
+  </si>
+  <si>
+    <t>mining</t>
   </si>
 </sst>
 </file>
@@ -5838,7 +5838,7 @@
   <sheetPr>
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" customWidth="1"/>
@@ -5877,7 +5877,7 @@
         <v>330</v>
       </c>
       <c r="B2" t="str">
-        <f t="shared" ref="B2:B53" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
+        <f t="shared" ref="B2:B52" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Frostburn</v>
       </c>
       <c r="C2" t="s">
@@ -5909,7 +5909,7 @@
         <v>429</v>
       </c>
       <c r="E3" t="str">
-        <f t="shared" ref="E3:E19" si="1">"res://ui/rites/"&amp;A3&amp;".png"</f>
+        <f t="shared" ref="E3:E52" si="1">"res://ui/rites/"&amp;A3&amp;".png"</f>
         <v>res://ui/rites/ward.png</v>
       </c>
       <c r="F3" t="b">
@@ -6067,10 +6067,10 @@
         <v>Concuss</v>
       </c>
       <c r="C11" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="D11" t="s">
-        <v>435</v>
+        <v>422</v>
       </c>
       <c r="E11" t="str">
         <f t="shared" si="1"/>
@@ -6082,11 +6082,11 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>347</v>
+        <v>436</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
-        <v>Salvage</v>
+        <v>Mining</v>
       </c>
       <c r="C12" t="s">
         <v>319</v>
@@ -6096,7 +6096,7 @@
       </c>
       <c r="E12" t="str">
         <f t="shared" si="1"/>
-        <v>res://ui/rites/salvage.png</v>
+        <v>res://ui/rites/mining.png</v>
       </c>
       <c r="G12">
         <v>2</v>
@@ -6126,21 +6126,21 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>349</v>
+        <v>324</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
-        <v>Swell</v>
+        <v>Tithe</v>
       </c>
       <c r="C14" t="s">
-        <v>436</v>
+        <v>323</v>
       </c>
       <c r="D14" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="E14" t="str">
         <f t="shared" si="1"/>
-        <v>res://ui/rites/swell.png</v>
+        <v>res://ui/rites/tithe.png</v>
       </c>
       <c r="G14">
         <v>1</v>
@@ -6148,21 +6148,21 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
-        <v>Tithe</v>
+        <v>Groove</v>
       </c>
       <c r="C15" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="D15" t="s">
         <v>430</v>
       </c>
       <c r="E15" t="str">
         <f t="shared" si="1"/>
-        <v>res://ui/rites/tithe.png</v>
+        <v>res://ui/rites/groove.png</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -6170,43 +6170,46 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
-        <v>Groove</v>
+        <v>Boil</v>
       </c>
       <c r="C16" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
       <c r="D16" t="s">
-        <v>430</v>
+        <v>17</v>
       </c>
       <c r="E16" t="str">
         <f t="shared" si="1"/>
-        <v>res://ui/rites/groove.png</v>
+        <v>res://ui/rites/boil.png</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>327</v>
+        <v>350</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
-        <v>Boil</v>
+        <v>Tempered</v>
       </c>
       <c r="C17" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="D17" t="s">
-        <v>17</v>
+        <v>422</v>
       </c>
       <c r="E17" t="str">
         <f t="shared" si="1"/>
-        <v>res://ui/rites/boil.png</v>
+        <v>res://ui/rites/tempered.png</v>
+      </c>
+      <c r="F17" t="b">
+        <v>1</v>
       </c>
       <c r="G17">
         <v>2</v>
@@ -6214,617 +6217,728 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
-        <v>Tempered</v>
+        <v>Swell</v>
       </c>
       <c r="C18" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D18" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="E18" t="str">
         <f t="shared" si="1"/>
-        <v>res://ui/rites/tempered.png</v>
-      </c>
-      <c r="F18" t="b">
-        <v>1</v>
-      </c>
-      <c r="G18">
-        <v>2</v>
+        <v>res://ui/rites/swell.png</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
-        <v>Swell</v>
+        <v>Ember</v>
       </c>
       <c r="C19" t="s">
-        <v>329</v>
+        <v>354</v>
       </c>
       <c r="D19" t="s">
-        <v>427</v>
+        <v>16</v>
       </c>
       <c r="E19" t="str">
         <f t="shared" si="1"/>
-        <v>res://ui/rites/swell.png</v>
+        <v>res://ui/rites/ember.png</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
-        <v>Ember</v>
+        <v>Smolder</v>
       </c>
       <c r="C20" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D20" t="s">
         <v>16</v>
       </c>
+      <c r="E20" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/smolder.png</v>
+      </c>
       <c r="G20">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
-        <v>Smolder</v>
+        <v>Mercy</v>
       </c>
       <c r="C21" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D21" t="s">
-        <v>16</v>
+        <v>392</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/mercy.png</v>
       </c>
       <c r="G21">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
-        <v>Mercy</v>
+        <v>Heft</v>
       </c>
       <c r="C22" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="D22" t="s">
         <v>392</v>
       </c>
+      <c r="E22" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/heft.png</v>
+      </c>
       <c r="G22">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
-        <v>Heft</v>
+        <v>Followthrough</v>
       </c>
       <c r="C23" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D23" t="s">
         <v>392</v>
       </c>
+      <c r="E23" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/followthrough.png</v>
+      </c>
       <c r="G23">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
-        <v>Followthrough</v>
+        <v>Martyr</v>
       </c>
       <c r="C24" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="D24" t="s">
-        <v>392</v>
+        <v>391</v>
+      </c>
+      <c r="E24" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/martyr.png</v>
       </c>
       <c r="G24">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
-        <v>Martyr</v>
+        <v>Penance</v>
       </c>
       <c r="C25" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="D25" t="s">
         <v>391</v>
       </c>
+      <c r="E25" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/penance.png</v>
+      </c>
       <c r="G25">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
-        <v>Penance</v>
+        <v>Surrogate</v>
       </c>
       <c r="C26" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="D26" t="s">
         <v>391</v>
       </c>
+      <c r="E26" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/surrogate.png</v>
+      </c>
       <c r="G26">
         <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
-        <v>Surrogate</v>
+        <v>Glass</v>
       </c>
       <c r="C27" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D27" t="s">
         <v>391</v>
       </c>
+      <c r="E27" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/glass.png</v>
+      </c>
       <c r="G27">
         <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
-        <v>Glass</v>
+        <v>Payback</v>
       </c>
       <c r="C28" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D28" t="s">
         <v>391</v>
       </c>
+      <c r="E28" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/payback.png</v>
+      </c>
       <c r="G28">
         <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="0"/>
-        <v>Payback</v>
+        <v>Reduce</v>
       </c>
       <c r="C29" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D29" t="s">
         <v>391</v>
       </c>
+      <c r="E29" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/reduce.png</v>
+      </c>
       <c r="G29">
         <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="0"/>
-        <v>Reduce</v>
+        <v>Surplus</v>
       </c>
       <c r="C30" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="D30" t="s">
-        <v>391</v>
+        <v>390</v>
+      </c>
+      <c r="E30" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/surplus.png</v>
       </c>
       <c r="G30">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="0"/>
-        <v>Surplus</v>
+        <v>Refund</v>
       </c>
       <c r="C31" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D31" t="s">
         <v>390</v>
       </c>
+      <c r="E31" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/refund.png</v>
+      </c>
       <c r="G31">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="0"/>
-        <v>Refund</v>
+        <v>Subsidy</v>
       </c>
       <c r="C32" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="D32" t="s">
         <v>390</v>
       </c>
+      <c r="E32" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/subsidy.png</v>
+      </c>
       <c r="G32">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="0"/>
-        <v>Subsidy</v>
+        <v>Swarm</v>
       </c>
       <c r="C33" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="D33" t="s">
         <v>390</v>
       </c>
+      <c r="E33" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/swarm.png</v>
+      </c>
       <c r="G33">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>381</v>
+        <v>347</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="0"/>
-        <v>Swarm</v>
+        <v>Salvage</v>
       </c>
       <c r="C34" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D34" t="s">
         <v>390</v>
       </c>
+      <c r="E34" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/salvage.png</v>
+      </c>
       <c r="G34">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>347</v>
+        <v>384</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="0"/>
-        <v>Salvage</v>
+        <v>Premium</v>
       </c>
       <c r="C35" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D35" t="s">
         <v>390</v>
       </c>
+      <c r="E35" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/premium.png</v>
+      </c>
       <c r="G35">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="0"/>
-        <v>Premium</v>
+        <v>Vigil</v>
       </c>
       <c r="C36" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D36" t="s">
         <v>390</v>
       </c>
+      <c r="E36" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/vigil.png</v>
+      </c>
       <c r="G36">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="0"/>
-        <v>Vigil</v>
+        <v>Keeper</v>
       </c>
       <c r="C37" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="D37" t="s">
         <v>390</v>
       </c>
+      <c r="E37" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/keeper.png</v>
+      </c>
       <c r="G37">
         <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="0"/>
-        <v>Keeper</v>
+        <v>Unburden</v>
       </c>
       <c r="C38" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="D38" t="s">
-        <v>390</v>
-      </c>
-      <c r="G38">
-        <v>1</v>
+        <v>422</v>
+      </c>
+      <c r="E38" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/unburden.png</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="0"/>
-        <v>Unburden</v>
+        <v>Courier</v>
       </c>
       <c r="C39" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="D39" t="s">
         <v>422</v>
       </c>
+      <c r="E39" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/courier.png</v>
+      </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="0"/>
-        <v>Courier</v>
+        <v>Auspice</v>
       </c>
       <c r="C40" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D40" t="s">
         <v>422</v>
       </c>
+      <c r="E40" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/auspice.png</v>
+      </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="0"/>
-        <v>Auspice</v>
+        <v>Brittle</v>
       </c>
       <c r="C41" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D41" t="s">
         <v>422</v>
       </c>
+      <c r="E41" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/brittle.png</v>
+      </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="0"/>
-        <v>Brittle</v>
+        <v>Imbue</v>
       </c>
       <c r="C42" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D42" t="s">
         <v>422</v>
       </c>
+      <c r="E42" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/imbue.png</v>
+      </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="0"/>
-        <v>Imbue</v>
+        <v>Sepsis</v>
       </c>
       <c r="C43" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="D43" t="s">
-        <v>422</v>
+        <v>421</v>
+      </c>
+      <c r="E43" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/sepsis.png</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="0"/>
-        <v>Sepsis</v>
+        <v>Glacier</v>
       </c>
       <c r="C44" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="D44" t="s">
-        <v>421</v>
+        <v>17</v>
+      </c>
+      <c r="E44" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/glacier.png</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="0"/>
-        <v>Glacier</v>
+        <v>Hairpin</v>
       </c>
       <c r="C45" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D45" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="E45" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/hairpin.png</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="0"/>
-        <v>Hairpin</v>
+        <v>Leftover</v>
       </c>
       <c r="C46" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="D46" t="s">
         <v>18</v>
       </c>
+      <c r="E46" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/leftover.png</v>
+      </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="0"/>
-        <v>Leftover</v>
+        <v>Daze</v>
       </c>
       <c r="C47" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D47" t="s">
         <v>18</v>
       </c>
+      <c r="E47" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/daze.png</v>
+      </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="0"/>
-        <v>Daze</v>
+        <v>Sickly</v>
       </c>
       <c r="C48" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="D48" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+        <v>420</v>
+      </c>
+      <c r="E48" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/sickly.png</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="0"/>
-        <v>Sickly</v>
+        <v>Wide</v>
       </c>
       <c r="C49" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="D49" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+      <c r="E49" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/wide.png</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>414</v>
+        <v>270</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="0"/>
-        <v>Wide</v>
+        <v>Fright</v>
       </c>
       <c r="C50" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="D50" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+      <c r="E50" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/fright.png</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>270</v>
+        <v>424</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="0"/>
-        <v>Fright</v>
+        <v>Fuse</v>
       </c>
       <c r="C51" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="D51" t="s">
         <v>418</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E51" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/fuse.png</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="0"/>
-        <v>Fuse</v>
+        <v>Clearcut</v>
       </c>
       <c r="C52" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D52" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>426</v>
-      </c>
-      <c r="B53" t="str">
-        <f t="shared" si="0"/>
-        <v>Clearcut</v>
-      </c>
-      <c r="C53" t="s">
-        <v>425</v>
-      </c>
-      <c r="D53" t="s">
         <v>433</v>
       </c>
+      <c r="E52" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/clearcut.png</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G19" xr:uid="{9F642FAC-7326-47E8-9F14-D9D50EC3456E}"/>
+  <autoFilter ref="A1:G18" xr:uid="{9F642FAC-7326-47E8-9F14-D9D50EC3456E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Implement enemy navigation enhancements and update related documentation
- Introduced a new navigation system for enemy packs, allowing them to surround players using ring slots instead of stacking on their feet, improving tactical movement.
- Updated `DECISIONS.md` to document the rationale behind the new navigation mechanics and their impact on gameplay.
- Revised `GAME_BRIEF.md` to clarify the behavior of chaser enemies and their new slot-based approach.
- Enhanced `PROJECT_MAP.md` to reflect changes in the navigation component and its integration into enemy AI.
- Adjusted the `navigation_component.gd` to support the new slot assignment logic and improve enemy pathfinding efficiency.
- Updated the ogre enemy configuration to prefer forward slots during pursuit, enhancing their tactical behavior.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BCE543D-063E-4B49-BA66-906644CD52E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C984E57-CCAB-40EE-B5A4-57621683C44F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -195,72 +195,39 @@
     <t>coal</t>
   </si>
   <si>
-    <t>Burn on enemy hit</t>
-  </si>
-  <si>
     <t>fury</t>
   </si>
   <si>
-    <t>Damage</t>
-  </si>
-  <si>
     <t>blast</t>
   </si>
   <si>
-    <t>On hit, that % of the damage also hits nearby enemies</t>
-  </si>
-  <si>
     <t>rime</t>
   </si>
   <si>
-    <t>Chill enemy on hit</t>
-  </si>
-  <si>
     <t>sooth</t>
   </si>
   <si>
-    <t>This orb deals less damage to players</t>
-  </si>
-  <si>
     <t>bounty</t>
   </si>
   <si>
-    <t>Glyph drop chance from enemies</t>
-  </si>
-  <si>
     <t>static</t>
   </si>
   <si>
-    <t>Shock on enemy hit</t>
-  </si>
-  <si>
     <t>shear</t>
   </si>
   <si>
-    <t>Critical chance</t>
-  </si>
-  <si>
     <t>drag</t>
   </si>
   <si>
-    <t>Decreases speed</t>
-  </si>
-  <si>
     <t>blight</t>
   </si>
   <si>
     <t>dense</t>
   </si>
   <si>
-    <t>Increases weight</t>
-  </si>
-  <si>
     <t>crush</t>
   </si>
   <si>
-    <t>Critical damage</t>
-  </si>
-  <si>
     <t>orb_id</t>
   </si>
   <si>
@@ -933,9 +900,6 @@
     <t>Stacks on hit. Lowers damage dealt and increases damage received by 5% per stack.</t>
   </si>
   <si>
-    <t>Blight on enemy hit</t>
-  </si>
-  <si>
     <t>spore</t>
   </si>
   <si>
@@ -1357,6 +1321,42 @@
   </si>
   <si>
     <t>mining</t>
+  </si>
+  <si>
+    <t>Increase Splash by X</t>
+  </si>
+  <si>
+    <t>Increase Chill by X</t>
+  </si>
+  <si>
+    <t>Increase Burn by X</t>
+  </si>
+  <si>
+    <t>Decrease Self Damage by X</t>
+  </si>
+  <si>
+    <t>Increase Glyph Drop by X</t>
+  </si>
+  <si>
+    <t>Increase Shock by X</t>
+  </si>
+  <si>
+    <t>Decrease Speed by X</t>
+  </si>
+  <si>
+    <t>Increase Blight by X</t>
+  </si>
+  <si>
+    <t>Increase Damage by X</t>
+  </si>
+  <si>
+    <t>Increases Weight by X</t>
+  </si>
+  <si>
+    <t>Increase Crit Damage by X</t>
+  </si>
+  <si>
+    <t>Increase Crit Chance by X</t>
   </si>
 </sst>
 </file>
@@ -1980,7 +1980,7 @@
         <v>18</v>
       </c>
       <c r="U1" s="9" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="V1" s="13" t="s">
         <v>20</v>
@@ -2135,7 +2135,7 @@
         <v>Contagion</v>
       </c>
       <c r="C4" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
       <c r="D4" t="s">
         <v>30</v>
@@ -2210,7 +2210,7 @@
         <v>Ghost</v>
       </c>
       <c r="C5" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="D5" t="s">
         <v>27</v>
@@ -2285,7 +2285,7 @@
         <v>Inferno</v>
       </c>
       <c r="C6" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
       <c r="D6" t="s">
         <v>28</v>
@@ -2360,7 +2360,7 @@
         <v>Shard</v>
       </c>
       <c r="C7" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="D7" t="s">
         <v>34</v>
@@ -2435,7 +2435,7 @@
         <v>Runic</v>
       </c>
       <c r="C8" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="D8" t="s">
         <v>34</v>
@@ -2563,7 +2563,7 @@
         <v>Yes</v>
       </c>
       <c r="I10" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="V10" t="str">
         <f t="shared" si="3"/>
@@ -2582,7 +2582,7 @@
         <v>Destroyer</v>
       </c>
       <c r="C11" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="D11" t="s">
         <v>28</v>
@@ -2650,14 +2650,14 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Vulcano</v>
       </c>
       <c r="C12" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="D12" t="s">
         <v>28</v>
@@ -2677,7 +2677,7 @@
         <v>Yes</v>
       </c>
       <c r="I12" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="J12">
         <v>5</v>
@@ -2725,14 +2725,14 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" ref="B13:B44" si="4">PROPER(SUBSTITUTE(A13,"_"," "))</f>
         <v>Lure</v>
       </c>
       <c r="C13" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="D13" t="s">
         <v>34</v>
@@ -2762,7 +2762,7 @@
         <v/>
       </c>
       <c r="C14" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="D14" t="s">
         <v>34</v>
@@ -2788,14 +2788,14 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="4"/>
         <v>Hunger</v>
       </c>
       <c r="C15" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="D15" t="s">
         <v>30</v>
@@ -2821,14 +2821,14 @@
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="4"/>
         <v>Vengance</v>
       </c>
       <c r="C16" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="D16" t="s">
         <v>27</v>
@@ -2848,7 +2848,7 @@
         <v>Yes</v>
       </c>
       <c r="I16" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="V16" t="str">
         <f t="shared" si="5"/>
@@ -2857,14 +2857,14 @@
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="4"/>
         <v>Hunter</v>
       </c>
       <c r="C17" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="D17" t="s">
         <v>28</v>
@@ -2890,14 +2890,14 @@
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="4"/>
         <v>Nova</v>
       </c>
       <c r="C18" t="s">
-        <v>292</v>
+        <v>281</v>
       </c>
       <c r="D18" t="s">
         <v>34</v>
@@ -2965,14 +2965,14 @@
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="4"/>
         <v>Charge</v>
       </c>
       <c r="C19" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="D19" t="s">
         <v>27</v>
@@ -3974,7 +3974,7 @@
         <v>Coal</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>427</v>
       </c>
       <c r="D2" t="s">
         <v>28</v>
@@ -3998,14 +3998,14 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Fury</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>433</v>
       </c>
       <c r="D3" t="s">
         <v>28</v>
@@ -4029,14 +4029,14 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Blast</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>425</v>
       </c>
       <c r="D4" t="s">
         <v>28</v>
@@ -4060,14 +4060,14 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Rime</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>426</v>
       </c>
       <c r="D5" t="s">
         <v>34</v>
@@ -4091,14 +4091,14 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Sooth</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>428</v>
       </c>
       <c r="D6" t="s">
         <v>34</v>
@@ -4122,14 +4122,14 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Bounty</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>429</v>
       </c>
       <c r="D7" t="s">
         <v>34</v>
@@ -4153,14 +4153,14 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Static</v>
       </c>
       <c r="C8" t="s">
-        <v>61</v>
+        <v>430</v>
       </c>
       <c r="D8" t="s">
         <v>27</v>
@@ -4184,14 +4184,14 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Shear</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>436</v>
       </c>
       <c r="D9" t="s">
         <v>27</v>
@@ -4215,14 +4215,14 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>Drag</v>
       </c>
       <c r="C10" t="s">
-        <v>65</v>
+        <v>431</v>
       </c>
       <c r="D10" t="s">
         <v>27</v>
@@ -4246,20 +4246,20 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Spore</v>
       </c>
       <c r="C11" t="s">
-        <v>295</v>
+        <v>432</v>
       </c>
       <c r="D11" t="s">
         <v>30</v>
       </c>
       <c r="E11" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -4277,14 +4277,14 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Dense</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>434</v>
       </c>
       <c r="D12" t="s">
         <v>30</v>
@@ -4308,14 +4308,14 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Crush</v>
       </c>
       <c r="C13" t="s">
-        <v>70</v>
+        <v>435</v>
       </c>
       <c r="D13" t="s">
         <v>30</v>
@@ -4375,7 +4375,7 @@
         <v>Damage</v>
       </c>
       <c r="C2" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4387,7 +4387,7 @@
         <v>Splash</v>
       </c>
       <c r="C3" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4399,7 +4399,7 @@
         <v>Burn</v>
       </c>
       <c r="C4" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4411,7 +4411,7 @@
         <v>Self Damage</v>
       </c>
       <c r="C5" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4423,7 +4423,7 @@
         <v>Glyph Drop</v>
       </c>
       <c r="C6" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4435,7 +4435,7 @@
         <v>Chill</v>
       </c>
       <c r="C7" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4447,7 +4447,7 @@
         <v>Crit Chance</v>
       </c>
       <c r="C8" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -4459,7 +4459,7 @@
         <v>Speed</v>
       </c>
       <c r="C9" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -4471,7 +4471,7 @@
         <v>Shock</v>
       </c>
       <c r="C10" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -4483,7 +4483,7 @@
         <v>Weight</v>
       </c>
       <c r="C11" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -4495,19 +4495,19 @@
         <v>Crit Damage</v>
       </c>
       <c r="C12" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Blight</v>
       </c>
       <c r="C13" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>
@@ -4539,7 +4539,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>42</v>
@@ -4559,7 +4559,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B27" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
@@ -4569,7 +4569,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="E2" t="s">
         <v>27</v>
@@ -4590,7 +4590,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
@@ -4600,7 +4600,7 @@
         <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="E3" t="s">
         <v>28</v>
@@ -4621,7 +4621,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
@@ -4631,7 +4631,7 @@
         <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="E4" t="s">
         <v>28</v>
@@ -4652,7 +4652,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
@@ -4662,7 +4662,7 @@
         <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="E5" t="s">
         <v>27</v>
@@ -4683,7 +4683,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
@@ -4693,7 +4693,7 @@
         <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="E6" t="s">
         <v>28</v>
@@ -4714,7 +4714,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
@@ -4724,7 +4724,7 @@
         <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="E7" t="s">
         <v>34</v>
@@ -4745,7 +4745,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
@@ -4755,7 +4755,7 @@
         <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="E8" t="s">
         <v>27</v>
@@ -4776,7 +4776,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
@@ -4786,7 +4786,7 @@
         <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="E9" t="s">
         <v>27</v>
@@ -4807,7 +4807,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -4817,7 +4817,7 @@
         <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="1"/>
@@ -4829,7 +4829,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
@@ -4839,7 +4839,7 @@
         <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="H11" t="str">
         <f t="shared" si="1"/>
@@ -4851,7 +4851,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
@@ -4861,7 +4861,7 @@
         <v>33</v>
       </c>
       <c r="D12" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="1"/>
@@ -4873,7 +4873,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
@@ -4883,7 +4883,7 @@
         <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="H13" t="str">
         <f t="shared" si="1"/>
@@ -4895,7 +4895,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
@@ -4905,7 +4905,7 @@
         <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="1"/>
@@ -4917,7 +4917,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
@@ -4927,7 +4927,7 @@
         <v>29</v>
       </c>
       <c r="D15" t="s">
-        <v>300</v>
+        <v>288</v>
       </c>
       <c r="H15" t="str">
         <f t="shared" si="1"/>
@@ -4939,7 +4939,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
@@ -4949,7 +4949,7 @@
         <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="E16" t="s">
         <v>34</v>
@@ -4970,7 +4970,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
@@ -4980,7 +4980,7 @@
         <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="E17" t="s">
         <v>28</v>
@@ -5001,7 +5001,7 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
@@ -5011,7 +5011,7 @@
         <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="E18" t="s">
         <v>34</v>
@@ -5028,7 +5028,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
@@ -5038,7 +5038,7 @@
         <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="E19" t="s">
         <v>30</v>
@@ -5059,7 +5059,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
@@ -5069,7 +5069,7 @@
         <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E20" t="s">
         <v>28</v>
@@ -5090,7 +5090,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
@@ -5100,7 +5100,7 @@
         <v>36</v>
       </c>
       <c r="D21" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="E21" t="s">
         <v>27</v>
@@ -5121,7 +5121,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
@@ -5131,7 +5131,7 @@
         <v>36</v>
       </c>
       <c r="D22" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="H22" t="str">
         <f t="shared" si="1"/>
@@ -5143,17 +5143,17 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>Experience</v>
       </c>
       <c r="C23" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="D23" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="H23" t="str">
         <f t="shared" si="1"/>
@@ -5165,17 +5165,17 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v>Stalk</v>
       </c>
       <c r="C24" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="D24" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="H24" t="str">
         <f t="shared" si="1"/>
@@ -5187,17 +5187,17 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>Fright</v>
       </c>
       <c r="C25" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="D25" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="1"/>
@@ -5209,17 +5209,17 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
         <v>Gravity</v>
       </c>
       <c r="C26" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="D26" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="H26" t="str">
         <f t="shared" si="1"/>
@@ -5231,17 +5231,17 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
         <v>Recharge</v>
       </c>
       <c r="C27" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="D27" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="E27" t="s">
         <v>27</v>
@@ -5262,10 +5262,10 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C28" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="D28" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="E28" t="s">
         <v>27</v>
@@ -5286,10 +5286,10 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C29" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="D29" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="E29" t="s">
         <v>27</v>
@@ -5310,10 +5310,10 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C30" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="D30" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="H30" t="str">
         <f t="shared" si="1"/>
@@ -5331,7 +5331,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="H32" t="str">
         <f t="shared" si="1"/>
@@ -5860,31 +5860,31 @@
         <v>42</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B52" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Frostburn</v>
       </c>
       <c r="C2" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="D2" t="s">
-        <v>428</v>
+        <v>416</v>
       </c>
       <c r="E2" t="str">
         <f>"res://ui/rites/"&amp;A2&amp;".png"</f>
@@ -5893,20 +5893,23 @@
       <c r="F2" t="b">
         <v>1</v>
       </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Ward</v>
       </c>
       <c r="C3" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="D3" t="s">
-        <v>429</v>
+        <v>417</v>
       </c>
       <c r="E3" t="str">
         <f t="shared" ref="E3:E52" si="1">"res://ui/rites/"&amp;A3&amp;".png"</f>
@@ -5921,17 +5924,17 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Efficiancy</v>
       </c>
       <c r="C4" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="D4" t="s">
-        <v>430</v>
+        <v>418</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="1"/>
@@ -5940,17 +5943,17 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Rebate</v>
       </c>
       <c r="C5" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="D5" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="1"/>
@@ -5959,17 +5962,17 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Grace</v>
       </c>
       <c r="C6" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="D6" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="E6" t="str">
         <f t="shared" si="1"/>
@@ -5978,17 +5981,17 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Flux</v>
       </c>
       <c r="C7" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="D7" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="1"/>
@@ -5997,36 +6000,39 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Accelerant</v>
       </c>
       <c r="C8" t="s">
-        <v>431</v>
+        <v>419</v>
       </c>
       <c r="D8" t="s">
-        <v>432</v>
+        <v>420</v>
       </c>
       <c r="E8" t="str">
         <f t="shared" si="1"/>
         <v>res://ui/rites/accelerant.png</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Clash</v>
       </c>
       <c r="C9" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="D9" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" si="1"/>
@@ -6035,20 +6041,23 @@
       <c r="F9" t="b">
         <v>1</v>
       </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>Skewer</v>
       </c>
       <c r="C10" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="D10" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
       <c r="E10" t="str">
         <f t="shared" si="1"/>
@@ -6060,17 +6069,17 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Concuss</v>
       </c>
       <c r="C11" t="s">
-        <v>435</v>
+        <v>423</v>
       </c>
       <c r="D11" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="E11" t="str">
         <f t="shared" si="1"/>
@@ -6082,17 +6091,17 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>436</v>
+        <v>424</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Mining</v>
       </c>
       <c r="C12" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="D12" t="s">
-        <v>433</v>
+        <v>421</v>
       </c>
       <c r="E12" t="str">
         <f t="shared" si="1"/>
@@ -6104,17 +6113,17 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Ballast</v>
       </c>
       <c r="C13" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="D13" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="E13" t="str">
         <f t="shared" si="1"/>
@@ -6126,17 +6135,17 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>Tithe</v>
       </c>
       <c r="C14" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="D14" t="s">
-        <v>430</v>
+        <v>418</v>
       </c>
       <c r="E14" t="str">
         <f t="shared" si="1"/>
@@ -6148,17 +6157,17 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
         <v>Groove</v>
       </c>
       <c r="C15" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="D15" t="s">
-        <v>430</v>
+        <v>418</v>
       </c>
       <c r="E15" t="str">
         <f t="shared" si="1"/>
@@ -6170,14 +6179,14 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
         <v>Boil</v>
       </c>
       <c r="C16" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
       <c r="D16" t="s">
         <v>17</v>
@@ -6192,17 +6201,17 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>Tempered</v>
       </c>
       <c r="C17" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="D17" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="E17" t="str">
         <f t="shared" si="1"/>
@@ -6217,17 +6226,17 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>Swell</v>
       </c>
       <c r="C18" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="D18" t="s">
-        <v>427</v>
+        <v>415</v>
       </c>
       <c r="E18" t="str">
         <f t="shared" si="1"/>
@@ -6236,14 +6245,14 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
         <v>Ember</v>
       </c>
       <c r="C19" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
       <c r="D19" t="s">
         <v>16</v>
@@ -6258,14 +6267,14 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
         <v>Smolder</v>
       </c>
       <c r="C20" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="D20" t="s">
         <v>16</v>
@@ -6280,17 +6289,17 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
         <v>Mercy</v>
       </c>
       <c r="C21" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="D21" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="E21" t="str">
         <f t="shared" si="1"/>
@@ -6302,17 +6311,17 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v>Heft</v>
       </c>
       <c r="C22" t="s">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="D22" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="E22" t="str">
         <f t="shared" si="1"/>
@@ -6324,17 +6333,17 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>Followthrough</v>
       </c>
       <c r="C23" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
       <c r="D23" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="E23" t="str">
         <f t="shared" si="1"/>
@@ -6346,17 +6355,17 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v>Martyr</v>
       </c>
       <c r="C24" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="D24" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="E24" t="str">
         <f t="shared" si="1"/>
@@ -6368,17 +6377,17 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>Penance</v>
       </c>
       <c r="C25" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="D25" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="E25" t="str">
         <f t="shared" si="1"/>
@@ -6390,17 +6399,17 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
         <v>Surrogate</v>
       </c>
       <c r="C26" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
       <c r="D26" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="E26" t="str">
         <f t="shared" si="1"/>
@@ -6412,17 +6421,17 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
         <v>Glass</v>
       </c>
       <c r="C27" t="s">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="D27" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="E27" t="str">
         <f t="shared" si="1"/>
@@ -6434,17 +6443,17 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>Payback</v>
       </c>
       <c r="C28" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="D28" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="E28" t="str">
         <f t="shared" si="1"/>
@@ -6456,17 +6465,17 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>Reduce</v>
       </c>
       <c r="C29" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
       <c r="D29" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="E29" t="str">
         <f t="shared" si="1"/>
@@ -6478,17 +6487,17 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="0"/>
         <v>Surplus</v>
       </c>
       <c r="C30" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
       <c r="D30" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="E30" t="str">
         <f t="shared" si="1"/>
@@ -6500,17 +6509,17 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>Refund</v>
       </c>
       <c r="C31" t="s">
+        <v>366</v>
+      </c>
+      <c r="D31" t="s">
         <v>378</v>
-      </c>
-      <c r="D31" t="s">
-        <v>390</v>
       </c>
       <c r="E31" t="str">
         <f t="shared" si="1"/>
@@ -6522,17 +6531,17 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="0"/>
         <v>Subsidy</v>
       </c>
       <c r="C32" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="D32" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="E32" t="str">
         <f t="shared" si="1"/>
@@ -6544,17 +6553,17 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="0"/>
         <v>Swarm</v>
       </c>
       <c r="C33" t="s">
-        <v>382</v>
+        <v>370</v>
       </c>
       <c r="D33" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="E33" t="str">
         <f t="shared" si="1"/>
@@ -6566,17 +6575,17 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="0"/>
         <v>Salvage</v>
       </c>
       <c r="C34" t="s">
-        <v>383</v>
+        <v>371</v>
       </c>
       <c r="D34" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="E34" t="str">
         <f t="shared" si="1"/>
@@ -6588,17 +6597,17 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>384</v>
+        <v>372</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="0"/>
         <v>Premium</v>
       </c>
       <c r="C35" t="s">
-        <v>385</v>
+        <v>373</v>
       </c>
       <c r="D35" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="E35" t="str">
         <f t="shared" si="1"/>
@@ -6610,17 +6619,17 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>387</v>
+        <v>375</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="0"/>
         <v>Vigil</v>
       </c>
       <c r="C36" t="s">
-        <v>386</v>
+        <v>374</v>
       </c>
       <c r="D36" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="E36" t="str">
         <f t="shared" si="1"/>
@@ -6632,17 +6641,17 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>388</v>
+        <v>376</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="0"/>
         <v>Keeper</v>
       </c>
       <c r="C37" t="s">
-        <v>389</v>
+        <v>377</v>
       </c>
       <c r="D37" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="E37" t="str">
         <f t="shared" si="1"/>
@@ -6654,17 +6663,17 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>394</v>
+        <v>382</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="0"/>
         <v>Unburden</v>
       </c>
       <c r="C38" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="D38" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="E38" t="str">
         <f t="shared" si="1"/>
@@ -6673,17 +6682,17 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="0"/>
         <v>Courier</v>
       </c>
       <c r="C39" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="D39" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="E39" t="str">
         <f t="shared" si="1"/>
@@ -6692,17 +6701,17 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>402</v>
+        <v>390</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="0"/>
         <v>Auspice</v>
       </c>
       <c r="C40" t="s">
-        <v>397</v>
+        <v>385</v>
       </c>
       <c r="D40" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="E40" t="str">
         <f t="shared" si="1"/>
@@ -6711,17 +6720,17 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>401</v>
+        <v>389</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="0"/>
         <v>Brittle</v>
       </c>
       <c r="C41" t="s">
-        <v>398</v>
+        <v>386</v>
       </c>
       <c r="D41" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="E41" t="str">
         <f t="shared" si="1"/>
@@ -6730,17 +6739,17 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>399</v>
+        <v>387</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="0"/>
         <v>Imbue</v>
       </c>
       <c r="C42" t="s">
-        <v>400</v>
+        <v>388</v>
       </c>
       <c r="D42" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="E42" t="str">
         <f t="shared" si="1"/>
@@ -6749,17 +6758,17 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="0"/>
         <v>Sepsis</v>
       </c>
       <c r="C43" t="s">
-        <v>404</v>
+        <v>392</v>
       </c>
       <c r="D43" t="s">
-        <v>421</v>
+        <v>409</v>
       </c>
       <c r="E43" t="str">
         <f t="shared" si="1"/>
@@ -6768,14 +6777,14 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="0"/>
         <v>Glacier</v>
       </c>
       <c r="C44" t="s">
-        <v>406</v>
+        <v>394</v>
       </c>
       <c r="D44" t="s">
         <v>17</v>
@@ -6787,14 +6796,14 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>407</v>
+        <v>395</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="0"/>
         <v>Hairpin</v>
       </c>
       <c r="C45" t="s">
-        <v>408</v>
+        <v>396</v>
       </c>
       <c r="D45" t="s">
         <v>18</v>
@@ -6806,14 +6815,14 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>409</v>
+        <v>397</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="0"/>
         <v>Leftover</v>
       </c>
       <c r="C46" t="s">
-        <v>410</v>
+        <v>398</v>
       </c>
       <c r="D46" t="s">
         <v>18</v>
@@ -6825,14 +6834,14 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>412</v>
+        <v>400</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="0"/>
         <v>Daze</v>
       </c>
       <c r="C47" t="s">
-        <v>411</v>
+        <v>399</v>
       </c>
       <c r="D47" t="s">
         <v>18</v>
@@ -6844,17 +6853,17 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>415</v>
+        <v>403</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="0"/>
         <v>Sickly</v>
       </c>
       <c r="C48" t="s">
-        <v>416</v>
+        <v>404</v>
       </c>
       <c r="D48" t="s">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="E48" t="str">
         <f t="shared" si="1"/>
@@ -6863,17 +6872,17 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>414</v>
+        <v>402</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="0"/>
         <v>Wide</v>
       </c>
       <c r="C49" t="s">
-        <v>413</v>
+        <v>401</v>
       </c>
       <c r="D49" t="s">
-        <v>419</v>
+        <v>407</v>
       </c>
       <c r="E49" t="str">
         <f t="shared" si="1"/>
@@ -6882,17 +6891,17 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="0"/>
         <v>Fright</v>
       </c>
       <c r="C50" t="s">
-        <v>417</v>
+        <v>405</v>
       </c>
       <c r="D50" t="s">
-        <v>418</v>
+        <v>406</v>
       </c>
       <c r="E50" t="str">
         <f t="shared" si="1"/>
@@ -6901,17 +6910,17 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>424</v>
+        <v>412</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="0"/>
         <v>Fuse</v>
       </c>
       <c r="C51" t="s">
-        <v>423</v>
+        <v>411</v>
       </c>
       <c r="D51" t="s">
-        <v>418</v>
+        <v>406</v>
       </c>
       <c r="E51" t="str">
         <f t="shared" si="1"/>
@@ -6920,17 +6929,17 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>426</v>
+        <v>414</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="0"/>
         <v>Clearcut</v>
       </c>
       <c r="C52" t="s">
-        <v>425</v>
+        <v>413</v>
       </c>
       <c r="D52" t="s">
-        <v>433</v>
+        <v>421</v>
       </c>
       <c r="E52" t="str">
         <f t="shared" si="1"/>
@@ -6976,19 +6985,19 @@
         <v>Wayward</v>
       </c>
       <c r="C2" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Attracted</v>
       </c>
       <c r="C3" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -7000,175 +7009,175 @@
         <v>Spite</v>
       </c>
       <c r="C4" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Rooted</v>
       </c>
       <c r="C5" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Patrol</v>
       </c>
       <c r="C6" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Familiar</v>
       </c>
       <c r="C7" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Rail</v>
       </c>
       <c r="C8" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Tide</v>
       </c>
       <c r="C9" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>Blink</v>
       </c>
       <c r="C10" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Loyal</v>
       </c>
       <c r="C11" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Hexed</v>
       </c>
       <c r="C12" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Stalker</v>
       </c>
       <c r="C13" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>Herd</v>
       </c>
       <c r="C14" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
         <v>Greedy</v>
       </c>
       <c r="C15" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
         <v>Oathbound</v>
       </c>
       <c r="C16" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>Echo</v>
       </c>
       <c r="C17" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>Phasing</v>
       </c>
       <c r="C18" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -7211,55 +7220,55 @@
         <v>42</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q1" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="R1" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="T1" s="4" t="s">
         <v>141</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>152</v>
       </c>
       <c r="U1" s="3" t="s">
         <v>21</v>
@@ -7267,17 +7276,17 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B33" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Reception Desk</v>
       </c>
       <c r="C2" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="D2" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="F2" s="2">
         <v>0</v>
@@ -7298,13 +7307,13 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="O2">
         <v>2</v>
       </c>
       <c r="T2" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="U2" t="b">
         <v>1</v>
@@ -7312,17 +7321,17 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Straw Pallet</v>
       </c>
       <c r="C3" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="D3" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="F3" s="2">
         <v>1</v>
@@ -7343,10 +7352,10 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M3" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O3">
         <v>2</v>
@@ -7360,17 +7369,17 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Wood Frame Bed</v>
       </c>
       <c r="C4" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="D4" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="F4" s="2">
         <v>0</v>
@@ -7391,10 +7400,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M4" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O4">
         <v>2</v>
@@ -7403,10 +7412,10 @@
         <v>0</v>
       </c>
       <c r="S4" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="T4" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="U4" t="b">
         <v>1</v>
@@ -7414,17 +7423,17 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Bunk Bed</v>
       </c>
       <c r="C5" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="D5" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="F5" s="2">
         <v>0</v>
@@ -7445,10 +7454,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M5" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O5">
         <v>2</v>
@@ -7457,10 +7466,10 @@
         <v>1</v>
       </c>
       <c r="S5" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="T5" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="U5" t="b">
         <v>1</v>
@@ -7468,17 +7477,17 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Canopy Bed</v>
       </c>
       <c r="C6" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="D6" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="F6" s="2">
         <v>0</v>
@@ -7499,10 +7508,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M6" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O6">
         <v>2</v>
@@ -7516,17 +7525,17 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Budget Wardrobe</v>
       </c>
       <c r="C7" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="D7" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="F7" s="2">
         <v>0</v>
@@ -7547,10 +7556,10 @@
         <v>2</v>
       </c>
       <c r="L7" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M7" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O7">
         <v>3</v>
@@ -7559,10 +7568,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="T7" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="U7" t="b">
         <v>1</v>
@@ -7570,17 +7579,17 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Fine Wardrobe</v>
       </c>
       <c r="C8" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="D8" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="F8" s="2">
         <v>0</v>
@@ -7601,10 +7610,10 @@
         <v>4</v>
       </c>
       <c r="L8" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M8" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O8">
         <v>3</v>
@@ -7613,10 +7622,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="T8" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="U8" t="b">
         <v>1</v>
@@ -7624,17 +7633,17 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Ornate Wardrobe</v>
       </c>
       <c r="D9" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="E9" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="F9" s="2">
         <v>0</v>
@@ -7655,10 +7664,10 @@
         <v>7</v>
       </c>
       <c r="L9" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M9" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O9">
         <v>3</v>
@@ -7667,10 +7676,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="T9" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="U9" t="b">
         <v>1</v>
@@ -7678,7 +7687,7 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -7703,10 +7712,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M10" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O10">
         <v>1</v>
@@ -7720,14 +7729,14 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Wash Basin</v>
       </c>
       <c r="E11" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="F11" s="2">
         <v>0</v>
@@ -7748,10 +7757,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M11" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O11">
         <v>1</v>
@@ -7765,14 +7774,14 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Artisan Rug</v>
       </c>
       <c r="E12" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="F12" s="2">
         <v>0</v>
@@ -7793,7 +7802,7 @@
         <v>4</v>
       </c>
       <c r="L12" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="O12">
         <v>2</v>
@@ -7807,14 +7816,14 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Mirror</v>
       </c>
       <c r="E13" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="F13" s="2">
         <v>0</v>
@@ -7835,10 +7844,10 @@
         <v>3</v>
       </c>
       <c r="L13" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M13" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O13">
         <v>1</v>
@@ -7852,14 +7861,14 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>Trunk</v>
       </c>
       <c r="C14" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="F14" s="2">
         <v>0</v>
@@ -7880,10 +7889,10 @@
         <v>1</v>
       </c>
       <c r="L14" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M14" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O14">
         <v>2</v>
@@ -7897,7 +7906,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
@@ -7922,7 +7931,7 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="O15">
         <v>3</v>
@@ -7936,7 +7945,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
@@ -7961,10 +7970,10 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M16" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="O16">
         <v>1</v>
@@ -7978,14 +7987,14 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>Small Houseplant</v>
       </c>
       <c r="D17" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="F17" s="2">
         <v>0</v>
@@ -8006,7 +8015,7 @@
         <v>4</v>
       </c>
       <c r="L17" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="O17">
         <v>1</v>
@@ -8015,10 +8024,10 @@
         <v>0</v>
       </c>
       <c r="S17" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="T17" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="U17" t="b">
         <v>1</v>
@@ -8026,14 +8035,14 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>Big Houseplant</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="F18" s="2">
         <v>0</v>
@@ -8054,7 +8063,7 @@
         <v>6</v>
       </c>
       <c r="L18" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="O18">
         <v>2</v>
@@ -8068,14 +8077,14 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
         <v>Chamber Pot</v>
       </c>
       <c r="C19" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="F19" s="2">
         <v>0</v>
@@ -8096,10 +8105,10 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M19" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="O19">
         <v>1</v>
@@ -8113,17 +8122,17 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
         <v>Cooking Order Desk</v>
       </c>
       <c r="C20" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="D20" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="F20" s="2">
         <v>0</v>
@@ -8144,10 +8153,10 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M20" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="O20">
         <v>2</v>
@@ -8156,10 +8165,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="T20" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="U20" t="b">
         <v>1</v>
@@ -8167,17 +8176,17 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
         <v>Cooking Couldron</v>
       </c>
       <c r="C21" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="D21" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="F21" s="2">
         <v>0</v>
@@ -8198,10 +8207,10 @@
         <v>0</v>
       </c>
       <c r="L21" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M21" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="O21">
         <v>2</v>
@@ -8210,10 +8219,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="T21" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="U21" t="b">
         <v>1</v>
@@ -8221,14 +8230,14 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v>Small Seating Table</v>
       </c>
       <c r="D22" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="F22" s="2">
         <v>0</v>
@@ -8249,10 +8258,10 @@
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M22" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="O22">
         <v>2</v>
@@ -8261,10 +8270,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="T22" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="U22" t="b">
         <v>1</v>
@@ -8272,17 +8281,17 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>Pass Table</v>
       </c>
       <c r="C23" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="D23" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="F23" s="2">
         <v>0</v>
@@ -8303,10 +8312,10 @@
         <v>1</v>
       </c>
       <c r="L23" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M23" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="O23">
         <v>2</v>
@@ -8315,10 +8324,10 @@
         <v>0</v>
       </c>
       <c r="S23" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="T23" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="U23" t="b">
         <v>1</v>
@@ -8326,17 +8335,17 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v>Crate</v>
       </c>
       <c r="C24" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="D24" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="F24" s="2">
         <v>0</v>
@@ -8357,7 +8366,7 @@
         <v>0</v>
       </c>
       <c r="L24" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="O24">
         <v>2</v>
@@ -8366,10 +8375,10 @@
         <v>0</v>
       </c>
       <c r="S24" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="T24" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="U24" t="b">
         <v>1</v>
@@ -8377,17 +8386,17 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>Barrel</v>
       </c>
       <c r="C25" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="D25" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="F25" s="2">
         <v>0</v>
@@ -8408,7 +8417,7 @@
         <v>0</v>
       </c>
       <c r="L25" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="O25">
         <v>2</v>
@@ -8417,10 +8426,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="T25" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="U25" t="b">
         <v>1</v>
@@ -8428,17 +8437,17 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
         <v>Wall Torch</v>
       </c>
       <c r="C26" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="D26" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="F26" s="2">
         <v>0</v>
@@ -8459,7 +8468,7 @@
         <v>0</v>
       </c>
       <c r="L26" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="O26">
         <v>0</v>
@@ -8471,10 +8480,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="T26" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="U26" t="b">
         <v>1</v>
@@ -8482,17 +8491,17 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
         <v>Condiment Shelf</v>
       </c>
       <c r="C27" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="D27" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="F27" s="2">
         <v>0</v>
@@ -8513,10 +8522,10 @@
         <v>2</v>
       </c>
       <c r="L27" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="M27" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="O27">
         <v>1</v>
@@ -8528,10 +8537,10 @@
         <v>0</v>
       </c>
       <c r="S27" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="T27" t="s">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="U27" t="b">
         <v>1</v>
@@ -8539,17 +8548,17 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>Condiment Shelf Small</v>
       </c>
       <c r="C28" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="D28" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="F28" s="2">
         <v>0</v>
@@ -8570,10 +8579,10 @@
         <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="M28" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="O28">
         <v>1</v>
@@ -8585,10 +8594,10 @@
         <v>0</v>
       </c>
       <c r="S28" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="T28" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="U28" t="b">
         <v>1</v>
@@ -8596,17 +8605,17 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>Hanging Frying Pans</v>
       </c>
       <c r="C29" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="D29" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="F29" s="2">
         <v>0</v>
@@ -8627,10 +8636,10 @@
         <v>0</v>
       </c>
       <c r="L29" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="M29" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="O29">
         <v>0</v>
@@ -8641,14 +8650,14 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="0"/>
         <v>Butcher Table</v>
       </c>
       <c r="D30" t="s">
-        <v>246</v>
+        <v>235</v>
       </c>
       <c r="F30" s="2">
         <v>0</v>
@@ -8669,10 +8678,10 @@
         <v>3</v>
       </c>
       <c r="L30" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="M30" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="O30">
         <v>2</v>
@@ -8683,14 +8692,14 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>247</v>
+        <v>236</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>Hanging Meat</v>
       </c>
       <c r="D31" t="s">
-        <v>246</v>
+        <v>235</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -8873,10 +8882,10 @@
   <sheetData>
     <row r="2" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="C2" t="s">
         <v>28</v>
@@ -8909,343 +8918,343 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="B1" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="C1" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B17" s="11" t="s">
         <v>16</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B18" s="11" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B19" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>19</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>20</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B22" s="11" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>0</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B26" s="12" t="s">
         <v>43</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B27" s="12" t="s">
         <v>44</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>45</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B29" s="12" t="s">
         <v>46</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B30" s="12" t="s">
         <v>47</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>20</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -9256,7 +9265,7 @@
         <v>0</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -9267,7 +9276,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -9278,150 +9287,150 @@
         <v>42</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="B35" s="15" t="s">
         <v>0</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>1</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>42</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="B39" s="15" t="s">
         <v>3</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>4</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="15" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="B41" s="15" t="s">
         <v>5</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>21</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>0</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>1</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>42</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="B47" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -9432,7 +9441,7 @@
         <v>0</v>
       </c>
       <c r="C48" s="17" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -9443,7 +9452,7 @@
         <v>1</v>
       </c>
       <c r="C49" s="17" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -9454,7 +9463,7 @@
         <v>42</v>
       </c>
       <c r="C50" s="17" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance intermission mechanics and refine shop integration
- Implemented a new intermission system that recalls orbs and stashes breakables after level clears, maintaining gameplay flow.
- Updated the shop mechanics to materialize between levels, allowing players to purchase glyphs and rites using circle mana.
- Revised enemy spawning logic to scale waves based on the current stage, enhancing challenge progression.
- Enhanced documentation in `GAME_BRIEF.md` and `PROJECT_MAP.md` to reflect the new intermission and shop functionalities.
- Adjusted various scene files to support the updated intermission and shop mechanics, ensuring seamless gameplay transitions.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C984E57-CCAB-40EE-B5A4-57621683C44F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4F43A45-4D94-4279-BC91-34DF93FA40BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -2029,7 +2029,7 @@
         <v>0</v>
       </c>
       <c r="Q2" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="R2">
         <v>0</v>
@@ -2104,7 +2104,7 @@
         <v>0</v>
       </c>
       <c r="Q3" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="R3">
         <v>0</v>
@@ -2179,7 +2179,7 @@
         <v>0.01</v>
       </c>
       <c r="Q4" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -2254,7 +2254,7 @@
         <v>0</v>
       </c>
       <c r="Q5" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="R5">
         <v>0</v>
@@ -2329,7 +2329,7 @@
         <v>0.05</v>
       </c>
       <c r="Q6" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="R6">
         <v>3</v>
@@ -2404,7 +2404,7 @@
         <v>0.05</v>
       </c>
       <c r="Q7" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="R7">
         <v>3</v>
@@ -2476,7 +2476,7 @@
         <v>0.05</v>
       </c>
       <c r="Q8" s="8">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="R8">
         <v>3</v>
@@ -2626,7 +2626,7 @@
         <v>0.1</v>
       </c>
       <c r="Q11" s="8">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
       <c r="R11">
         <v>3</v>
@@ -2701,7 +2701,7 @@
         <v>0</v>
       </c>
       <c r="Q12" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="R12">
         <v>2</v>
@@ -2941,7 +2941,7 @@
         <v>0.1</v>
       </c>
       <c r="Q18" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="R18">
         <v>0</v>

</xml_diff>

<commit_message>
Refine glyph drop mechanics and update related documentation
- Adjusted glyph drop logic to ensure that glyphs only spawn from orb kills, removing fallback drops from non-orb sources.
- Updated the `GAME_BRIEF.md` to reflect the new glyph drop mechanics and their integration into gameplay.
- Revised `PROJECT_MAP.md` to document changes related to glyph drop sources and their organization within the project structure.
- Enhanced `level.gd` to streamline glyph drop calculations and ensure consistency with the new mechanics.
- Removed obsolete glyph drop chance variable from the desert scene to simplify configuration.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\Too Many Orbs\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4F43A45-4D94-4279-BC91-34DF93FA40BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C07668BC-19AB-4ACB-996A-B44E29556B0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="441">
   <si>
     <t>id</t>
   </si>
@@ -957,9 +957,6 @@
     <t>On redirect, lower the cooldown of the next frost nova by 0.2 seconds</t>
   </si>
   <si>
-    <t>Each time 3 or more stacks of Frost is inflicted, inflict 1 burn</t>
-  </si>
-  <si>
     <t>Activating the summoning circle costs 50% less</t>
   </si>
   <si>
@@ -1357,6 +1354,21 @@
   </si>
   <si>
     <t>Increase Crit Chance by X</t>
+  </si>
+  <si>
+    <t>rally</t>
+  </si>
+  <si>
+    <t>assistance</t>
+  </si>
+  <si>
+    <t>A breakable destroyed by an enemy has a 40% glyph drop chance</t>
+  </si>
+  <si>
+    <t>breakable, glyph</t>
+  </si>
+  <si>
+    <t>Each time 3 or more stacks of Chill is inflicted, inflict 1 burn</t>
   </si>
 </sst>
 </file>
@@ -2757,9 +2769,12 @@
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>436</v>
+      </c>
       <c r="B14" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Rally</v>
       </c>
       <c r="C14" t="s">
         <v>250</v>
@@ -2783,7 +2798,7 @@
       </c>
       <c r="V14" t="str">
         <f t="shared" ref="V14:V18" si="5">"res://entities/orbs/blank/"&amp;A14&amp;"_orb.tscn"</f>
-        <v>res://entities/orbs/blank/_orb.tscn</v>
+        <v>res://entities/orbs/blank/rally_orb.tscn</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -3974,7 +3989,7 @@
         <v>Coal</v>
       </c>
       <c r="C2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="D2" t="s">
         <v>28</v>
@@ -4005,7 +4020,7 @@
         <v>Fury</v>
       </c>
       <c r="C3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D3" t="s">
         <v>28</v>
@@ -4036,7 +4051,7 @@
         <v>Blast</v>
       </c>
       <c r="C4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D4" t="s">
         <v>28</v>
@@ -4067,7 +4082,7 @@
         <v>Rime</v>
       </c>
       <c r="C5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D5" t="s">
         <v>34</v>
@@ -4098,7 +4113,7 @@
         <v>Sooth</v>
       </c>
       <c r="C6" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="D6" t="s">
         <v>34</v>
@@ -4129,7 +4144,7 @@
         <v>Bounty</v>
       </c>
       <c r="C7" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D7" t="s">
         <v>34</v>
@@ -4160,7 +4175,7 @@
         <v>Static</v>
       </c>
       <c r="C8" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="D8" t="s">
         <v>27</v>
@@ -4191,7 +4206,7 @@
         <v>Shear</v>
       </c>
       <c r="C9" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="D9" t="s">
         <v>27</v>
@@ -4222,7 +4237,7 @@
         <v>Drag</v>
       </c>
       <c r="C10" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="D10" t="s">
         <v>27</v>
@@ -4253,7 +4268,7 @@
         <v>Spore</v>
       </c>
       <c r="C11" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="D11" t="s">
         <v>30</v>
@@ -4284,7 +4299,7 @@
         <v>Dense</v>
       </c>
       <c r="C12" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D12" t="s">
         <v>30</v>
@@ -4315,7 +4330,7 @@
         <v>Crush</v>
       </c>
       <c r="C13" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="D13" t="s">
         <v>30</v>
@@ -5331,7 +5346,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H32" t="str">
         <f t="shared" si="1"/>
@@ -5838,7 +5853,7 @@
   <sheetPr>
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" customWidth="1"/>
@@ -5860,31 +5875,31 @@
         <v>42</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B2" t="str">
-        <f t="shared" ref="B2:B52" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
+        <f t="shared" ref="B2:B53" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Frostburn</v>
       </c>
       <c r="C2" t="s">
-        <v>303</v>
+        <v>440</v>
       </c>
       <c r="D2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E2" t="str">
         <f>"res://ui/rites/"&amp;A2&amp;".png"</f>
@@ -5899,20 +5914,20 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Ward</v>
       </c>
       <c r="C3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E3" t="str">
-        <f t="shared" ref="E3:E52" si="1">"res://ui/rites/"&amp;A3&amp;".png"</f>
+        <f t="shared" ref="E3:E53" si="1">"res://ui/rites/"&amp;A3&amp;".png"</f>
         <v>res://ui/rites/ward.png</v>
       </c>
       <c r="F3" t="b">
@@ -5924,17 +5939,17 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Efficiancy</v>
       </c>
       <c r="C4" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D4" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="1"/>
@@ -5943,17 +5958,17 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>327</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Rebate</v>
+      </c>
+      <c r="C5" t="s">
         <v>328</v>
       </c>
-      <c r="B5" t="str">
-        <f t="shared" si="0"/>
-        <v>Rebate</v>
-      </c>
-      <c r="C5" t="s">
-        <v>329</v>
-      </c>
       <c r="D5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="1"/>
@@ -5962,17 +5977,17 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Grace</v>
       </c>
       <c r="C6" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D6" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E6" t="str">
         <f t="shared" si="1"/>
@@ -5981,17 +5996,17 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Flux</v>
       </c>
       <c r="C7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="1"/>
@@ -6000,17 +6015,17 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Accelerant</v>
       </c>
       <c r="C8" t="s">
+        <v>418</v>
+      </c>
+      <c r="D8" t="s">
         <v>419</v>
-      </c>
-      <c r="D8" t="s">
-        <v>420</v>
       </c>
       <c r="E8" t="str">
         <f t="shared" si="1"/>
@@ -6022,14 +6037,14 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Clash</v>
       </c>
       <c r="C9" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D9" t="s">
         <v>237</v>
@@ -6047,17 +6062,17 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>Skewer</v>
       </c>
       <c r="C10" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D10" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E10" t="str">
         <f t="shared" si="1"/>
@@ -6069,17 +6084,17 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Concuss</v>
       </c>
       <c r="C11" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D11" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E11" t="str">
         <f t="shared" si="1"/>
@@ -6091,17 +6106,17 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Mining</v>
       </c>
       <c r="C12" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D12" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E12" t="str">
         <f t="shared" si="1"/>
@@ -6113,17 +6128,17 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Ballast</v>
       </c>
       <c r="C13" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D13" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E13" t="str">
         <f t="shared" si="1"/>
@@ -6135,17 +6150,17 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>Tithe</v>
       </c>
       <c r="C14" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D14" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E14" t="str">
         <f t="shared" si="1"/>
@@ -6157,17 +6172,17 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
         <v>Groove</v>
       </c>
       <c r="C15" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D15" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E15" t="str">
         <f t="shared" si="1"/>
@@ -6179,14 +6194,14 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
         <v>Boil</v>
       </c>
       <c r="C16" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D16" t="s">
         <v>17</v>
@@ -6201,17 +6216,17 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>Tempered</v>
       </c>
       <c r="C17" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D17" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E17" t="str">
         <f t="shared" si="1"/>
@@ -6226,17 +6241,17 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>Swell</v>
       </c>
       <c r="C18" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D18" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E18" t="str">
         <f t="shared" si="1"/>
@@ -6245,14 +6260,14 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>340</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
+        <v>Ember</v>
+      </c>
+      <c r="C19" t="s">
         <v>341</v>
-      </c>
-      <c r="B19" t="str">
-        <f t="shared" si="0"/>
-        <v>Ember</v>
-      </c>
-      <c r="C19" t="s">
-        <v>342</v>
       </c>
       <c r="D19" t="s">
         <v>16</v>
@@ -6267,14 +6282,14 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>342</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>Smolder</v>
+      </c>
+      <c r="C20" t="s">
         <v>343</v>
-      </c>
-      <c r="B20" t="str">
-        <f t="shared" si="0"/>
-        <v>Smolder</v>
-      </c>
-      <c r="C20" t="s">
-        <v>344</v>
       </c>
       <c r="D20" t="s">
         <v>16</v>
@@ -6289,17 +6304,17 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
         <v>Mercy</v>
       </c>
       <c r="C21" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D21" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E21" t="str">
         <f t="shared" si="1"/>
@@ -6311,17 +6326,17 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v>Heft</v>
       </c>
       <c r="C22" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D22" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E22" t="str">
         <f t="shared" si="1"/>
@@ -6333,17 +6348,17 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>Followthrough</v>
       </c>
       <c r="C23" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D23" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E23" t="str">
         <f t="shared" si="1"/>
@@ -6355,17 +6370,17 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>350</v>
+      </c>
+      <c r="B24" t="str">
+        <f t="shared" si="0"/>
+        <v>Martyr</v>
+      </c>
+      <c r="C24" t="s">
         <v>351</v>
       </c>
-      <c r="B24" t="str">
-        <f t="shared" si="0"/>
-        <v>Martyr</v>
-      </c>
-      <c r="C24" t="s">
-        <v>352</v>
-      </c>
       <c r="D24" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E24" t="str">
         <f t="shared" si="1"/>
@@ -6377,17 +6392,17 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>352</v>
+      </c>
+      <c r="B25" t="str">
+        <f t="shared" si="0"/>
+        <v>Penance</v>
+      </c>
+      <c r="C25" t="s">
         <v>353</v>
       </c>
-      <c r="B25" t="str">
-        <f t="shared" si="0"/>
-        <v>Penance</v>
-      </c>
-      <c r="C25" t="s">
-        <v>354</v>
-      </c>
       <c r="D25" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E25" t="str">
         <f t="shared" si="1"/>
@@ -6399,17 +6414,17 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>354</v>
+      </c>
+      <c r="B26" t="str">
+        <f t="shared" si="0"/>
+        <v>Surrogate</v>
+      </c>
+      <c r="C26" t="s">
         <v>355</v>
       </c>
-      <c r="B26" t="str">
-        <f t="shared" si="0"/>
-        <v>Surrogate</v>
-      </c>
-      <c r="C26" t="s">
-        <v>356</v>
-      </c>
       <c r="D26" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E26" t="str">
         <f t="shared" si="1"/>
@@ -6421,17 +6436,17 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>356</v>
+      </c>
+      <c r="B27" t="str">
+        <f t="shared" si="0"/>
+        <v>Glass</v>
+      </c>
+      <c r="C27" t="s">
         <v>357</v>
       </c>
-      <c r="B27" t="str">
-        <f t="shared" si="0"/>
-        <v>Glass</v>
-      </c>
-      <c r="C27" t="s">
-        <v>358</v>
-      </c>
       <c r="D27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E27" t="str">
         <f t="shared" si="1"/>
@@ -6443,17 +6458,17 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>358</v>
+      </c>
+      <c r="B28" t="str">
+        <f t="shared" si="0"/>
+        <v>Payback</v>
+      </c>
+      <c r="C28" t="s">
         <v>359</v>
       </c>
-      <c r="B28" t="str">
-        <f t="shared" si="0"/>
-        <v>Payback</v>
-      </c>
-      <c r="C28" t="s">
-        <v>360</v>
-      </c>
       <c r="D28" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E28" t="str">
         <f t="shared" si="1"/>
@@ -6465,17 +6480,17 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>360</v>
+      </c>
+      <c r="B29" t="str">
+        <f t="shared" si="0"/>
+        <v>Reduce</v>
+      </c>
+      <c r="C29" t="s">
         <v>361</v>
       </c>
-      <c r="B29" t="str">
-        <f t="shared" si="0"/>
-        <v>Reduce</v>
-      </c>
-      <c r="C29" t="s">
-        <v>362</v>
-      </c>
       <c r="D29" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E29" t="str">
         <f t="shared" si="1"/>
@@ -6487,17 +6502,17 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>362</v>
+      </c>
+      <c r="B30" t="str">
+        <f t="shared" si="0"/>
+        <v>Surplus</v>
+      </c>
+      <c r="C30" t="s">
         <v>363</v>
       </c>
-      <c r="B30" t="str">
-        <f t="shared" si="0"/>
-        <v>Surplus</v>
-      </c>
-      <c r="C30" t="s">
-        <v>364</v>
-      </c>
       <c r="D30" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E30" t="str">
         <f t="shared" si="1"/>
@@ -6509,17 +6524,17 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>364</v>
+      </c>
+      <c r="B31" t="str">
+        <f t="shared" si="0"/>
+        <v>Refund</v>
+      </c>
+      <c r="C31" t="s">
         <v>365</v>
       </c>
-      <c r="B31" t="str">
-        <f t="shared" si="0"/>
-        <v>Refund</v>
-      </c>
-      <c r="C31" t="s">
-        <v>366</v>
-      </c>
       <c r="D31" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E31" t="str">
         <f t="shared" si="1"/>
@@ -6531,17 +6546,17 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>366</v>
+      </c>
+      <c r="B32" t="str">
+        <f t="shared" si="0"/>
+        <v>Subsidy</v>
+      </c>
+      <c r="C32" t="s">
         <v>367</v>
       </c>
-      <c r="B32" t="str">
-        <f t="shared" si="0"/>
-        <v>Subsidy</v>
-      </c>
-      <c r="C32" t="s">
-        <v>368</v>
-      </c>
       <c r="D32" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E32" t="str">
         <f t="shared" si="1"/>
@@ -6553,17 +6568,17 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>368</v>
+      </c>
+      <c r="B33" t="str">
+        <f t="shared" si="0"/>
+        <v>Swarm</v>
+      </c>
+      <c r="C33" t="s">
         <v>369</v>
       </c>
-      <c r="B33" t="str">
-        <f t="shared" si="0"/>
-        <v>Swarm</v>
-      </c>
-      <c r="C33" t="s">
-        <v>370</v>
-      </c>
       <c r="D33" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E33" t="str">
         <f t="shared" si="1"/>
@@ -6575,17 +6590,17 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="0"/>
         <v>Salvage</v>
       </c>
       <c r="C34" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="D34" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E34" t="str">
         <f t="shared" si="1"/>
@@ -6597,17 +6612,17 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>371</v>
+      </c>
+      <c r="B35" t="str">
+        <f t="shared" si="0"/>
+        <v>Premium</v>
+      </c>
+      <c r="C35" t="s">
         <v>372</v>
       </c>
-      <c r="B35" t="str">
-        <f t="shared" si="0"/>
-        <v>Premium</v>
-      </c>
-      <c r="C35" t="s">
-        <v>373</v>
-      </c>
       <c r="D35" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E35" t="str">
         <f t="shared" si="1"/>
@@ -6619,17 +6634,17 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="0"/>
         <v>Vigil</v>
       </c>
       <c r="C36" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D36" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E36" t="str">
         <f t="shared" si="1"/>
@@ -6641,17 +6656,17 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>375</v>
+      </c>
+      <c r="B37" t="str">
+        <f t="shared" si="0"/>
+        <v>Keeper</v>
+      </c>
+      <c r="C37" t="s">
         <v>376</v>
       </c>
-      <c r="B37" t="str">
-        <f t="shared" si="0"/>
-        <v>Keeper</v>
-      </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>377</v>
-      </c>
-      <c r="D37" t="s">
-        <v>378</v>
       </c>
       <c r="E37" t="str">
         <f t="shared" si="1"/>
@@ -6663,17 +6678,17 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="0"/>
         <v>Unburden</v>
       </c>
       <c r="C38" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="D38" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E38" t="str">
         <f t="shared" si="1"/>
@@ -6682,17 +6697,17 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>382</v>
+      </c>
+      <c r="B39" t="str">
+        <f t="shared" si="0"/>
+        <v>Courier</v>
+      </c>
+      <c r="C39" t="s">
         <v>383</v>
       </c>
-      <c r="B39" t="str">
-        <f t="shared" si="0"/>
-        <v>Courier</v>
-      </c>
-      <c r="C39" t="s">
-        <v>384</v>
-      </c>
       <c r="D39" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E39" t="str">
         <f t="shared" si="1"/>
@@ -6701,17 +6716,17 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="0"/>
         <v>Auspice</v>
       </c>
       <c r="C40" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D40" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E40" t="str">
         <f t="shared" si="1"/>
@@ -6720,17 +6735,17 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="0"/>
         <v>Brittle</v>
       </c>
       <c r="C41" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D41" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E41" t="str">
         <f t="shared" si="1"/>
@@ -6739,17 +6754,17 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>386</v>
+      </c>
+      <c r="B42" t="str">
+        <f t="shared" si="0"/>
+        <v>Imbue</v>
+      </c>
+      <c r="C42" t="s">
         <v>387</v>
       </c>
-      <c r="B42" t="str">
-        <f t="shared" si="0"/>
-        <v>Imbue</v>
-      </c>
-      <c r="C42" t="s">
-        <v>388</v>
-      </c>
       <c r="D42" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E42" t="str">
         <f t="shared" si="1"/>
@@ -6758,17 +6773,17 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>390</v>
+      </c>
+      <c r="B43" t="str">
+        <f t="shared" si="0"/>
+        <v>Sepsis</v>
+      </c>
+      <c r="C43" t="s">
         <v>391</v>
       </c>
-      <c r="B43" t="str">
-        <f t="shared" si="0"/>
-        <v>Sepsis</v>
-      </c>
-      <c r="C43" t="s">
-        <v>392</v>
-      </c>
       <c r="D43" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E43" t="str">
         <f t="shared" si="1"/>
@@ -6777,14 +6792,14 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>392</v>
+      </c>
+      <c r="B44" t="str">
+        <f t="shared" si="0"/>
+        <v>Glacier</v>
+      </c>
+      <c r="C44" t="s">
         <v>393</v>
-      </c>
-      <c r="B44" t="str">
-        <f t="shared" si="0"/>
-        <v>Glacier</v>
-      </c>
-      <c r="C44" t="s">
-        <v>394</v>
       </c>
       <c r="D44" t="s">
         <v>17</v>
@@ -6796,14 +6811,14 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>394</v>
+      </c>
+      <c r="B45" t="str">
+        <f t="shared" si="0"/>
+        <v>Hairpin</v>
+      </c>
+      <c r="C45" t="s">
         <v>395</v>
-      </c>
-      <c r="B45" t="str">
-        <f t="shared" si="0"/>
-        <v>Hairpin</v>
-      </c>
-      <c r="C45" t="s">
-        <v>396</v>
       </c>
       <c r="D45" t="s">
         <v>18</v>
@@ -6815,14 +6830,14 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>396</v>
+      </c>
+      <c r="B46" t="str">
+        <f t="shared" si="0"/>
+        <v>Leftover</v>
+      </c>
+      <c r="C46" t="s">
         <v>397</v>
-      </c>
-      <c r="B46" t="str">
-        <f t="shared" si="0"/>
-        <v>Leftover</v>
-      </c>
-      <c r="C46" t="s">
-        <v>398</v>
       </c>
       <c r="D46" t="s">
         <v>18</v>
@@ -6834,14 +6849,14 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="0"/>
         <v>Daze</v>
       </c>
       <c r="C47" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D47" t="s">
         <v>18</v>
@@ -6853,43 +6868,43 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>402</v>
+      </c>
+      <c r="B48" t="str">
+        <f t="shared" si="0"/>
+        <v>Sickly</v>
+      </c>
+      <c r="C48" t="s">
         <v>403</v>
       </c>
-      <c r="B48" t="str">
-        <f t="shared" si="0"/>
-        <v>Sickly</v>
-      </c>
-      <c r="C48" t="s">
-        <v>404</v>
-      </c>
       <c r="D48" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E48" t="str">
         <f t="shared" si="1"/>
         <v>res://ui/rites/sickly.png</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="0"/>
         <v>Wide</v>
       </c>
       <c r="C49" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D49" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E49" t="str">
         <f t="shared" si="1"/>
         <v>res://ui/rites/wide.png</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>259</v>
       </c>
@@ -6898,52 +6913,74 @@
         <v>Fright</v>
       </c>
       <c r="C50" t="s">
+        <v>404</v>
+      </c>
+      <c r="D50" t="s">
         <v>405</v>
       </c>
-      <c r="D50" t="s">
-        <v>406</v>
-      </c>
       <c r="E50" t="str">
         <f t="shared" si="1"/>
         <v>res://ui/rites/fright.png</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>411</v>
+      </c>
+      <c r="B51" t="str">
+        <f t="shared" si="0"/>
+        <v>Fuse</v>
+      </c>
+      <c r="C51" t="s">
+        <v>410</v>
+      </c>
+      <c r="D51" t="s">
+        <v>405</v>
+      </c>
+      <c r="E51" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/fuse.png</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>413</v>
+      </c>
+      <c r="B52" t="str">
+        <f t="shared" si="0"/>
+        <v>Clearcut</v>
+      </c>
+      <c r="C52" t="s">
         <v>412</v>
       </c>
-      <c r="B51" t="str">
-        <f t="shared" si="0"/>
-        <v>Fuse</v>
-      </c>
-      <c r="C51" t="s">
-        <v>411</v>
-      </c>
-      <c r="D51" t="s">
-        <v>406</v>
-      </c>
-      <c r="E51" t="str">
-        <f t="shared" si="1"/>
-        <v>res://ui/rites/fuse.png</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>414</v>
-      </c>
-      <c r="B52" t="str">
-        <f t="shared" si="0"/>
-        <v>Clearcut</v>
-      </c>
-      <c r="C52" t="s">
-        <v>413</v>
-      </c>
       <c r="D52" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E52" t="str">
         <f t="shared" si="1"/>
         <v>res://ui/rites/clearcut.png</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>437</v>
+      </c>
+      <c r="B53" t="str">
+        <f t="shared" si="0"/>
+        <v>Assistance</v>
+      </c>
+      <c r="C53" t="s">
+        <v>438</v>
+      </c>
+      <c r="D53" t="s">
+        <v>439</v>
+      </c>
+      <c r="E53" t="str">
+        <f t="shared" si="1"/>
+        <v>res://ui/rites/assistance.png</v>
+      </c>
+      <c r="G53">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -9380,7 +9417,7 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>0</v>
@@ -9391,7 +9428,7 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>1</v>
@@ -9402,7 +9439,7 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>42</v>
@@ -9413,10 +9450,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C46" s="14" t="s">
         <v>241</v>
@@ -9424,7 +9461,7 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B47" s="14" t="s">
         <v>21</v>

</xml_diff>